<commit_message>
Improvements for Properties and their handling
</commit_message>
<xml_diff>
--- a/AWB-RestApi-PropertyDictionary.xlsx
+++ b/AWB-RestApi-PropertyDictionary.xlsx
@@ -1,21 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\20_GIT\01_AWB\eclipseProjects\de.enflexit.awb\bundles\web\de.enflexit.awb.ws.restapi\xAPI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{826B0FA9-8E7C-4E54-930B-A4822E697B51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AC9A81E-0D7E-4BB3-98F2-B991F8535523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Property-Definition" sheetId="1" r:id="rId1"/>
+    <sheet name="Java-Code" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
   <si>
     <t>key</t>
   </si>
@@ -50,7 +52,46 @@
     <t>performative</t>
   </si>
   <si>
-    <t>DB.</t>
+    <t>direction</t>
+  </si>
+  <si>
+    <t>GET</t>
+  </si>
+  <si>
+    <t>DB.SYSTEMS</t>
+  </si>
+  <si>
+    <t>String</t>
+  </si>
+  <si>
+    <t>dbSystem[X]</t>
+  </si>
+  <si>
+    <t>e.g. 'Apache Derby', 'MariaDB', …</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>AWB-Integration Bundle</t>
+  </si>
+  <si>
+    <t>de.enflexit.db.hibernate</t>
+  </si>
+  <si>
+    <t>Get only. Probably returns several indexed properties. Returns all registered HibernateDatabaseServices with ther names.</t>
+  </si>
+  <si>
+    <t>DB.FACTORIES</t>
+  </si>
+  <si>
+    <t>factory[X]</t>
+  </si>
+  <si>
+    <t>Get only. Probably returns several indexed properties. Returns all registered Hibernate database factories with their name.</t>
+  </si>
+  <si>
+    <t>e.g. 'de.enfexit.awb.bgsystem.db'</t>
   </si>
 </sst>
 </file>
@@ -377,36 +418,99 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.140625" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="33.140625" customWidth="1"/>
-    <col min="4" max="4" width="27.7109375" customWidth="1"/>
+    <col min="1" max="2" width="21.140625" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="33.140625" customWidth="1"/>
+    <col min="5" max="6" width="34.85546875" customWidth="1"/>
+    <col min="7" max="7" width="113.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="F1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F30A1E73-A707-4178-9C72-9AC27F9EE5F7}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Extend DB.Factories for property calls
</commit_message>
<xml_diff>
--- a/AWB-RestApi-PropertyDictionary.xlsx
+++ b/AWB-RestApi-PropertyDictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\20_GIT\01_AWB\eclipseProjects\de.enflexit.awb\bundles\web\de.enflexit.awb.ws.restapi\xAPI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AC9A81E-0D7E-4BB3-98F2-B991F8535523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FEC2AF3-870D-4614-87DF-A37287231B7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,6 @@
     <sheet name="Java-Code" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="42">
   <si>
     <t>key</t>
   </si>
@@ -88,17 +87,89 @@
     <t>factory[X]</t>
   </si>
   <si>
-    <t>Get only. Probably returns several indexed properties. Returns all registered Hibernate database factories with their name.</t>
-  </si>
-  <si>
     <t>e.g. 'de.enfexit.awb.bgsystem.db'</t>
+  </si>
+  <si>
+    <t>DB.DERBY.NETWORKSERVER</t>
+  </si>
+  <si>
+    <t>GET + SET</t>
+  </si>
+  <si>
+    <t>isStartDerbyNetworkServer</t>
+  </si>
+  <si>
+    <t>Boolean</t>
+  </si>
+  <si>
+    <t>true | false</t>
+  </si>
+  <si>
+    <t>indicator to start a derby network server</t>
+  </si>
+  <si>
+    <t>host-IP</t>
+  </si>
+  <si>
+    <t>localhost</t>
+  </si>
+  <si>
+    <t>port</t>
+  </si>
+  <si>
+    <t>Integer</t>
+  </si>
+  <si>
+    <t>1527</t>
+  </si>
+  <si>
+    <t>Host or IP-Address</t>
+  </si>
+  <si>
+    <t>Port of the DB-Server</t>
+  </si>
+  <si>
+    <t>userName</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>xxxxx</t>
+  </si>
+  <si>
+    <t>******</t>
+  </si>
+  <si>
+    <t>The username to access the DB-Server</t>
+  </si>
+  <si>
+    <t>The password to access the DB-Server</t>
+  </si>
+  <si>
+    <t>factory[X].state</t>
+  </si>
+  <si>
+    <t>valueOptions</t>
+  </si>
+  <si>
+    <t>[NotAvailableYet (Not available yet), Destroyed (SessionFactory was destroyed), CheckDBConnection (Checking database connection ...), CheckDBConectionFailed (Database connection test failed!), InitializationProcessStarted (Initialize SessionFactory), InitializationProcessFailed (Initialization of SessionFactory failed), Created (Successfully Initialized)]</t>
+  </si>
+  <si>
+    <t>Returns all registered Hibernate database factories with their name.</t>
+  </si>
+  <si>
+    <t>Returns the states of the corresponding factory (see value Options)</t>
+  </si>
+  <si>
+    <t>e.g. 'Created'</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -113,6 +184,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -135,9 +212,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -418,17 +497,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="21.140625" customWidth="1"/>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
     <col min="4" max="4" width="33.140625" customWidth="1"/>
-    <col min="5" max="6" width="34.85546875" customWidth="1"/>
-    <col min="7" max="7" width="113.7109375" customWidth="1"/>
+    <col min="5" max="5" width="34.85546875" customWidth="1"/>
+    <col min="6" max="6" width="41.28515625" customWidth="1"/>
+    <col min="7" max="7" width="34.85546875" customWidth="1"/>
+    <col min="8" max="8" width="113.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -445,13 +527,16 @@
         <v>1</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -467,14 +552,14 @@
       <c r="E2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -488,13 +573,155 @@
         <v>7</v>
       </c>
       <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="G4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>17</v>
       </c>
-      <c r="F3" t="s">
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" t="s">
         <v>12</v>
       </c>
-      <c r="G3" t="s">
-        <v>16</v>
+      <c r="H5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="2"/>
+      <c r="G7" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s">
+        <v>32</v>
+      </c>
+      <c r="G8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G9" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -505,12 +732,61 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F30A1E73-A707-4178-9C72-9AC27F9EE5F7}">
-  <dimension ref="A1"/>
+  <dimension ref="A2:A9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="str">
+        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A2,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C2 &amp; CHAR(34)&amp; ";"</f>
+        <v>public static String DB_SYSTEMS = "dbSystem[X]";</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="str">
+        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A3,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C3 &amp; CHAR(34)&amp; ";"</f>
+        <v>public static String DB_FACTORIES = "factory[X]";</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="str">
+        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A4,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C4 &amp; CHAR(34)&amp; ";"</f>
+        <v>public static String DB_FACTORIES = "factory[X].state";</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="str">
+        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A5,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C5 &amp; CHAR(34)&amp; ";"</f>
+        <v>public static String DB_DERBY_NETWORKSERVER = "isStartDerbyNetworkServer";</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="str">
+        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A6,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C6 &amp; CHAR(34)&amp; ";"</f>
+        <v>public static String DB_DERBY_NETWORKSERVER = "host-IP";</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="str">
+        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A7,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C7 &amp; CHAR(34)&amp; ";"</f>
+        <v>public static String DB_DERBY_NETWORKSERVER = "port";</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="str">
+        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A8,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C8 &amp; CHAR(34)&amp; ";"</f>
+        <v>public static String DB_DERBY_NETWORKSERVER = "userName";</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="str">
+        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A9,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C9 &amp; CHAR(34)&amp; ";"</f>
+        <v>public static String DB_DERBY_NETWORKSERVER = "password";</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Improved PropertyDictionary for connection settings
</commit_message>
<xml_diff>
--- a/AWB-RestApi-PropertyDictionary.xlsx
+++ b/AWB-RestApi-PropertyDictionary.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\20_GIT\01_AWB\eclipseProjects\de.enflexit.awb\bundles\web\de.enflexit.awb.ws.restapi\xAPI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://enflexit.sharepoint.com/sites/Web-UI/Freigegebene Dokumente/General/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FEC2AF3-870D-4614-87DF-A37287231B7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="139" documentId="13_ncr:1_{79BC29FB-AD0F-4206-B7CB-2FF474441C84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C18A84FA-5010-4EB8-9831-C28D83F9F985}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="76">
   <si>
     <t>key</t>
   </si>
@@ -163,6 +163,108 @@
   </si>
   <si>
     <t>e.g. 'Created'</t>
+  </si>
+  <si>
+    <t>DB.CONN.GENERAL</t>
+  </si>
+  <si>
+    <t>useForEveryDatabaseConnection</t>
+  </si>
+  <si>
+    <t>de.enflexit.db.derby</t>
+  </si>
+  <si>
+    <t>DB.SYSTEMS.PARAMETER</t>
+  </si>
+  <si>
+    <t>e.g. 'MariaDB'</t>
+  </si>
+  <si>
+    <t>dbSystem[X].hibernate.connection.password</t>
+  </si>
+  <si>
+    <t>dbSystem[X].hibernate.connection.username</t>
+  </si>
+  <si>
+    <t>dbSystem[X].hibernate.connection.driver_class</t>
+  </si>
+  <si>
+    <t>eg. 'org.mariadb.jdbc.Driver'</t>
+  </si>
+  <si>
+    <t>eg. 'jdbc:mariadb://localhost:3306/agentWorkbench?createDatabaseIfNotExist=true'</t>
+  </si>
+  <si>
+    <t>eg. 'jdbc:mariadb://[HostOrIP]:[Port]/[Catalog]?createDatabaseIfNotExist=true'</t>
+  </si>
+  <si>
+    <t>dbSystem[X].hibernate.default_catalog</t>
+  </si>
+  <si>
+    <t>eg. 'agentWorkbench'</t>
+  </si>
+  <si>
+    <t>eg. 'admin'</t>
+  </si>
+  <si>
+    <t>eg. 'secret'</t>
+  </si>
+  <si>
+    <t>dbSystem</t>
+  </si>
+  <si>
+    <t>eg. 'jdbc:mariadb://myServer:1234/myDatabase?createDatabaseIfNotExist=true'</t>
+  </si>
+  <si>
+    <t>eg. 'myDatabase'</t>
+  </si>
+  <si>
+    <t>eg. 'secretPassword'</t>
+  </si>
+  <si>
+    <t>eg. 'superUser'</t>
+  </si>
+  <si>
+    <t>hibernate.connection.driver_class</t>
+  </si>
+  <si>
+    <t>hibernate.connection.url</t>
+  </si>
+  <si>
+    <t>hibernate.default_catalog</t>
+  </si>
+  <si>
+    <t>hibernate.connection.username</t>
+  </si>
+  <si>
+    <t>hibernate.connection.password</t>
+  </si>
+  <si>
+    <t>dbSystem[X].hibernate.connection.url</t>
+  </si>
+  <si>
+    <t>dbSystem[X].hibernate.connection.url.mask</t>
+  </si>
+  <si>
+    <t>Done Server-Side</t>
+  </si>
+  <si>
+    <t>Done Client-Side</t>
+  </si>
+  <si>
+    <t>True</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>DB.CONN.FACTORY</t>
+  </si>
+  <si>
+    <t>factoryID</t>
+  </si>
+  <si>
+    <t>e.g. 'de.enflexit.awb.bgsystem.db'</t>
   </si>
 </sst>
 </file>
@@ -212,17 +314,159 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="13">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF9999"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -497,20 +741,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
-    <col min="2" max="2" width="21.140625" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="33.140625" customWidth="1"/>
-    <col min="5" max="5" width="34.85546875" customWidth="1"/>
-    <col min="6" max="6" width="41.28515625" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" customWidth="1"/>
+    <col min="3" max="3" width="54.140625" customWidth="1"/>
+    <col min="4" max="4" width="17.140625" customWidth="1"/>
+    <col min="5" max="5" width="79" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" customWidth="1"/>
     <col min="7" max="7" width="34.85546875" customWidth="1"/>
-    <col min="8" max="8" width="113.7109375" customWidth="1"/>
+    <col min="8" max="9" width="17.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="113.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -532,11 +777,17 @@
       <c r="G1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -555,176 +806,642 @@
       <c r="G2" t="s">
         <v>12</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="J2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D3" t="s">
         <v>7</v>
       </c>
       <c r="E3" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="G3" t="s">
         <v>12</v>
       </c>
-      <c r="H3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H3" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="D4" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>38</v>
+      <c r="E4" t="s">
+        <v>50</v>
       </c>
       <c r="G4" t="s">
         <v>12</v>
       </c>
-      <c r="H4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H4" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>67</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="G5" t="s">
         <v>12</v>
       </c>
-      <c r="H5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H5" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
+        <v>68</v>
       </c>
       <c r="D6" t="s">
         <v>7</v>
       </c>
       <c r="E6" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="G6" t="s">
         <v>12</v>
       </c>
-      <c r="H6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H6" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="D7" t="s">
-        <v>26</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E7" t="s">
+        <v>54</v>
+      </c>
       <c r="G7" t="s">
         <v>12</v>
       </c>
-      <c r="H7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H7" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="D8" t="s">
         <v>7</v>
       </c>
       <c r="E8" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="G8" t="s">
         <v>12</v>
       </c>
-      <c r="H8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H8" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s">
         <v>7</v>
       </c>
       <c r="E9" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="G9" t="s">
         <v>12</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G10" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="J10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="G11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="J11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" t="s">
+        <v>44</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="J12" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" t="s">
+        <v>24</v>
+      </c>
+      <c r="G13" t="s">
+        <v>44</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="J13" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" t="s">
+        <v>26</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="2"/>
+      <c r="G14" t="s">
+        <v>44</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="J14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" t="s">
+        <v>32</v>
+      </c>
+      <c r="G15" t="s">
+        <v>44</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="J15" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" t="s">
+        <v>31</v>
+      </c>
+      <c r="D16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" t="s">
+        <v>33</v>
+      </c>
+      <c r="G16" t="s">
+        <v>44</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="J16" t="s">
         <v>35</v>
       </c>
     </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" t="s">
+        <v>20</v>
+      </c>
+      <c r="E17" t="s">
+        <v>21</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" t="s">
+        <v>57</v>
+      </c>
+      <c r="D18" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" t="s">
+        <v>46</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" t="s">
+        <v>62</v>
+      </c>
+      <c r="D19" t="s">
+        <v>7</v>
+      </c>
+      <c r="E19" t="s">
+        <v>50</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" t="s">
+        <v>63</v>
+      </c>
+      <c r="D20" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" t="s">
+        <v>58</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" t="s">
+        <v>64</v>
+      </c>
+      <c r="D21" t="s">
+        <v>7</v>
+      </c>
+      <c r="E21" t="s">
+        <v>59</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" t="s">
+        <v>65</v>
+      </c>
+      <c r="D22" t="s">
+        <v>7</v>
+      </c>
+      <c r="E22" t="s">
+        <v>61</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" t="s">
+        <v>66</v>
+      </c>
+      <c r="D23" t="s">
+        <v>7</v>
+      </c>
+      <c r="E23" t="s">
+        <v>60</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>73</v>
+      </c>
+      <c r="B24" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" t="s">
+        <v>74</v>
+      </c>
+      <c r="D24" t="s">
+        <v>7</v>
+      </c>
+      <c r="E24" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" t="s">
+        <v>57</v>
+      </c>
+      <c r="D25" t="s">
+        <v>7</v>
+      </c>
+      <c r="E25" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>73</v>
+      </c>
+      <c r="B26" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" t="s">
+        <v>62</v>
+      </c>
+      <c r="D26" t="s">
+        <v>7</v>
+      </c>
+      <c r="E26" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>73</v>
+      </c>
+      <c r="B27" t="s">
+        <v>18</v>
+      </c>
+      <c r="C27" t="s">
+        <v>63</v>
+      </c>
+      <c r="D27" t="s">
+        <v>7</v>
+      </c>
+      <c r="E27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>73</v>
+      </c>
+      <c r="B28" t="s">
+        <v>18</v>
+      </c>
+      <c r="C28" t="s">
+        <v>64</v>
+      </c>
+      <c r="D28" t="s">
+        <v>7</v>
+      </c>
+      <c r="E28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>73</v>
+      </c>
+      <c r="B29" t="s">
+        <v>18</v>
+      </c>
+      <c r="C29" t="s">
+        <v>65</v>
+      </c>
+      <c r="D29" t="s">
+        <v>7</v>
+      </c>
+      <c r="E29" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>73</v>
+      </c>
+      <c r="B30" t="s">
+        <v>18</v>
+      </c>
+      <c r="C30" t="s">
+        <v>66</v>
+      </c>
+      <c r="D30" t="s">
+        <v>7</v>
+      </c>
+      <c r="E30" t="s">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="H2:I23">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
+      <formula>"In Progress"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
+      <formula>"True"</formula>
+    </cfRule>
+    <cfRule type="containsBlanks" dxfId="3" priority="7">
+      <formula>LEN(TRIM(H2))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H24:I30">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+      <formula>"In Progress"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>"True"</formula>
+    </cfRule>
+    <cfRule type="containsBlanks" dxfId="0" priority="3">
+      <formula>LEN(TRIM(H24))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -746,47 +1463,300 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
-        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A3,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C3 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A10,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C10 &amp; CHAR(34)&amp; ";"</f>
         <v>public static String DB_FACTORIES = "factory[X]";</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
-        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A4,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C4 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A11,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C11 &amp; CHAR(34)&amp; ";"</f>
         <v>public static String DB_FACTORIES = "factory[X].state";</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
-        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A5,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C5 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A12,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C12 &amp; CHAR(34)&amp; ";"</f>
         <v>public static String DB_DERBY_NETWORKSERVER = "isStartDerbyNetworkServer";</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
-        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A6,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C6 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A13,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C13 &amp; CHAR(34)&amp; ";"</f>
         <v>public static String DB_DERBY_NETWORKSERVER = "host-IP";</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
-        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A7,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C7 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A14,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C14 &amp; CHAR(34)&amp; ";"</f>
         <v>public static String DB_DERBY_NETWORKSERVER = "port";</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
-        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A8,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C8 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A15,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C15 &amp; CHAR(34)&amp; ";"</f>
         <v>public static String DB_DERBY_NETWORKSERVER = "userName";</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
-        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A9,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C9 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public static String "&amp; SUBSTITUTE('Property-Definition'!A16,".","_")&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!C16 &amp; CHAR(34)&amp; ";"</f>
         <v>public static String DB_DERBY_NETWORKSERVER = "password";</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101004FB79D76D905EB41B4AD64ED4839597F" ma:contentTypeVersion="11" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="0622d98e252eab518d4b54f931ba6851">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="897f6830-f425-409d-b8f5-ce1019056d9e" xmlns:ns3="f2404b4d-361b-46d3-b2ec-035eed29e274" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dd5f302b3846fd12003b89c8f5b7df36" ns2:_="" ns3:_="">
+    <xsd:import namespace="897f6830-f425-409d-b8f5-ce1019056d9e"/>
+    <xsd:import namespace="f2404b4d-361b-46d3-b2ec-035eed29e274"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="897f6830-f425-409d-b8f5-ce1019056d9e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Bildmarkierungen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="e15d79c3-0059-4ac5-86a1-cea3d911e6f7" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="13" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="14" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="17" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="f2404b4d-361b-46d3-b2ec-035eed29e274" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{0b6d854a-ba95-410b-89a3-6da5fcfbdf48}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="f2404b4d-361b-46d3-b2ec-035eed29e274">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Inhaltstyp"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titel"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="897f6830-f425-409d-b8f5-ce1019056d9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="f2404b4d-361b-46d3-b2ec-035eed29e274" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A33EE264-283E-4F19-BA61-B3264EA417E2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="897f6830-f425-409d-b8f5-ce1019056d9e"/>
+    <ds:schemaRef ds:uri="f2404b4d-361b-46d3-b2ec-035eed29e274"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF16440F-B0E0-4269-97EE-BEB05B0223C8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="897f6830-f425-409d-b8f5-ce1019056d9e"/>
+    <ds:schemaRef ds:uri="f2404b4d-361b-46d3-b2ec-035eed29e274"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Added the performative "DB.CONN.TEST" to AWB-RestApi-PropertyDictionary
</commit_message>
<xml_diff>
--- a/AWB-RestApi-PropertyDictionary.xlsx
+++ b/AWB-RestApi-PropertyDictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\AgentWorkbench\eclipseProjects\de.enflexit.awb\bundles\web\xApi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1826633A-B76C-4AE6-9F15-B4AFA8E394CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3D83042-72FF-4DF6-81BC-39EE4F446ABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="85">
   <si>
     <t>key</t>
   </si>
@@ -252,9 +252,6 @@
     <t>True</t>
   </si>
   <si>
-    <t>In Progress</t>
-  </si>
-  <si>
     <t>factoryID</t>
   </si>
   <si>
@@ -292,6 +289,9 @@
   </si>
   <si>
     <t>factory[X].hibernate.connection.password</t>
+  </si>
+  <si>
+    <t>DB.CONN.TEST</t>
   </si>
 </sst>
 </file>
@@ -356,37 +356,7 @@
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9999"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -698,7 +668,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="28.7265625" customWidth="1"/>
@@ -766,6 +736,9 @@
       <c r="H2" s="5" t="s">
         <v>70</v>
       </c>
+      <c r="I2" s="5" t="s">
+        <v>70</v>
+      </c>
       <c r="J2" t="s">
         <v>13</v>
       </c>
@@ -792,6 +765,9 @@
       <c r="H3" s="5" t="s">
         <v>70</v>
       </c>
+      <c r="I3" s="5" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -815,6 +791,9 @@
       <c r="H4" s="5" t="s">
         <v>70</v>
       </c>
+      <c r="I4" s="5" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
@@ -838,6 +817,9 @@
       <c r="H5" s="5" t="s">
         <v>70</v>
       </c>
+      <c r="I5" s="5" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
@@ -861,6 +843,9 @@
       <c r="H6" s="5" t="s">
         <v>70</v>
       </c>
+      <c r="I6" s="5" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -884,6 +869,9 @@
       <c r="H7" s="5" t="s">
         <v>70</v>
       </c>
+      <c r="I7" s="5" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
@@ -907,6 +895,9 @@
       <c r="H8" s="5" t="s">
         <v>70</v>
       </c>
+      <c r="I8" s="5" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -930,6 +921,9 @@
       <c r="H9" s="5" t="s">
         <v>70</v>
       </c>
+      <c r="I9" s="5" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
@@ -953,6 +947,9 @@
       <c r="H10" s="5" t="s">
         <v>70</v>
       </c>
+      <c r="I10" s="5" t="s">
+        <v>70</v>
+      </c>
       <c r="J10" t="s">
         <v>39</v>
       </c>
@@ -982,6 +979,9 @@
       <c r="H11" s="5" t="s">
         <v>70</v>
       </c>
+      <c r="I11" s="5" t="s">
+        <v>70</v>
+      </c>
       <c r="J11" t="s">
         <v>40</v>
       </c>
@@ -1008,6 +1008,9 @@
       <c r="H12" s="5" t="s">
         <v>70</v>
       </c>
+      <c r="I12" s="5" t="s">
+        <v>70</v>
+      </c>
       <c r="J12" t="s">
         <v>22</v>
       </c>
@@ -1034,6 +1037,9 @@
       <c r="H13" s="5" t="s">
         <v>70</v>
       </c>
+      <c r="I13" s="5" t="s">
+        <v>70</v>
+      </c>
       <c r="J13" t="s">
         <v>28</v>
       </c>
@@ -1061,6 +1067,9 @@
       <c r="H14" s="5" t="s">
         <v>70</v>
       </c>
+      <c r="I14" s="5" t="s">
+        <v>70</v>
+      </c>
       <c r="J14" t="s">
         <v>29</v>
       </c>
@@ -1087,6 +1096,9 @@
       <c r="H15" s="5" t="s">
         <v>70</v>
       </c>
+      <c r="I15" s="5" t="s">
+        <v>70</v>
+      </c>
       <c r="J15" t="s">
         <v>34</v>
       </c>
@@ -1113,11 +1125,14 @@
       <c r="H16" s="5" t="s">
         <v>70</v>
       </c>
+      <c r="I16" s="5" t="s">
+        <v>70</v>
+      </c>
       <c r="J16" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>42</v>
       </c>
@@ -1125,7 +1140,7 @@
         <v>18</v>
       </c>
       <c r="C17" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D17" t="s">
         <v>20</v>
@@ -1139,8 +1154,11 @@
       <c r="H17" s="5" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I17" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>42</v>
       </c>
@@ -1162,8 +1180,11 @@
       <c r="H18" s="5" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I18" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>42</v>
       </c>
@@ -1185,8 +1206,11 @@
       <c r="H19" s="5" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I19" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>42</v>
       </c>
@@ -1208,8 +1232,11 @@
       <c r="H20" s="5" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I20" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>42</v>
       </c>
@@ -1231,8 +1258,11 @@
       <c r="H21" s="5" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I21" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>42</v>
       </c>
@@ -1254,8 +1284,11 @@
       <c r="H22" s="5" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I22" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>42</v>
       </c>
@@ -1277,36 +1310,45 @@
       <c r="H23" s="5" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I23" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B24" t="s">
         <v>5</v>
       </c>
       <c r="C24" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D24" t="s">
         <v>7</v>
       </c>
       <c r="E24" t="s">
-        <v>73</v>
+        <v>72</v>
+      </c>
+      <c r="G24" t="s">
+        <v>12</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B25" t="s">
         <v>5</v>
       </c>
       <c r="C25" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D25" t="s">
         <v>7</v>
@@ -1314,19 +1356,25 @@
       <c r="E25" t="s">
         <v>45</v>
       </c>
+      <c r="G25" t="s">
+        <v>12</v>
+      </c>
       <c r="H25" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B26" t="s">
         <v>5</v>
       </c>
       <c r="C26" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D26" t="s">
         <v>7</v>
@@ -1334,19 +1382,25 @@
       <c r="E26" t="s">
         <v>49</v>
       </c>
+      <c r="G26" t="s">
+        <v>12</v>
+      </c>
       <c r="H26" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B27" t="s">
         <v>5</v>
       </c>
       <c r="C27" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D27" t="s">
         <v>7</v>
@@ -1354,19 +1408,25 @@
       <c r="E27" t="s">
         <v>57</v>
       </c>
+      <c r="G27" t="s">
+        <v>12</v>
+      </c>
       <c r="H27" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B28" t="s">
         <v>5</v>
       </c>
       <c r="C28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D28" t="s">
         <v>7</v>
@@ -1374,19 +1434,25 @@
       <c r="E28" t="s">
         <v>58</v>
       </c>
+      <c r="G28" t="s">
+        <v>12</v>
+      </c>
       <c r="H28" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B29" t="s">
         <v>5</v>
       </c>
       <c r="C29" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D29" t="s">
         <v>7</v>
@@ -1394,19 +1460,25 @@
       <c r="E29" t="s">
         <v>60</v>
       </c>
+      <c r="G29" t="s">
+        <v>12</v>
+      </c>
       <c r="H29" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B30" t="s">
         <v>5</v>
       </c>
       <c r="C30" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D30" t="s">
         <v>7</v>
@@ -1414,36 +1486,48 @@
       <c r="E30" t="s">
         <v>59</v>
       </c>
+      <c r="G30" t="s">
+        <v>12</v>
+      </c>
       <c r="H30" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>76</v>
+      </c>
+      <c r="B31" t="s">
+        <v>74</v>
+      </c>
+      <c r="C31" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>77</v>
-      </c>
-      <c r="B31" t="s">
-        <v>75</v>
-      </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
+        <v>7</v>
+      </c>
+      <c r="E31" t="s">
         <v>72</v>
       </c>
-      <c r="D31" t="s">
-        <v>7</v>
-      </c>
-      <c r="E31" t="s">
-        <v>73</v>
+      <c r="G31" t="s">
+        <v>12</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+      <c r="I31" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B32" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C32" t="s">
         <v>56</v>
@@ -1454,16 +1538,22 @@
       <c r="E32" t="s">
         <v>45</v>
       </c>
+      <c r="G32" t="s">
+        <v>12</v>
+      </c>
       <c r="H32" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+      <c r="I32" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B33" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C33" t="s">
         <v>61</v>
@@ -1474,16 +1564,22 @@
       <c r="E33" t="s">
         <v>49</v>
       </c>
+      <c r="G33" t="s">
+        <v>12</v>
+      </c>
       <c r="H33" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B34" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C34" t="s">
         <v>62</v>
@@ -1494,16 +1590,22 @@
       <c r="E34" t="s">
         <v>57</v>
       </c>
+      <c r="G34" t="s">
+        <v>12</v>
+      </c>
       <c r="H34" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B35" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C35" t="s">
         <v>63</v>
@@ -1514,16 +1616,22 @@
       <c r="E35" t="s">
         <v>58</v>
       </c>
+      <c r="G35" t="s">
+        <v>12</v>
+      </c>
       <c r="H35" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+      <c r="I35" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B36" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C36" t="s">
         <v>64</v>
@@ -1534,16 +1642,22 @@
       <c r="E36" t="s">
         <v>60</v>
       </c>
+      <c r="G36" t="s">
+        <v>12</v>
+      </c>
       <c r="H36" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+      <c r="I36" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B37" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C37" t="s">
         <v>65</v>
@@ -1554,23 +1668,156 @@
       <c r="E37" t="s">
         <v>59</v>
       </c>
+      <c r="G37" t="s">
+        <v>12</v>
+      </c>
       <c r="H37" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
+      </c>
+      <c r="I37" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>84</v>
+      </c>
+      <c r="B38" t="s">
+        <v>74</v>
+      </c>
+      <c r="C38" t="s">
+        <v>56</v>
+      </c>
+      <c r="D38" t="s">
+        <v>7</v>
+      </c>
+      <c r="E38" t="s">
+        <v>45</v>
+      </c>
+      <c r="G38" t="s">
+        <v>12</v>
+      </c>
+      <c r="H38" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>84</v>
+      </c>
+      <c r="B39" t="s">
+        <v>74</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39" t="s">
+        <v>7</v>
+      </c>
+      <c r="E39" t="s">
+        <v>49</v>
+      </c>
+      <c r="G39" t="s">
+        <v>12</v>
+      </c>
+      <c r="H39" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>84</v>
+      </c>
+      <c r="B40" t="s">
+        <v>74</v>
+      </c>
+      <c r="C40" t="s">
+        <v>62</v>
+      </c>
+      <c r="D40" t="s">
+        <v>7</v>
+      </c>
+      <c r="E40" t="s">
+        <v>57</v>
+      </c>
+      <c r="G40" t="s">
+        <v>12</v>
+      </c>
+      <c r="H40" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>84</v>
+      </c>
+      <c r="B41" t="s">
+        <v>74</v>
+      </c>
+      <c r="C41" t="s">
+        <v>63</v>
+      </c>
+      <c r="D41" t="s">
+        <v>7</v>
+      </c>
+      <c r="E41" t="s">
+        <v>58</v>
+      </c>
+      <c r="G41" t="s">
+        <v>12</v>
+      </c>
+      <c r="H41" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>84</v>
+      </c>
+      <c r="B42" t="s">
+        <v>74</v>
+      </c>
+      <c r="C42" t="s">
+        <v>64</v>
+      </c>
+      <c r="D42" t="s">
+        <v>7</v>
+      </c>
+      <c r="E42" t="s">
+        <v>60</v>
+      </c>
+      <c r="G42" t="s">
+        <v>12</v>
+      </c>
+      <c r="H42" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>84</v>
+      </c>
+      <c r="B43" t="s">
+        <v>74</v>
+      </c>
+      <c r="C43" t="s">
+        <v>65</v>
+      </c>
+      <c r="D43" t="s">
+        <v>7</v>
+      </c>
+      <c r="E43" t="s">
+        <v>59</v>
+      </c>
+      <c r="G43" t="s">
+        <v>12</v>
+      </c>
+      <c r="H43" s="5" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:I30">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
-      <formula>"In Progress"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
-      <formula>"True"</formula>
-    </cfRule>
-    <cfRule type="containsBlanks" dxfId="3" priority="6">
-      <formula>LEN(TRIM(H2))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H31:I37">
+  <conditionalFormatting sqref="H2:I43">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>
@@ -1578,7 +1825,7 @@
       <formula>"True"</formula>
     </cfRule>
     <cfRule type="containsBlanks" dxfId="0" priority="3">
-      <formula>LEN(TRIM(H31))=0</formula>
+      <formula>LEN(TRIM(H2))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1657,6 +1904,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="897f6830-f425-409d-b8f5-ce1019056d9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="f2404b4d-361b-46d3-b2ec-035eed29e274" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101004FB79D76D905EB41B4AD64ED4839597F" ma:contentTypeVersion="11" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="0622d98e252eab518d4b54f931ba6851">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="897f6830-f425-409d-b8f5-ce1019056d9e" xmlns:ns3="f2404b4d-361b-46d3-b2ec-035eed29e274" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dd5f302b3846fd12003b89c8f5b7df36" ns2:_="" ns3:_="">
     <xsd:import namespace="897f6830-f425-409d-b8f5-ce1019056d9e"/>
@@ -1851,17 +2109,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="897f6830-f425-409d-b8f5-ce1019056d9e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="f2404b4d-361b-46d3-b2ec-035eed29e274" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
   <ds:schemaRefs>
@@ -1871,6 +2118,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF16440F-B0E0-4269-97EE-BEB05B0223C8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="897f6830-f425-409d-b8f5-ce1019056d9e"/>
+    <ds:schemaRef ds:uri="f2404b4d-361b-46d3-b2ec-035eed29e274"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A33EE264-283E-4F19-BA61-B3264EA417E2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1887,15 +2145,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF16440F-B0E0-4269-97EE-BEB05B0223C8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="897f6830-f425-409d-b8f5-ce1019056d9e"/>
-    <ds:schemaRef ds:uri="f2404b4d-361b-46d3-b2ec-035eed29e274"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updated restapiPropertyDictionary Java code generation.
</commit_message>
<xml_diff>
--- a/AWB-RestApi-PropertyDictionary.xlsx
+++ b/AWB-RestApi-PropertyDictionary.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\AgentWorkbench\eclipseProjects\de.enflexit.awb\bundles\web\xApi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AEF8AAF-C845-4942-8C9B-A574FB5C1D1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27507518-1AE7-4149-A7A0-648A1B12E337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38290" yWindow="10770" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Property-Definition" sheetId="1" r:id="rId1"/>
     <sheet name="Java-Code" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Java-Code'!$A$1:$B$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Java-Code'!$A$1:$B$93</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="194">
   <si>
     <t>key</t>
   </si>
@@ -439,9 +439,6 @@
   </si>
   <si>
     <t>always de.enflexit.awb.bgSystem.db</t>
-  </si>
-  <si>
-    <t>bgsystem.auto_init</t>
   </si>
   <si>
     <t>server.master.protocol</t>
@@ -1004,7 +1001,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K93"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="28.7265625" customWidth="1"/>
@@ -2205,7 +2202,7 @@
         <v>103</v>
       </c>
       <c r="H44" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I44" s="5" t="s">
         <v>59</v>
@@ -2231,7 +2228,7 @@
         <v>116</v>
       </c>
       <c r="H45" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I45" s="5" t="s">
         <v>59</v>
@@ -2257,7 +2254,7 @@
         <v>117</v>
       </c>
       <c r="H46" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I46" s="5" t="s">
         <v>59</v>
@@ -2283,7 +2280,7 @@
         <v>117</v>
       </c>
       <c r="H47" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I47" s="5" t="s">
         <v>59</v>
@@ -2300,7 +2297,7 @@
         <v>74</v>
       </c>
       <c r="D48" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E48" t="s">
         <v>7</v>
@@ -2312,7 +2309,7 @@
         <v>75</v>
       </c>
       <c r="H48" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I48" s="5" t="s">
         <v>59</v>
@@ -2341,7 +2338,7 @@
         <v>129</v>
       </c>
       <c r="H49" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I49" s="5" t="s">
         <v>59</v>
@@ -2367,7 +2364,7 @@
         <v>118</v>
       </c>
       <c r="H50" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I50" s="5" t="s">
         <v>59</v>
@@ -2393,7 +2390,7 @@
         <v>119</v>
       </c>
       <c r="H51" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I51" s="5" t="s">
         <v>59</v>
@@ -2422,7 +2419,7 @@
         <v>75</v>
       </c>
       <c r="H52" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I52" s="5" t="s">
         <v>59</v>
@@ -2448,7 +2445,7 @@
         <v>121</v>
       </c>
       <c r="H53" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I53" s="5" t="s">
         <v>59</v>
@@ -2474,10 +2471,10 @@
         <v>102</v>
       </c>
       <c r="G54" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H54" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I54" s="5" t="s">
         <v>59</v>
@@ -2503,7 +2500,7 @@
         <v>122</v>
       </c>
       <c r="H55" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I55" s="5" t="s">
         <v>59</v>
@@ -2529,7 +2526,7 @@
         <v>123</v>
       </c>
       <c r="H56" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I56" s="5" t="s">
         <v>59</v>
@@ -2555,7 +2552,7 @@
         <v>124</v>
       </c>
       <c r="H57" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I57" s="5" t="s">
         <v>59</v>
@@ -2572,16 +2569,16 @@
         <v>5</v>
       </c>
       <c r="D58" t="s">
+        <v>138</v>
+      </c>
+      <c r="E58" t="s">
+        <v>7</v>
+      </c>
+      <c r="F58" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="E58" t="s">
-        <v>7</v>
-      </c>
-      <c r="F58" s="6" t="s">
-        <v>140</v>
-      </c>
       <c r="H58" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I58" s="5" t="s">
         <v>59</v>
@@ -2607,7 +2604,7 @@
         <v>132</v>
       </c>
       <c r="H59" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I59" s="5" t="s">
         <v>59</v>
@@ -2618,65 +2615,71 @@
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="C60" t="s">
         <v>5</v>
       </c>
       <c r="D60" t="s">
-        <v>133</v>
-      </c>
-      <c r="H60" t="s">
-        <v>137</v>
+        <v>127</v>
+      </c>
+      <c r="E60" t="s">
+        <v>7</v>
+      </c>
+      <c r="F60" t="s">
+        <v>122</v>
       </c>
       <c r="I60" s="5" t="s">
         <v>59</v>
       </c>
       <c r="J60" s="5" t="s">
         <v>59</v>
+      </c>
+      <c r="K60" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C61" t="s">
         <v>5</v>
       </c>
       <c r="D61" t="s">
-        <v>127</v>
+        <v>92</v>
       </c>
       <c r="E61" t="s">
         <v>7</v>
       </c>
       <c r="F61" t="s">
-        <v>122</v>
+        <v>93</v>
       </c>
       <c r="I61" s="5" t="s">
         <v>59</v>
       </c>
       <c r="J61" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="K61" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>94</v>
+        <v>95</v>
+      </c>
+      <c r="B62" t="s">
+        <v>97</v>
       </c>
       <c r="C62" t="s">
         <v>5</v>
       </c>
       <c r="D62" t="s">
-        <v>92</v>
+        <v>137</v>
       </c>
       <c r="E62" t="s">
         <v>7</v>
       </c>
       <c r="F62" t="s">
-        <v>93</v>
+        <v>126</v>
       </c>
       <c r="I62" s="5" t="s">
         <v>59</v>
@@ -2687,27 +2690,21 @@
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>95</v>
-      </c>
-      <c r="B63" t="s">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="C63" t="s">
         <v>5</v>
       </c>
       <c r="D63" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E63" t="s">
         <v>7</v>
       </c>
       <c r="F63" t="s">
-        <v>126</v>
+        <v>172</v>
       </c>
       <c r="I63" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="J63" s="5" t="s">
         <v>59</v>
       </c>
     </row>
@@ -2725,7 +2722,7 @@
         <v>7</v>
       </c>
       <c r="F64" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I64" s="5" t="s">
         <v>59</v>
@@ -2742,10 +2739,10 @@
         <v>142</v>
       </c>
       <c r="E65" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="F65" t="s">
-        <v>175</v>
+        <v>21</v>
       </c>
       <c r="I65" s="5" t="s">
         <v>59</v>
@@ -2762,10 +2759,10 @@
         <v>143</v>
       </c>
       <c r="E66" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="F66" t="s">
-        <v>21</v>
+        <v>183</v>
       </c>
       <c r="I66" s="5" t="s">
         <v>59</v>
@@ -2785,7 +2782,7 @@
         <v>7</v>
       </c>
       <c r="F67" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="I67" s="5" t="s">
         <v>59</v>
@@ -2802,10 +2799,10 @@
         <v>145</v>
       </c>
       <c r="E68" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="F68" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="I68" s="5" t="s">
         <v>59</v>
@@ -2822,10 +2819,10 @@
         <v>146</v>
       </c>
       <c r="E69" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="F69" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="I69" s="5" t="s">
         <v>59</v>
@@ -2842,10 +2839,10 @@
         <v>147</v>
       </c>
       <c r="E70" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="F70" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="I70" s="5" t="s">
         <v>59</v>
@@ -2885,7 +2882,7 @@
         <v>26</v>
       </c>
       <c r="F72" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I72" s="5" t="s">
         <v>59</v>
@@ -2905,7 +2902,7 @@
         <v>26</v>
       </c>
       <c r="F73" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="I73" s="5" t="s">
         <v>59</v>
@@ -2922,10 +2919,10 @@
         <v>151</v>
       </c>
       <c r="E74" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="F74" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="I74" s="5" t="s">
         <v>59</v>
@@ -2979,13 +2976,13 @@
         <v>5</v>
       </c>
       <c r="D77" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E77" t="s">
         <v>7</v>
       </c>
       <c r="F77" t="s">
-        <v>192</v>
+        <v>175</v>
       </c>
       <c r="I77" s="5" t="s">
         <v>59</v>
@@ -2999,10 +2996,10 @@
         <v>5</v>
       </c>
       <c r="D78" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E78" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="F78" t="s">
         <v>176</v>
@@ -3019,13 +3016,13 @@
         <v>5</v>
       </c>
       <c r="D79" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E79" t="s">
         <v>26</v>
       </c>
       <c r="F79" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="I79" s="5" t="s">
         <v>59</v>
@@ -3065,7 +3062,7 @@
         <v>26</v>
       </c>
       <c r="F81" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="I81" s="5" t="s">
         <v>59</v>
@@ -3082,10 +3079,10 @@
         <v>159</v>
       </c>
       <c r="E82" t="s">
-        <v>26</v>
+        <v>160</v>
       </c>
       <c r="F82" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="I82" s="5" t="s">
         <v>59</v>
@@ -3099,13 +3096,13 @@
         <v>5</v>
       </c>
       <c r="D83" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="E83" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="F83" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="I83" s="5" t="s">
         <v>59</v>
@@ -3122,7 +3119,7 @@
         <v>168</v>
       </c>
       <c r="E84" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F84" t="s">
         <v>186</v>
@@ -3142,10 +3139,10 @@
         <v>169</v>
       </c>
       <c r="E85" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F85" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I85" s="5" t="s">
         <v>59</v>
@@ -3162,10 +3159,10 @@
         <v>170</v>
       </c>
       <c r="E86" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F86" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I86" s="5" t="s">
         <v>59</v>
@@ -3179,13 +3176,13 @@
         <v>5</v>
       </c>
       <c r="D87" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="E87" t="s">
-        <v>172</v>
+        <v>20</v>
       </c>
       <c r="F87" t="s">
-        <v>187</v>
+        <v>21</v>
       </c>
       <c r="I87" s="5" t="s">
         <v>59</v>
@@ -3202,10 +3199,10 @@
         <v>162</v>
       </c>
       <c r="E88" t="s">
-        <v>20</v>
+        <v>160</v>
       </c>
       <c r="F88" t="s">
-        <v>21</v>
+        <v>179</v>
       </c>
       <c r="I88" s="5" t="s">
         <v>59</v>
@@ -3222,10 +3219,10 @@
         <v>163</v>
       </c>
       <c r="E89" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F89" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="I89" s="5" t="s">
         <v>59</v>
@@ -3242,10 +3239,10 @@
         <v>164</v>
       </c>
       <c r="E90" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F90" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I90" s="5" t="s">
         <v>59</v>
@@ -3262,7 +3259,7 @@
         <v>165</v>
       </c>
       <c r="E91" t="s">
-        <v>161</v>
+        <v>26</v>
       </c>
       <c r="F91" t="s">
         <v>181</v>
@@ -3282,37 +3279,17 @@
         <v>166</v>
       </c>
       <c r="E92" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F92" t="s">
-        <v>182</v>
+        <v>21</v>
       </c>
       <c r="I92" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A93" t="s">
-        <v>83</v>
-      </c>
-      <c r="C93" t="s">
-        <v>5</v>
-      </c>
-      <c r="D93" t="s">
-        <v>167</v>
-      </c>
-      <c r="E93" t="s">
-        <v>20</v>
-      </c>
-      <c r="F93" t="s">
-        <v>21</v>
-      </c>
-      <c r="I93" s="5" t="s">
-        <v>59</v>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:J43 J44:J63 I44:I93">
+  <conditionalFormatting sqref="I2:J43 J44:J62 I44:I92">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>
@@ -3330,8 +3307,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F30A1E73-A707-4178-9C72-9AC27F9EE5F7}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:B135"/>
+  <dimension ref="A1:B93"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24.6328125" bestFit="1" customWidth="1"/>
@@ -3344,2163 +3320,1773 @@
         <v>performative</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="str">
         <f>'Property-Definition'!A2</f>
         <v>DB.SYSTEMS</v>
       </c>
       <c r="B2" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D2,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D2 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String DBSYSTEM[X] = "dbSystem[X]";</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D2,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D2
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String DBSYSTEM = "dbSystem[X]";</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="str">
         <f>'Property-Definition'!A3</f>
         <v>DB.SYSTEMS.PARAMETER</v>
       </c>
       <c r="B3" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D3,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D3 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String DBSYSTEM[X] = "dbSystem[X]";</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D3,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D3
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String DBSYSTEM = "dbSystem[X]";</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="str">
         <f>'Property-Definition'!A4</f>
         <v>DB.SYSTEMS.PARAMETER</v>
       </c>
       <c r="B4" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D4,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D4 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String DBSYSTEM[X]_HIBERNATE_CONNECTION_DRIVER_CLASS = "dbSystem[X].hibernate.connection.driver_class";</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D4,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D4
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_DRIVER_CLASS = "dbSystem[X].hibernate.connection.driver_class";</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="str">
         <f>'Property-Definition'!A5</f>
         <v>DB.SYSTEMS.PARAMETER</v>
       </c>
       <c r="B5" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D5,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D5 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String DBSYSTEM[X]_HIBERNATE_CONNECTION_URL = "dbSystem[X].hibernate.connection.url";</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D5,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D5
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_URL = "dbSystem[X].hibernate.connection.url";</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="str">
         <f>'Property-Definition'!A6</f>
         <v>DB.SYSTEMS.PARAMETER</v>
       </c>
       <c r="B6" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D6,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D6 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String DBSYSTEM[X]_HIBERNATE_CONNECTION_URL_MASK = "dbSystem[X].hibernate.connection.url.mask";</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D6,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D6
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_URL_MASK = "dbSystem[X].hibernate.connection.url.mask";</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="str">
         <f>'Property-Definition'!A7</f>
         <v>DB.SYSTEMS.PARAMETER</v>
       </c>
       <c r="B7" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D7,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D7 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String DBSYSTEM[X]_HIBERNATE_DEFAULT_CATALOG = "dbSystem[X].hibernate.default_catalog";</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D7,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D7
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String DBSYSTEM_HIBERNATE_DEFAULT_CATALOG = "dbSystem[X].hibernate.default_catalog";</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="str">
         <f>'Property-Definition'!A8</f>
         <v>DB.SYSTEMS.PARAMETER</v>
       </c>
       <c r="B8" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D8,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D8 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String DBSYSTEM[X]_HIBERNATE_CONNECTION_USERNAME = "dbSystem[X].hibernate.connection.username";</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D8,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D8
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_USERNAME = "dbSystem[X].hibernate.connection.username";</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="str">
         <f>'Property-Definition'!A9</f>
         <v>DB.SYSTEMS.PARAMETER</v>
       </c>
       <c r="B9" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D9,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D9 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String DBSYSTEM[X]_HIBERNATE_CONNECTION_PASSWORD = "dbSystem[X].hibernate.connection.password";</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D9,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D9
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_PASSWORD = "dbSystem[X].hibernate.connection.password";</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="str">
         <f>'Property-Definition'!A10</f>
         <v>DB.FACTORIES</v>
       </c>
       <c r="B10" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D10,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D10 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String FACTORY[X] = "factory[X]";</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D10,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D10
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String FACTORY = "factory[X]";</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="str">
         <f>'Property-Definition'!A11</f>
         <v>DB.FACTORIES</v>
       </c>
       <c r="B11" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D11,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D11 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String FACTORY[X]_STATE = "factory[X].state";</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D11,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D11
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String FACTORY_STATE = "factory[X].state";</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="str">
         <f>'Property-Definition'!A12</f>
         <v>DB.DERBY.NETWORKSERVER</v>
       </c>
       <c r="B12" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D12,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D12 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D12,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D12
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String ISSTARTDERBYNETWORKSERVER = "isStartDerbyNetworkServer";</v>
       </c>
     </row>
-    <row r="13" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="str">
         <f>'Property-Definition'!A13</f>
         <v>DB.DERBY.NETWORKSERVER</v>
       </c>
       <c r="B13" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D13,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D13 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D13,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D13
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String HOST-IP = "host-IP";</v>
       </c>
     </row>
-    <row r="14" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="str">
         <f>'Property-Definition'!A14</f>
         <v>DB.DERBY.NETWORKSERVER</v>
       </c>
       <c r="B14" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D14,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D14 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D14,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D14
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String PORT = "port";</v>
       </c>
     </row>
-    <row r="15" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="str">
         <f>'Property-Definition'!A15</f>
         <v>DB.DERBY.NETWORKSERVER</v>
       </c>
       <c r="B15" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D15,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D15 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D15,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D15
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String USERNAME = "userName";</v>
       </c>
     </row>
-    <row r="16" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="str">
         <f>'Property-Definition'!A16</f>
         <v>DB.DERBY.NETWORKSERVER</v>
       </c>
       <c r="B16" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D16,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D16 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D16,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D16
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String PASSWORD = "password";</v>
       </c>
     </row>
-    <row r="17" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="str">
         <f>'Property-Definition'!A17</f>
         <v>DB.CONN.GENERAL</v>
       </c>
       <c r="B17" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D17,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D17 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D17,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D17
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String USEFOREVERYFACTORY = "useForEveryFactory";</v>
       </c>
     </row>
-    <row r="18" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="str">
         <f>'Property-Definition'!A18</f>
         <v>DB.CONN.GENERAL</v>
       </c>
       <c r="B18" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D18,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D18 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D18,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D18
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String DBSYSTEM = "dbSystem";</v>
       </c>
     </row>
-    <row r="19" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="str">
         <f>'Property-Definition'!A19</f>
         <v>DB.CONN.GENERAL</v>
       </c>
       <c r="B19" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D19,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D19 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D19,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D19
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String HIBERNATE_CONNECTION_DRIVER_CLASS = "hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="20" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="str">
         <f>'Property-Definition'!A20</f>
         <v>DB.CONN.GENERAL</v>
       </c>
       <c r="B20" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D20,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D20 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D20,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D20
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String HIBERNATE_CONNECTION_URL = "hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="21" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="str">
         <f>'Property-Definition'!A21</f>
         <v>DB.CONN.GENERAL</v>
       </c>
       <c r="B21" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D21,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D21 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D21,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D21
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String HIBERNATE_DEFAULT_CATALOG = "hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="22" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="str">
         <f>'Property-Definition'!A22</f>
         <v>DB.CONN.GENERAL</v>
       </c>
       <c r="B22" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D22,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D22 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D22,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D22
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String HIBERNATE_CONNECTION_USERNAME = "hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="23" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="str">
         <f>'Property-Definition'!A23</f>
         <v>DB.CONN.GENERAL</v>
       </c>
       <c r="B23" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D23,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D23 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D23,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D23
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String HIBERNATE_CONNECTION_PASSWORD = "hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="24" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="str">
         <f>'Property-Definition'!A24</f>
         <v>DB.CONN.FACTORY.GET</v>
       </c>
       <c r="B24" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D24,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D24 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String FACTORY[X]_FACTORYID = "factory[X].factoryID";</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D24,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D24
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String FACTORY_FACTORYID = "factory[X].factoryID";</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="str">
         <f>'Property-Definition'!A25</f>
         <v>DB.CONN.FACTORY.GET</v>
       </c>
       <c r="B25" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D25,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D25 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String FACTORY[X]_DBSYSTEM = "factory[X].dbSystem";</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D25,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D25
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String FACTORY_DBSYSTEM = "factory[X].dbSystem";</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="str">
         <f>'Property-Definition'!A26</f>
         <v>DB.CONN.FACTORY.GET</v>
       </c>
       <c r="B26" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D26,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D26 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String FACTORY[X]_HIBERNATE_CONNECTION_DRIVER_CLASS = "factory[X].hibernate.connection.driver_class";</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D26,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D26
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String FACTORY_HIBERNATE_CONNECTION_DRIVER_CLASS = "factory[X].hibernate.connection.driver_class";</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="str">
         <f>'Property-Definition'!A27</f>
         <v>DB.CONN.FACTORY.GET</v>
       </c>
       <c r="B27" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D27,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D27 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String FACTORY[X]_HIBERNATE_CONNECTION_URL = "factory[X].hibernate.connection.url";</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D27,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D27
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String FACTORY_HIBERNATE_CONNECTION_URL = "factory[X].hibernate.connection.url";</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="str">
         <f>'Property-Definition'!A28</f>
         <v>DB.CONN.FACTORY.GET</v>
       </c>
       <c r="B28" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D28,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D28 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String FACTORY[X]_HIBERNATE_DEFAULT_CATALOG = "factory[X].hibernate.default_catalog";</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D28,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D28
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String FACTORY_HIBERNATE_DEFAULT_CATALOG = "factory[X].hibernate.default_catalog";</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="str">
         <f>'Property-Definition'!A29</f>
         <v>DB.CONN.FACTORY.GET</v>
       </c>
       <c r="B29" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D29,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D29 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String FACTORY[X]_HIBERNATE_CONNECTION_USERNAME = "factory[X].hibernate.connection.username";</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D29,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D29
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String FACTORY_HIBERNATE_CONNECTION_USERNAME = "factory[X].hibernate.connection.username";</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="str">
         <f>'Property-Definition'!A30</f>
         <v>DB.CONN.FACTORY.GET</v>
       </c>
       <c r="B30" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D30,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D30 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String FACTORY[X]_HIBERNATE_CONNECTION_PASSWORD = "factory[X].hibernate.connection.password";</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D30,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D30
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String FACTORY_HIBERNATE_CONNECTION_PASSWORD = "factory[X].hibernate.connection.password";</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="str">
         <f>'Property-Definition'!A31</f>
         <v>DB.CONN.FACTORY.SET</v>
       </c>
       <c r="B31" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D31,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D31 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D31,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D31
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String FACTORYID = "factoryID";</v>
       </c>
     </row>
-    <row r="32" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="str">
         <f>'Property-Definition'!A32</f>
         <v>DB.CONN.FACTORY.SET</v>
       </c>
       <c r="B32" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D32,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D32 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D32,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D32
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String DBSYSTEM = "dbSystem";</v>
       </c>
     </row>
-    <row r="33" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="str">
         <f>'Property-Definition'!A33</f>
         <v>DB.CONN.FACTORY.SET</v>
       </c>
       <c r="B33" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D33,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D33 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D33,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D33
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String HIBERNATE_CONNECTION_DRIVER_CLASS = "hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="34" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="str">
         <f>'Property-Definition'!A34</f>
         <v>DB.CONN.FACTORY.SET</v>
       </c>
       <c r="B34" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D34,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D34 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D34,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D34
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String HIBERNATE_CONNECTION_URL = "hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="35" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="str">
         <f>'Property-Definition'!A35</f>
         <v>DB.CONN.FACTORY.SET</v>
       </c>
       <c r="B35" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D35,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D35 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D35,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D35
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String HIBERNATE_DEFAULT_CATALOG = "hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="36" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="str">
         <f>'Property-Definition'!A36</f>
         <v>DB.CONN.FACTORY.SET</v>
       </c>
       <c r="B36" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D36,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D36 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D36,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D36
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String HIBERNATE_CONNECTION_USERNAME = "hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="37" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="str">
         <f>'Property-Definition'!A37</f>
         <v>DB.CONN.FACTORY.SET</v>
       </c>
       <c r="B37" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D37,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D37 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D37,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D37
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String HIBERNATE_CONNECTION_PASSWORD = "hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="38" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="str">
         <f>'Property-Definition'!A38</f>
         <v>DB.CONN.TEST</v>
       </c>
       <c r="B38" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D38,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D38 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D38,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D38
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String DBSYSTEM = "dbSystem";</v>
       </c>
     </row>
-    <row r="39" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="str">
         <f>'Property-Definition'!A39</f>
         <v>DB.CONN.TEST</v>
       </c>
       <c r="B39" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D39,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D39 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D39,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D39
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String HIBERNATE_CONNECTION_DRIVER_CLASS = "hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="40" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="str">
         <f>'Property-Definition'!A40</f>
         <v>DB.CONN.TEST</v>
       </c>
       <c r="B40" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D40,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D40 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D40,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D40
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String HIBERNATE_CONNECTION_URL = "hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="41" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="str">
         <f>'Property-Definition'!A41</f>
         <v>DB.CONN.TEST</v>
       </c>
       <c r="B41" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D41,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D41 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D41,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D41
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String HIBERNATE_DEFAULT_CATALOG = "hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="42" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="str">
         <f>'Property-Definition'!A42</f>
         <v>DB.CONN.TEST</v>
       </c>
       <c r="B42" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D42,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D42 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D42,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D42
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String HIBERNATE_CONNECTION_USERNAME = "hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="43" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="str">
         <f>'Property-Definition'!A43</f>
         <v>DB.CONN.TEST</v>
       </c>
       <c r="B43" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D43,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D43 &amp; CHAR(34)&amp; ";"</f>
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D43,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D43
+&amp; CHAR(34)
+&amp; ";"</f>
         <v>public final static String HIBERNATE_CONNECTION_PASSWORD = "hibernate.connection.password";</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="str">
-        <f>'Property-Definition'!A2</f>
-        <v>DB.SYSTEMS</v>
+        <f>'Property-Definition'!A44</f>
+        <v>EXEC.MODE</v>
       </c>
       <c r="B44" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D2,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D2
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String DBSYSTEM="dbSystem[X]";</v>
+        SUBSTITUTE('Property-Definition'!D44,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D44
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String EXEC_MODE = "exec.mode";</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="str">
-        <f>'Property-Definition'!A3</f>
-        <v>DB.SYSTEMS.PARAMETER</v>
+        <f>'Property-Definition'!A45</f>
+        <v>EXEC.MODE</v>
       </c>
       <c r="B45" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D3,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D3
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String DBSYSTEM="dbSystem[X]";</v>
+        SUBSTITUTE('Property-Definition'!D45,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D45
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String SERVER_MASTER_URL = "server.master.url";</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="str">
-        <f>'Property-Definition'!A4</f>
-        <v>DB.SYSTEMS.PARAMETER</v>
+        <f>'Property-Definition'!A46</f>
+        <v>EXEC.MODE</v>
       </c>
       <c r="B46" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D4,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D4
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_DRIVER_CLASS="dbSystem[X].hibernate.connection.driver_class";</v>
+        SUBSTITUTE('Property-Definition'!D46,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D46
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String SERVER_MASTER_PORT = "server.master.port";</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="str">
-        <f>'Property-Definition'!A5</f>
-        <v>DB.SYSTEMS.PARAMETER</v>
+        <f>'Property-Definition'!A47</f>
+        <v>EXEC.MODE</v>
       </c>
       <c r="B47" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D5,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D5
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_URL="dbSystem[X].hibernate.connection.url";</v>
+        SUBSTITUTE('Property-Definition'!D47,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D47
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String SERVER_MASTER_PORT_MTP = "server.master.port.mtp";</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="str">
-        <f>'Property-Definition'!A6</f>
-        <v>DB.SYSTEMS.PARAMETER</v>
+        <f>'Property-Definition'!A48</f>
+        <v>EXEC.MODE</v>
       </c>
       <c r="B48" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D6,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D6
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_URL_MASK="dbSystem[X].hibernate.connection.url.mask";</v>
+        SUBSTITUTE('Property-Definition'!D48,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D48
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String SERVER_MASTER_PROTOCOL = "server.master.protocol";</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="str">
-        <f>'Property-Definition'!A7</f>
-        <v>DB.SYSTEMS.PARAMETER</v>
+        <f>'Property-Definition'!A49</f>
+        <v>EXEC.MODE</v>
       </c>
       <c r="B49" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D7,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D7
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String DBSYSTEM_HIBERNATE_DEFAULT_CATALOG="dbSystem[X].hibernate.default_catalog";</v>
+        SUBSTITUTE('Property-Definition'!D49,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D49
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String LOCAL_MTP_CREATION = "local.mtp.creation";</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="str">
-        <f>'Property-Definition'!A8</f>
-        <v>DB.SYSTEMS.PARAMETER</v>
+        <f>'Property-Definition'!A50</f>
+        <v>EXEC.MODE</v>
       </c>
       <c r="B50" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D8,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D8
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_USERNAME="dbSystem[X].hibernate.connection.username";</v>
+        SUBSTITUTE('Property-Definition'!D50,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D50
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String LOCAL_MTP_URL = "local.mtp.url";</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="str">
-        <f>'Property-Definition'!A9</f>
-        <v>DB.SYSTEMS.PARAMETER</v>
+        <f>'Property-Definition'!A51</f>
+        <v>EXEC.MODE</v>
       </c>
       <c r="B51" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D9,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D9
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_PASSWORD="dbSystem[X].hibernate.connection.password";</v>
+        SUBSTITUTE('Property-Definition'!D51,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D51
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String LOCAL_MTP_PORT = "local.mtp.port";</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" t="str">
-        <f>'Property-Definition'!A10</f>
-        <v>DB.FACTORIES</v>
+        <f>'Property-Definition'!A52</f>
+        <v>EXEC.MODE</v>
       </c>
       <c r="B52" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D10,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D10
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String FACTORY="factory[X]";</v>
+        SUBSTITUTE('Property-Definition'!D52,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D52
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String LOCAL_MTP_PROTOCOL = "local.mtp.protocol";</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" t="str">
-        <f>'Property-Definition'!A11</f>
-        <v>DB.FACTORIES</v>
+        <f>'Property-Definition'!A53</f>
+        <v>EXEC.MODE</v>
       </c>
       <c r="B53" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D11,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D11
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String FACTORY_STATE="factory[X].state";</v>
+        SUBSTITUTE('Property-Definition'!D53,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D53
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String EMBEDDEDSYSTEM_PROJECT = "embeddedsystem.project";</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" t="str">
-        <f>'Property-Definition'!A12</f>
-        <v>DB.DERBY.NETWORKSERVER</v>
+        <f>'Property-Definition'!A54</f>
+        <v>EXEC.MODE</v>
       </c>
       <c r="B54" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D12,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D12
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String ISSTARTDERBYNETWORKSERVER="isStartDerbyNetworkServer";</v>
+        SUBSTITUTE('Property-Definition'!D54,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D54
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String DEVICE_SYSTEM_EXEC_MODE = "device_system_exec_mode";</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="str">
-        <f>'Property-Definition'!A13</f>
-        <v>DB.DERBY.NETWORKSERVER</v>
+        <f>'Property-Definition'!A55</f>
+        <v>EXEC.MODE</v>
       </c>
       <c r="B55" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D13,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D13
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String HOST-IP="host-IP";</v>
+        SUBSTITUTE('Property-Definition'!D55,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D55
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String EMBEDDEDSYSTEM_AGENT_CLASSNAME = "embeddedsystem.agent[X].classname";</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" t="str">
-        <f>'Property-Definition'!A14</f>
-        <v>DB.DERBY.NETWORKSERVER</v>
+        <f>'Property-Definition'!A56</f>
+        <v>EXEC.MODE</v>
       </c>
       <c r="B56" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D14,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D14
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String PORT="port";</v>
+        SUBSTITUTE('Property-Definition'!D56,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D56
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String EMBEDDEDSYSTEM_AGENT_AGENTNAME = "embeddedsystem.agent[X].agentname";</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="str">
-        <f>'Property-Definition'!A15</f>
-        <v>DB.DERBY.NETWORKSERVER</v>
+        <f>'Property-Definition'!A57</f>
+        <v>EXEC.MODE</v>
       </c>
       <c r="B57" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D15,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D15
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String USERNAME="userName";</v>
+        SUBSTITUTE('Property-Definition'!D57,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D57
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String SERVICE_SERVICE_SETUP = "service.service_setup";</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" t="str">
-        <f>'Property-Definition'!A16</f>
-        <v>DB.DERBY.NETWORKSERVER</v>
+        <f>'Property-Definition'!A58</f>
+        <v>EXEC.MODE</v>
       </c>
       <c r="B58" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D16,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D16
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String PASSWORD="password";</v>
+        SUBSTITUTE('Property-Definition'!D58,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D58
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String LOCAL_IP_SELECTION = "local.ip.selection[X]";</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" t="str">
-        <f>'Property-Definition'!A17</f>
-        <v>DB.CONN.GENERAL</v>
+        <f>'Property-Definition'!A59</f>
+        <v>EXEC.MODE</v>
       </c>
       <c r="B59" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D17,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D17
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String USEFOREVERYFACTORY="useForEveryFactory";</v>
+        SUBSTITUTE('Property-Definition'!D59,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D59
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String FACTORY_ID = "factory_id";</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A60" t="str">
-        <f>'Property-Definition'!A18</f>
-        <v>DB.CONN.GENERAL</v>
-      </c>
-      <c r="B60" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D18,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D18
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String DBSYSTEM="dbSystem";</v>
+      <c r="A60" t="e">
+        <f>'Property-Definition'!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="B60" t="e">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!#REF!,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!#REF!
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" t="str">
-        <f>'Property-Definition'!A19</f>
-        <v>DB.CONN.GENERAL</v>
+        <f>'Property-Definition'!A60</f>
+        <v>AWB.AGENTS</v>
       </c>
       <c r="B61" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D19,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D19
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String HIBERNATE_CONNECTION_DRIVER_CLASS="hibernate.connection.driver_class";</v>
+        SUBSTITUTE('Property-Definition'!D60,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D60
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String AGENT_CLASSNAME = "agent[X].classname";</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" t="str">
-        <f>'Property-Definition'!A20</f>
-        <v>DB.CONN.GENERAL</v>
+        <f>'Property-Definition'!A61</f>
+        <v>PROJECTS</v>
       </c>
       <c r="B62" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D20,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D20
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String HIBERNATE_CONNECTION_URL="hibernate.connection.url";</v>
+        SUBSTITUTE('Property-Definition'!D61,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D61
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String PROJECT = "project[X]";</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" t="str">
-        <f>'Property-Definition'!A21</f>
-        <v>DB.CONN.GENERAL</v>
+        <f>'Property-Definition'!A62</f>
+        <v>PROJECT.SETUPS[X]</v>
       </c>
       <c r="B63" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D21,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D21
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String HIBERNATE_DEFAULT_CATALOG="hibernate.default_catalog";</v>
+        SUBSTITUTE('Property-Definition'!D62,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D62
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String PROJECT_SETUP = "project[X].setup[X]";</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A64" t="str">
-        <f>'Property-Definition'!A22</f>
-        <v>DB.CONN.GENERAL</v>
+        <f>'Property-Definition'!A63</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B64" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D22,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D22
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String HIBERNATE_CONNECTION_USERNAME="hibernate.connection.username";</v>
+        SUBSTITUTE('Property-Definition'!D63,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D63
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_CONTACTAGENT = "bgplatform[X].contactagent";</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" t="str">
-        <f>'Property-Definition'!A23</f>
-        <v>DB.CONN.GENERAL</v>
+        <f>'Property-Definition'!A60</f>
+        <v>AWB.AGENTS</v>
       </c>
       <c r="B65" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D23,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D23
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String HIBERNATE_CONNECTION_PASSWORD="hibernate.connection.password";</v>
+        SUBSTITUTE('Property-Definition'!D64,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D64
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_PLATFORMNAME = "bgplatform[X].platformname";</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" t="str">
-        <f>'Property-Definition'!A24</f>
-        <v>DB.CONN.FACTORY.GET</v>
+        <f>'Property-Definition'!A61</f>
+        <v>PROJECTS</v>
       </c>
       <c r="B66" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D24,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D24
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String FACTORY_FACTORYID="factory[X].factoryID";</v>
+        SUBSTITUTE('Property-Definition'!D65,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D65
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_SERVER = "bgplatform[X].server";</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" t="str">
-        <f>'Property-Definition'!A25</f>
-        <v>DB.CONN.FACTORY.GET</v>
+        <f>'Property-Definition'!A62</f>
+        <v>PROJECT.SETUPS[X]</v>
       </c>
       <c r="B67" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D25,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D25
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String FACTORY_DBSYSTEM="factory[X].dbSystem";</v>
+        SUBSTITUTE('Property-Definition'!D66,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D66
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_IPADDRESS = "bgplatform[X].ipaddress";</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" t="str">
-        <f>'Property-Definition'!A26</f>
-        <v>DB.CONN.FACTORY.GET</v>
+        <f>'Property-Definition'!A67</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B68" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D26,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D26
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String FACTORY_HIBERNATE_CONNECTION_DRIVER_CLASS="factory[X].hibernate.connection.driver_class";</v>
+        SUBSTITUTE('Property-Definition'!D67,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D67
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_URL = "bgplatform[X].url";</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69" t="str">
-        <f>'Property-Definition'!A27</f>
-        <v>DB.CONN.FACTORY.GET</v>
+        <f>'Property-Definition'!A68</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B69" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D27,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D27
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String FACTORY_HIBERNATE_CONNECTION_URL="factory[X].hibernate.connection.url";</v>
+        SUBSTITUTE('Property-Definition'!D68,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D68
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_JADEPORT = "bgplatform[X].jadeport";</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" t="str">
-        <f>'Property-Definition'!A28</f>
-        <v>DB.CONN.FACTORY.GET</v>
+        <f>'Property-Definition'!A69</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B70" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D28,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D28
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String FACTORY_HIBERNATE_DEFAULT_CATALOG="factory[X].hibernate.default_catalog";</v>
+        SUBSTITUTE('Property-Definition'!D69,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D69
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_HTTPMTP = "bgplatform[X].httpmtp";</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71" t="str">
-        <f>'Property-Definition'!A29</f>
-        <v>DB.CONN.FACTORY.GET</v>
+        <f>'Property-Definition'!A70</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B71" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D29,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D29
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String FACTORY_HIBERNATE_CONNECTION_USERNAME="factory[X].hibernate.connection.username";</v>
+        SUBSTITUTE('Property-Definition'!D70,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D70
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_VERSIONMAJOR = "bgplatform[X].versionmajor";</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72" t="str">
-        <f>'Property-Definition'!A30</f>
-        <v>DB.CONN.FACTORY.GET</v>
+        <f>'Property-Definition'!A71</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B72" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D30,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D30
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String FACTORY_HIBERNATE_CONNECTION_PASSWORD="factory[X].hibernate.connection.password";</v>
+        SUBSTITUTE('Property-Definition'!D71,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D71
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_VERSIONMINOR = "bgplatform[X].versionminor";</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A73" t="str">
-        <f>'Property-Definition'!A31</f>
-        <v>DB.CONN.FACTORY.SET</v>
+        <f>'Property-Definition'!A72</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B73" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D31,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D31
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String FACTORYID="factoryID";</v>
+        SUBSTITUTE('Property-Definition'!D72,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D72
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_VERSIONMICRO = "bgplatform[X].versionmicro";</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A74" t="str">
-        <f>'Property-Definition'!A32</f>
-        <v>DB.CONN.FACTORY.SET</v>
+        <f>'Property-Definition'!A73</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B74" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D32,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D32
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String DBSYSTEM="dbSystem";</v>
+        SUBSTITUTE('Property-Definition'!D73,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D73
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_VERSIONBUILD = "bgplatform[X].versionbuild";</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A75" t="str">
-        <f>'Property-Definition'!A33</f>
-        <v>DB.CONN.FACTORY.SET</v>
+        <f>'Property-Definition'!A74</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B75" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D33,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D33
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String HIBERNATE_CONNECTION_DRIVER_CLASS="hibernate.connection.driver_class";</v>
+        SUBSTITUTE('Property-Definition'!D74,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D74
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_OS_NAME = "bgplatform[X].os.name";</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A76" t="str">
-        <f>'Property-Definition'!A34</f>
-        <v>DB.CONN.FACTORY.SET</v>
+        <f>'Property-Definition'!A75</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B76" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D34,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D34
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String HIBERNATE_CONNECTION_URL="hibernate.connection.url";</v>
+        SUBSTITUTE('Property-Definition'!D75,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D75
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_OS_VERSION = "bgplatform[X].os.version";</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A77" t="str">
-        <f>'Property-Definition'!A35</f>
-        <v>DB.CONN.FACTORY.SET</v>
+        <f>'Property-Definition'!A76</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B77" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D35,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D35
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String HIBERNATE_DEFAULT_CATALOG="hibernate.default_catalog";</v>
+        SUBSTITUTE('Property-Definition'!D76,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D76
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_OS_ARCHITECTURE = "bgplatform[X].os.architecture";</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A78" t="str">
-        <f>'Property-Definition'!A36</f>
-        <v>DB.CONN.FACTORY.SET</v>
+        <f>'Property-Definition'!A77</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B78" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D36,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D36
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String HIBERNATE_CONNECTION_USERNAME="hibernate.connection.username";</v>
+        SUBSTITUTE('Property-Definition'!D77,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D77
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_CPU_NAME = "bgplatform[X].cpu.name";</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A79" t="str">
-        <f>'Property-Definition'!A37</f>
-        <v>DB.CONN.FACTORY.SET</v>
+        <f>'Property-Definition'!A78</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B79" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D37,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D37
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String HIBERNATE_CONNECTION_PASSWORD="hibernate.connection.password";</v>
+        SUBSTITUTE('Property-Definition'!D78,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D78
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_CPU_NUMLOGICAL = "bgplatform[X].cpu.numlogical";</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A80" t="str">
-        <f>'Property-Definition'!A38</f>
-        <v>DB.CONN.TEST</v>
+        <f>'Property-Definition'!A79</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B80" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D38,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D38
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String DBSYSTEM="dbSystem";</v>
+        SUBSTITUTE('Property-Definition'!D79,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D79
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_CPU_NUMPHYSICAL = "bgplatform[X].cpu.numphysical";</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A81" t="str">
-        <f>'Property-Definition'!A39</f>
-        <v>DB.CONN.TEST</v>
+        <f>'Property-Definition'!A80</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B81" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D39,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D39
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String HIBERNATE_CONNECTION_DRIVER_CLASS="hibernate.connection.driver_class";</v>
+        SUBSTITUTE('Property-Definition'!D80,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D80
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_CPU_SPEEDMHZ = "bgplatform[X].cpu.speedmhz";</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A82" t="str">
-        <f>'Property-Definition'!A40</f>
-        <v>DB.CONN.TEST</v>
+        <f>'Property-Definition'!A81</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B82" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D40,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D40
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String HIBERNATE_CONNECTION_URL="hibernate.connection.url";</v>
+        SUBSTITUTE('Property-Definition'!D81,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D81
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_MEMORYMB = "bgplatform[X].memorymb";</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A83" t="str">
-        <f>'Property-Definition'!A41</f>
-        <v>DB.CONN.TEST</v>
+        <f>'Property-Definition'!A82</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B83" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D41,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D41
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String HIBERNATE_DEFAULT_CATALOG="hibernate.default_catalog";</v>
+        SUBSTITUTE('Property-Definition'!D82,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D82
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_BENCHMARKVALUE = "bgplatform[X].benchmarkvalue";</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A84" t="str">
-        <f>'Property-Definition'!A42</f>
-        <v>DB.CONN.TEST</v>
+        <f>'Property-Definition'!A83</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B84" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D42,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D42
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String HIBERNATE_CONNECTION_USERNAME="hibernate.connection.username";</v>
+        SUBSTITUTE('Property-Definition'!D83,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D83
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_TIME_ONLINESINCE = "bgplatform[X].time.onlinesince";</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A85" t="str">
-        <f>'Property-Definition'!A43</f>
-        <v>DB.CONN.TEST</v>
+        <f>'Property-Definition'!A84</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B85" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D43,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D43
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String HIBERNATE_CONNECTION_PASSWORD="hibernate.connection.password";</v>
+        SUBSTITUTE('Property-Definition'!D84,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D84
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_TIME_LASTCONTACT = "bgplatform[X].time.lastcontact";</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A86" t="str">
-        <f>'Property-Definition'!A44</f>
-        <v>EXEC.MODE</v>
+        <f>'Property-Definition'!A85</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B86" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D44,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D44
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String EXEC_MODE="exec.mode";</v>
+        SUBSTITUTE('Property-Definition'!D85,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D85
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_LOCALTIME_ONLINESINCE = "bgplatform[X].localtime.onlinesince";</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A87" t="str">
-        <f>'Property-Definition'!A45</f>
-        <v>EXEC.MODE</v>
+        <f>'Property-Definition'!A86</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B87" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D45,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D45
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String SERVER_MASTER_URL="server.master.url";</v>
+        SUBSTITUTE('Property-Definition'!D86,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D86
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_LOCALTIME_LASTCONTACT = "bgplatform[X].localtime.lastcontact";</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A88" t="str">
-        <f>'Property-Definition'!A46</f>
-        <v>EXEC.MODE</v>
+        <f>'Property-Definition'!A87</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B88" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D46,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D46
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String SERVER_MASTER_PORT="server.master.port";</v>
+        SUBSTITUTE('Property-Definition'!D87,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D87
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_CURRENTLYAVAILABLE = "bgplatform[X].currentlyavailable";</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A89" t="str">
-        <f>'Property-Definition'!A47</f>
-        <v>EXEC.MODE</v>
+        <f>'Property-Definition'!A88</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B89" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D47,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D47
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String SERVER_MASTER_PORT_MTP="server.master.port.mtp";</v>
+        SUBSTITUTE('Property-Definition'!D88,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D88
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_CURRENT_CPULOAD = "bgplatform[X].current.cpuload";</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A90" t="str">
-        <f>'Property-Definition'!A48</f>
-        <v>EXEC.MODE</v>
+        <f>'Property-Definition'!A89</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B90" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D48,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D48
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String SERVER_MASTER_PROTOCOL="server.master.protocol";</v>
+        SUBSTITUTE('Property-Definition'!D89,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D89
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_CURRENT_MEMORYLOAD = "bgplatform[X].current.memoryload";</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A91" t="str">
-        <f>'Property-Definition'!A49</f>
-        <v>EXEC.MODE</v>
+        <f>'Property-Definition'!A90</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B91" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D49,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D49
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String LOCAL_MTP_CREATION="local.mtp.creation";</v>
+        SUBSTITUTE('Property-Definition'!D90,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D90
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_CURRENT_MEMORYLOADJVM = "bgplatform[X].current.memoryloadjvm";</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A92" t="str">
-        <f>'Property-Definition'!A50</f>
-        <v>EXEC.MODE</v>
+        <f>'Property-Definition'!A91</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
       <c r="B92" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D50,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D50
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String LOCAL_MTP_URL="local.mtp.url";</v>
+        SUBSTITUTE('Property-Definition'!D91,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D91
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String BGPLATFORM_CURRENT_NUMTHREADS = "bgplatform[X].current.numthreads";</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A93" t="str">
-        <f>'Property-Definition'!A51</f>
-        <v>EXEC.MODE</v>
-      </c>
-      <c r="B93" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D51,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D51
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String LOCAL_MTP_PORT="local.mtp.port";</v>
-      </c>
-    </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A94" t="str">
-        <f>'Property-Definition'!A52</f>
-        <v>EXEC.MODE</v>
-      </c>
-      <c r="B94" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D52,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D52
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String LOCAL_MTP_PROTOCOL="local.mtp.protocol";</v>
-      </c>
-    </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A95" t="str">
-        <f>'Property-Definition'!A53</f>
-        <v>EXEC.MODE</v>
-      </c>
-      <c r="B95" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D53,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D53
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String EMBEDDEDSYSTEM_PROJECT="embeddedsystem.project";</v>
-      </c>
-    </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A96" t="str">
-        <f>'Property-Definition'!A54</f>
-        <v>EXEC.MODE</v>
-      </c>
-      <c r="B96" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D54,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D54
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String DEVICE_SYSTEM_EXEC_MODE="device_system_exec_mode";</v>
-      </c>
-    </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A97" t="str">
-        <f>'Property-Definition'!A55</f>
-        <v>EXEC.MODE</v>
-      </c>
-      <c r="B97" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D55,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D55
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String EMBEDDEDSYSTEM_AGENT_CLASSNAME="embeddedsystem.agent[X].classname";</v>
-      </c>
-    </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A98" t="str">
-        <f>'Property-Definition'!A56</f>
-        <v>EXEC.MODE</v>
-      </c>
-      <c r="B98" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D56,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D56
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String EMBEDDEDSYSTEM_AGENT_AGENTNAME="embeddedsystem.agent[X].agentname";</v>
-      </c>
-    </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A99" t="str">
-        <f>'Property-Definition'!A57</f>
-        <v>EXEC.MODE</v>
-      </c>
-      <c r="B99" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D57,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D57
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String SERVICE_SERVICE_SETUP="service.service_setup";</v>
-      </c>
-    </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A100" t="str">
-        <f>'Property-Definition'!A58</f>
-        <v>EXEC.MODE</v>
-      </c>
-      <c r="B100" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D58,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D58
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String LOCAL_IP_SELECTION="local.ip.selection[X]";</v>
-      </c>
-    </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A101" t="str">
-        <f>'Property-Definition'!A59</f>
-        <v>EXEC.MODE</v>
-      </c>
-      <c r="B101" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D59,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D59
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String FACTORY_ID="factory_id";</v>
-      </c>
-    </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A102" t="str">
-        <f>'Property-Definition'!A60</f>
-        <v>EXEC.MODE</v>
-      </c>
-      <c r="B102" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D60,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D60
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGSYSTEM_AUTO_INIT="bgsystem.auto_init";</v>
-      </c>
-    </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A103" t="str">
-        <f>'Property-Definition'!A61</f>
-        <v>AWB.AGENTS</v>
-      </c>
-      <c r="B103" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D61,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D61
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String AGENT_CLASSNAME="agent[X].classname";</v>
-      </c>
-    </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A104" t="str">
-        <f>'Property-Definition'!A62</f>
-        <v>PROJECTS</v>
-      </c>
-      <c r="B104" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D62,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D62
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String PROJECT="project[X]";</v>
-      </c>
-    </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A105" t="str">
-        <f>'Property-Definition'!A63</f>
-        <v>PROJECT.SETUPS[X]</v>
-      </c>
-      <c r="B105" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D63,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D63
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String PROJECT_SETUP="project[X].setup[X]";</v>
-      </c>
-    </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A106" t="str">
-        <f>'Property-Definition'!A64</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B106" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D64,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D64
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_CONTACTAGENT="bgplatform[X].contactagent";</v>
-      </c>
-    </row>
-    <row r="107" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A107" t="str">
-        <f>'Property-Definition'!A61</f>
-        <v>AWB.AGENTS</v>
-      </c>
-      <c r="B107" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D61,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D61 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String AGENT[X]_CLASSNAME = "agent[X].classname";</v>
-      </c>
-    </row>
-    <row r="108" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A108" t="str">
-        <f>'Property-Definition'!A62</f>
-        <v>PROJECTS</v>
-      </c>
-      <c r="B108" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D62,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D62 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String PROJECT[X] = "project[X]";</v>
-      </c>
-    </row>
-    <row r="109" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A109" t="str">
-        <f>'Property-Definition'!A63</f>
-        <v>PROJECT.SETUPS[X]</v>
-      </c>
-      <c r="B109" t="str">
-        <f>"public final static String "&amp; UPPER(SUBSTITUTE('Property-Definition'!D63,".","_"))&amp;" = "&amp; CHAR(34) &amp; 'Property-Definition'!D63 &amp; CHAR(34)&amp; ";"</f>
-        <v>public final static String PROJECT[X]_SETUP[X] = "project[X].setup[X]";</v>
-      </c>
-    </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A110" t="str">
-        <f>'Property-Definition'!A68</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B110" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D68,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D68
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_URL="bgplatform[X].url";</v>
-      </c>
-    </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A111" t="str">
-        <f>'Property-Definition'!A69</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B111" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D69,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D69
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_JADEPORT="bgplatform[X].jadeport";</v>
-      </c>
-    </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A112" t="str">
-        <f>'Property-Definition'!A70</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B112" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D70,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D70
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_HTTPMTP="bgplatform[X].httpmtp";</v>
-      </c>
-    </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A113" t="str">
-        <f>'Property-Definition'!A71</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B113" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D71,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D71
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_VERSIONMAJOR="bgplatform[X].versionmajor";</v>
-      </c>
-    </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A114" t="str">
-        <f>'Property-Definition'!A72</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B114" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D72,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D72
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_VERSIONMINOR="bgplatform[X].versionminor";</v>
-      </c>
-    </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A115" t="str">
-        <f>'Property-Definition'!A73</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B115" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D73,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D73
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_VERSIONMICRO="bgplatform[X].versionmicro";</v>
-      </c>
-    </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A116" t="str">
-        <f>'Property-Definition'!A74</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B116" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D74,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D74
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_VERSIONBUILD="bgplatform[X].versionbuild";</v>
-      </c>
-    </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A117" t="str">
-        <f>'Property-Definition'!A75</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B117" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D75,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D75
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_OS_NAME="bgplatform[X].os.name";</v>
-      </c>
-    </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A118" t="str">
-        <f>'Property-Definition'!A76</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B118" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D76,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D76
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_OS_VERSION="bgplatform[X].os.version";</v>
-      </c>
-    </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A119" t="str">
-        <f>'Property-Definition'!A77</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B119" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D77,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D77
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_OS_ARCHITECTURE="bgplatform[X].os.architecture";</v>
-      </c>
-    </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A120" t="str">
-        <f>'Property-Definition'!A78</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B120" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D78,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D78
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_CPU_NAME="bgplatform[X].cpu.name";</v>
-      </c>
-    </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A121" t="str">
-        <f>'Property-Definition'!A79</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B121" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D79,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D79
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_CPU_NUMLOGICAL="bgplatform[X].cpu.numlogical";</v>
-      </c>
-    </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A122" t="str">
-        <f>'Property-Definition'!A80</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B122" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D80,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D80
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_CPU_NUMPHYSICAL="bgplatform[X].cpu.numphysical";</v>
-      </c>
-    </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A123" t="str">
-        <f>'Property-Definition'!A81</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B123" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D81,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D81
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_CPU_SPEEDMHZ="bgplatform[X].cpu.speedmhz";</v>
-      </c>
-    </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A124" t="str">
-        <f>'Property-Definition'!A82</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B124" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D82,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D82
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_MEMORYMB="bgplatform[X].memorymb";</v>
-      </c>
-    </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A125" t="str">
-        <f>'Property-Definition'!A83</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B125" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D83,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D83
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_BENCHMARKVALUE="bgplatform[X].benchmarkvalue";</v>
-      </c>
-    </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A126" t="str">
-        <f>'Property-Definition'!A84</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B126" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D84,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D84
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_TIME_ONLINESINCE="bgplatform[X].time.onlinesince";</v>
-      </c>
-    </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A127" t="str">
-        <f>'Property-Definition'!A85</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B127" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D85,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D85
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_TIME_LASTCONTACT="bgplatform[X].time.lastcontact";</v>
-      </c>
-    </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A128" t="str">
-        <f>'Property-Definition'!A86</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B128" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D86,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D86
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_LOCALTIME_ONLINESINCE="bgplatform[X].localtime.onlinesince";</v>
-      </c>
-    </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A129" t="str">
-        <f>'Property-Definition'!A87</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B129" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D87,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D87
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_LOCALTIME_LASTCONTACT="bgplatform[X].localtime.lastcontact";</v>
-      </c>
-    </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A130" t="str">
-        <f>'Property-Definition'!A88</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B130" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D88,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D88
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_CURRENTLYAVAILABLE="bgplatform[X].currentlyavailable";</v>
-      </c>
-    </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A131" t="str">
-        <f>'Property-Definition'!A89</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B131" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D89,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D89
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_CURRENT_CPULOAD="bgplatform[X].current.cpuload";</v>
-      </c>
-    </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A132" t="str">
-        <f>'Property-Definition'!A90</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B132" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D90,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D90
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_CURRENT_MEMORYLOAD="bgplatform[X].current.memoryload";</v>
-      </c>
-    </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A133" t="str">
-        <f>'Property-Definition'!A91</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B133" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D91,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D91
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_CURRENT_MEMORYLOADJVM="bgplatform[X].current.memoryloadjvm";</v>
-      </c>
-    </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A134" t="str">
         <f>'Property-Definition'!A92</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
       </c>
-      <c r="B134" t="str">
+      <c r="B93" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
         SUBSTITUTE('Property-Definition'!D92,"[X]",""),".","_")
 )
-&amp; "="
+&amp; " = "
 &amp; CHAR(34)
 &amp; 'Property-Definition'!D92
 &amp; CHAR(34)
 &amp; ";"</f>
-        <v>public final static String BGPLATFORM_CURRENT_NUMTHREADS="bgplatform[X].current.numthreads";</v>
-      </c>
-    </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A135" t="str">
-        <f>'Property-Definition'!A93</f>
-        <v>EXEC.MASTER.SLAVES.GET</v>
-      </c>
-      <c r="B135" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D93,"[X]",""),".","_")
-)
-&amp; "="
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D93
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String BGPLATFORM_CURRENT_THRESHOLDEXCEEDED="bgplatform[X].current.thresholdexceeded";</v>
+        <v>public final static String BGPLATFORM_CURRENT_THRESHOLDEXCEEDED = "bgplatform[X].current.thresholdexceeded";</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B109" xr:uid="{F30A1E73-A707-4178-9C72-9AC27F9EE5F7}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="EXEC.MODE"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:B93" xr:uid="{F30A1E73-A707-4178-9C72-9AC27F9EE5F7}"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101004FB79D76D905EB41B4AD64ED4839597F" ma:contentTypeVersion="11" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="0622d98e252eab518d4b54f931ba6851">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="897f6830-f425-409d-b8f5-ce1019056d9e" xmlns:ns3="f2404b4d-361b-46d3-b2ec-035eed29e274" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dd5f302b3846fd12003b89c8f5b7df36" ns2:_="" ns3:_="">
     <xsd:import namespace="897f6830-f425-409d-b8f5-ce1019056d9e"/>
@@ -5695,15 +5281,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -5716,6 +5293,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A33EE264-283E-4F19-BA61-B3264EA417E2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5734,14 +5319,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF16440F-B0E0-4269-97EE-BEB05B0223C8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Added type-script table to workbook
</commit_message>
<xml_diff>
--- a/AWB-RestApi-PropertyDictionary.xlsx
+++ b/AWB-RestApi-PropertyDictionary.xlsx
@@ -5,19 +5,21 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\AgentWorkbench\eclipseProjects\de.enflexit.awb\bundles\web\xApi\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\20_GIT\01_AWB\eclipseProjects\de.enflexit.awb\bundles\web\xAPI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27507518-1AE7-4149-A7A0-648A1B12E337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D23A1BEB-51E5-48C5-A0CC-9A78FFFA8572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Property-Definition" sheetId="1" r:id="rId1"/>
     <sheet name="Java-Code" sheetId="2" r:id="rId2"/>
+    <sheet name="Type-Script-Code" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Java-Code'!$A$1:$B$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Type-Script-Code'!$A$1:$B$93</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="194">
   <si>
     <t>key</t>
   </si>
@@ -1002,20 +1004,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K92"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="28.7265625" customWidth="1"/>
-    <col min="3" max="3" width="14.26953125" customWidth="1"/>
-    <col min="4" max="4" width="54.1796875" customWidth="1"/>
-    <col min="5" max="5" width="17.1796875" customWidth="1"/>
+    <col min="1" max="2" width="28.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" customWidth="1"/>
+    <col min="4" max="4" width="54.140625" customWidth="1"/>
+    <col min="5" max="5" width="17.140625" customWidth="1"/>
     <col min="6" max="6" width="79" customWidth="1"/>
-    <col min="7" max="7" width="18.1796875" customWidth="1"/>
-    <col min="8" max="8" width="34.81640625" customWidth="1"/>
-    <col min="9" max="10" width="17.7265625" style="5" customWidth="1"/>
-    <col min="11" max="11" width="113.7265625" customWidth="1"/>
+    <col min="7" max="7" width="18.140625" customWidth="1"/>
+    <col min="8" max="8" width="34.85546875" customWidth="1"/>
+    <col min="9" max="10" width="17.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="113.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -1050,7 +1052,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1079,7 +1081,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>43</v>
       </c>
@@ -1105,7 +1107,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>43</v>
       </c>
@@ -1131,7 +1133,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -1157,7 +1159,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -1183,7 +1185,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>43</v>
       </c>
@@ -1209,7 +1211,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -1235,7 +1237,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>43</v>
       </c>
@@ -1261,7 +1263,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -1290,7 +1292,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -1322,7 +1324,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -1351,7 +1353,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -1380,7 +1382,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -1410,7 +1412,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -1439,7 +1441,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -1468,7 +1470,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>41</v>
       </c>
@@ -1497,7 +1499,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>41</v>
       </c>
@@ -1526,7 +1528,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>41</v>
       </c>
@@ -1552,7 +1554,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>41</v>
       </c>
@@ -1578,7 +1580,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>41</v>
       </c>
@@ -1604,7 +1606,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>41</v>
       </c>
@@ -1630,7 +1632,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>41</v>
       </c>
@@ -1656,7 +1658,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>64</v>
       </c>
@@ -1685,7 +1687,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>64</v>
       </c>
@@ -1714,7 +1716,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>64</v>
       </c>
@@ -1740,7 +1742,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>64</v>
       </c>
@@ -1766,7 +1768,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>64</v>
       </c>
@@ -1792,7 +1794,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>64</v>
       </c>
@@ -1818,7 +1820,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>64</v>
       </c>
@@ -1844,7 +1846,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>65</v>
       </c>
@@ -1870,7 +1872,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>65</v>
       </c>
@@ -1896,7 +1898,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>65</v>
       </c>
@@ -1922,7 +1924,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>65</v>
       </c>
@@ -1948,7 +1950,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>65</v>
       </c>
@@ -1974,7 +1976,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>65</v>
       </c>
@@ -2000,7 +2002,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>65</v>
       </c>
@@ -2026,7 +2028,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>73</v>
       </c>
@@ -2052,7 +2054,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>73</v>
       </c>
@@ -2078,7 +2080,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>73</v>
       </c>
@@ -2104,7 +2106,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>73</v>
       </c>
@@ -2130,7 +2132,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>73</v>
       </c>
@@ -2156,7 +2158,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>73</v>
       </c>
@@ -2182,7 +2184,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>82</v>
       </c>
@@ -2211,7 +2213,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>82</v>
       </c>
@@ -2237,7 +2239,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>82</v>
       </c>
@@ -2263,7 +2265,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>82</v>
       </c>
@@ -2289,7 +2291,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>82</v>
       </c>
@@ -2318,7 +2320,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>82</v>
       </c>
@@ -2347,7 +2349,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>82</v>
       </c>
@@ -2373,7 +2375,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>82</v>
       </c>
@@ -2399,7 +2401,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>82</v>
       </c>
@@ -2428,7 +2430,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>82</v>
       </c>
@@ -2454,7 +2456,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>82</v>
       </c>
@@ -2483,7 +2485,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>82</v>
       </c>
@@ -2509,7 +2511,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>82</v>
       </c>
@@ -2535,7 +2537,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>82</v>
       </c>
@@ -2561,7 +2563,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>82</v>
       </c>
@@ -2587,7 +2589,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>82</v>
       </c>
@@ -2613,7 +2615,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>91</v>
       </c>
@@ -2639,7 +2641,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>94</v>
       </c>
@@ -2662,7 +2664,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>95</v>
       </c>
@@ -2688,7 +2690,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>83</v>
       </c>
@@ -2708,7 +2710,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>83</v>
       </c>
@@ -2728,7 +2730,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>83</v>
       </c>
@@ -2748,7 +2750,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>83</v>
       </c>
@@ -2768,7 +2770,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>83</v>
       </c>
@@ -2788,7 +2790,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>83</v>
       </c>
@@ -2808,7 +2810,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>83</v>
       </c>
@@ -2828,7 +2830,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>83</v>
       </c>
@@ -2848,7 +2850,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>83</v>
       </c>
@@ -2868,7 +2870,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>83</v>
       </c>
@@ -2888,7 +2890,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>83</v>
       </c>
@@ -2908,7 +2910,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>83</v>
       </c>
@@ -2928,7 +2930,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>83</v>
       </c>
@@ -2948,7 +2950,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>83</v>
       </c>
@@ -2968,7 +2970,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>83</v>
       </c>
@@ -2988,7 +2990,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>83</v>
       </c>
@@ -3008,7 +3010,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>83</v>
       </c>
@@ -3028,7 +3030,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>83</v>
       </c>
@@ -3048,7 +3050,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>83</v>
       </c>
@@ -3068,7 +3070,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>83</v>
       </c>
@@ -3088,7 +3090,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>83</v>
       </c>
@@ -3108,7 +3110,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>83</v>
       </c>
@@ -3128,7 +3130,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>83</v>
       </c>
@@ -3148,7 +3150,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>83</v>
       </c>
@@ -3168,7 +3170,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>83</v>
       </c>
@@ -3188,7 +3190,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>83</v>
       </c>
@@ -3208,7 +3210,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>83</v>
       </c>
@@ -3228,7 +3230,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>83</v>
       </c>
@@ -3248,7 +3250,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>83</v>
       </c>
@@ -3268,7 +3270,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>83</v>
       </c>
@@ -3308,13 +3310,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F30A1E73-A707-4178-9C72-9AC27F9EE5F7}">
   <dimension ref="A1:B93"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7265625" customWidth="1"/>
+    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="str">
         <f>'Property-Definition'!A1</f>
         <v>performative</v>
@@ -3323,7 +3325,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="str">
         <f>'Property-Definition'!A2</f>
         <v>DB.SYSTEMS</v>
@@ -3342,7 +3344,7 @@
         <v>public final static String DBSYSTEM = "dbSystem[X]";</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
         <f>'Property-Definition'!A3</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3361,7 +3363,7 @@
         <v>public final static String DBSYSTEM = "dbSystem[X]";</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
         <f>'Property-Definition'!A4</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3380,7 +3382,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_DRIVER_CLASS = "dbSystem[X].hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
         <f>'Property-Definition'!A5</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3399,7 +3401,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_URL = "dbSystem[X].hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
         <f>'Property-Definition'!A6</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3418,7 +3420,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_URL_MASK = "dbSystem[X].hibernate.connection.url.mask";</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
         <f>'Property-Definition'!A7</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3437,7 +3439,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_DEFAULT_CATALOG = "dbSystem[X].hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
         <f>'Property-Definition'!A8</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3456,7 +3458,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_USERNAME = "dbSystem[X].hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
         <f>'Property-Definition'!A9</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3475,7 +3477,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_PASSWORD = "dbSystem[X].hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="str">
         <f>'Property-Definition'!A10</f>
         <v>DB.FACTORIES</v>
@@ -3494,7 +3496,7 @@
         <v>public final static String FACTORY = "factory[X]";</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="str">
         <f>'Property-Definition'!A11</f>
         <v>DB.FACTORIES</v>
@@ -3513,7 +3515,7 @@
         <v>public final static String FACTORY_STATE = "factory[X].state";</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
         <f>'Property-Definition'!A12</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -3532,7 +3534,7 @@
         <v>public final static String ISSTARTDERBYNETWORKSERVER = "isStartDerbyNetworkServer";</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
         <f>'Property-Definition'!A13</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -3551,7 +3553,7 @@
         <v>public final static String HOST-IP = "host-IP";</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="str">
         <f>'Property-Definition'!A14</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -3570,7 +3572,7 @@
         <v>public final static String PORT = "port";</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="str">
         <f>'Property-Definition'!A15</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -3589,7 +3591,7 @@
         <v>public final static String USERNAME = "userName";</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="str">
         <f>'Property-Definition'!A16</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -3608,7 +3610,7 @@
         <v>public final static String PASSWORD = "password";</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="str">
         <f>'Property-Definition'!A17</f>
         <v>DB.CONN.GENERAL</v>
@@ -3627,7 +3629,7 @@
         <v>public final static String USEFOREVERYFACTORY = "useForEveryFactory";</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="str">
         <f>'Property-Definition'!A18</f>
         <v>DB.CONN.GENERAL</v>
@@ -3646,7 +3648,7 @@
         <v>public final static String DBSYSTEM = "dbSystem";</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="str">
         <f>'Property-Definition'!A19</f>
         <v>DB.CONN.GENERAL</v>
@@ -3665,7 +3667,7 @@
         <v>public final static String HIBERNATE_CONNECTION_DRIVER_CLASS = "hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="str">
         <f>'Property-Definition'!A20</f>
         <v>DB.CONN.GENERAL</v>
@@ -3684,7 +3686,7 @@
         <v>public final static String HIBERNATE_CONNECTION_URL = "hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="str">
         <f>'Property-Definition'!A21</f>
         <v>DB.CONN.GENERAL</v>
@@ -3703,7 +3705,7 @@
         <v>public final static String HIBERNATE_DEFAULT_CATALOG = "hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="str">
         <f>'Property-Definition'!A22</f>
         <v>DB.CONN.GENERAL</v>
@@ -3722,7 +3724,7 @@
         <v>public final static String HIBERNATE_CONNECTION_USERNAME = "hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
         <f>'Property-Definition'!A23</f>
         <v>DB.CONN.GENERAL</v>
@@ -3741,7 +3743,7 @@
         <v>public final static String HIBERNATE_CONNECTION_PASSWORD = "hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="str">
         <f>'Property-Definition'!A24</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -3760,7 +3762,7 @@
         <v>public final static String FACTORY_FACTORYID = "factory[X].factoryID";</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="str">
         <f>'Property-Definition'!A25</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -3779,7 +3781,7 @@
         <v>public final static String FACTORY_DBSYSTEM = "factory[X].dbSystem";</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="str">
         <f>'Property-Definition'!A26</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -3798,7 +3800,7 @@
         <v>public final static String FACTORY_HIBERNATE_CONNECTION_DRIVER_CLASS = "factory[X].hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="str">
         <f>'Property-Definition'!A27</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -3817,7 +3819,7 @@
         <v>public final static String FACTORY_HIBERNATE_CONNECTION_URL = "factory[X].hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="str">
         <f>'Property-Definition'!A28</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -3836,7 +3838,7 @@
         <v>public final static String FACTORY_HIBERNATE_DEFAULT_CATALOG = "factory[X].hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="str">
         <f>'Property-Definition'!A29</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -3855,7 +3857,7 @@
         <v>public final static String FACTORY_HIBERNATE_CONNECTION_USERNAME = "factory[X].hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="str">
         <f>'Property-Definition'!A30</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -3874,7 +3876,7 @@
         <v>public final static String FACTORY_HIBERNATE_CONNECTION_PASSWORD = "factory[X].hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="str">
         <f>'Property-Definition'!A31</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -3893,7 +3895,7 @@
         <v>public final static String FACTORYID = "factoryID";</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="str">
         <f>'Property-Definition'!A32</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -3912,7 +3914,7 @@
         <v>public final static String DBSYSTEM = "dbSystem";</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="str">
         <f>'Property-Definition'!A33</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -3931,7 +3933,7 @@
         <v>public final static String HIBERNATE_CONNECTION_DRIVER_CLASS = "hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="str">
         <f>'Property-Definition'!A34</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -3950,7 +3952,7 @@
         <v>public final static String HIBERNATE_CONNECTION_URL = "hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="str">
         <f>'Property-Definition'!A35</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -3969,7 +3971,7 @@
         <v>public final static String HIBERNATE_DEFAULT_CATALOG = "hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="str">
         <f>'Property-Definition'!A36</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -3988,7 +3990,7 @@
         <v>public final static String HIBERNATE_CONNECTION_USERNAME = "hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="str">
         <f>'Property-Definition'!A37</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4007,7 +4009,7 @@
         <v>public final static String HIBERNATE_CONNECTION_PASSWORD = "hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="str">
         <f>'Property-Definition'!A38</f>
         <v>DB.CONN.TEST</v>
@@ -4026,7 +4028,7 @@
         <v>public final static String DBSYSTEM = "dbSystem";</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="str">
         <f>'Property-Definition'!A39</f>
         <v>DB.CONN.TEST</v>
@@ -4045,7 +4047,7 @@
         <v>public final static String HIBERNATE_CONNECTION_DRIVER_CLASS = "hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="str">
         <f>'Property-Definition'!A40</f>
         <v>DB.CONN.TEST</v>
@@ -4064,7 +4066,7 @@
         <v>public final static String HIBERNATE_CONNECTION_URL = "hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="str">
         <f>'Property-Definition'!A41</f>
         <v>DB.CONN.TEST</v>
@@ -4083,7 +4085,7 @@
         <v>public final static String HIBERNATE_DEFAULT_CATALOG = "hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="str">
         <f>'Property-Definition'!A42</f>
         <v>DB.CONN.TEST</v>
@@ -4102,7 +4104,7 @@
         <v>public final static String HIBERNATE_CONNECTION_USERNAME = "hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="str">
         <f>'Property-Definition'!A43</f>
         <v>DB.CONN.TEST</v>
@@ -4121,7 +4123,7 @@
         <v>public final static String HIBERNATE_CONNECTION_PASSWORD = "hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="str">
         <f>'Property-Definition'!A44</f>
         <v>EXEC.MODE</v>
@@ -4140,7 +4142,7 @@
         <v>public final static String EXEC_MODE = "exec.mode";</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="str">
         <f>'Property-Definition'!A45</f>
         <v>EXEC.MODE</v>
@@ -4159,7 +4161,7 @@
         <v>public final static String SERVER_MASTER_URL = "server.master.url";</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="str">
         <f>'Property-Definition'!A46</f>
         <v>EXEC.MODE</v>
@@ -4178,7 +4180,7 @@
         <v>public final static String SERVER_MASTER_PORT = "server.master.port";</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="str">
         <f>'Property-Definition'!A47</f>
         <v>EXEC.MODE</v>
@@ -4197,7 +4199,7 @@
         <v>public final static String SERVER_MASTER_PORT_MTP = "server.master.port.mtp";</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="str">
         <f>'Property-Definition'!A48</f>
         <v>EXEC.MODE</v>
@@ -4216,7 +4218,7 @@
         <v>public final static String SERVER_MASTER_PROTOCOL = "server.master.protocol";</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="str">
         <f>'Property-Definition'!A49</f>
         <v>EXEC.MODE</v>
@@ -4235,7 +4237,7 @@
         <v>public final static String LOCAL_MTP_CREATION = "local.mtp.creation";</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="str">
         <f>'Property-Definition'!A50</f>
         <v>EXEC.MODE</v>
@@ -4254,7 +4256,7 @@
         <v>public final static String LOCAL_MTP_URL = "local.mtp.url";</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="str">
         <f>'Property-Definition'!A51</f>
         <v>EXEC.MODE</v>
@@ -4273,7 +4275,7 @@
         <v>public final static String LOCAL_MTP_PORT = "local.mtp.port";</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="str">
         <f>'Property-Definition'!A52</f>
         <v>EXEC.MODE</v>
@@ -4292,7 +4294,7 @@
         <v>public final static String LOCAL_MTP_PROTOCOL = "local.mtp.protocol";</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="str">
         <f>'Property-Definition'!A53</f>
         <v>EXEC.MODE</v>
@@ -4311,7 +4313,7 @@
         <v>public final static String EMBEDDEDSYSTEM_PROJECT = "embeddedsystem.project";</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="str">
         <f>'Property-Definition'!A54</f>
         <v>EXEC.MODE</v>
@@ -4330,7 +4332,7 @@
         <v>public final static String DEVICE_SYSTEM_EXEC_MODE = "device_system_exec_mode";</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="str">
         <f>'Property-Definition'!A55</f>
         <v>EXEC.MODE</v>
@@ -4349,7 +4351,7 @@
         <v>public final static String EMBEDDEDSYSTEM_AGENT_CLASSNAME = "embeddedsystem.agent[X].classname";</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="str">
         <f>'Property-Definition'!A56</f>
         <v>EXEC.MODE</v>
@@ -4368,7 +4370,7 @@
         <v>public final static String EMBEDDEDSYSTEM_AGENT_AGENTNAME = "embeddedsystem.agent[X].agentname";</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="str">
         <f>'Property-Definition'!A57</f>
         <v>EXEC.MODE</v>
@@ -4387,7 +4389,7 @@
         <v>public final static String SERVICE_SERVICE_SETUP = "service.service_setup";</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="str">
         <f>'Property-Definition'!A58</f>
         <v>EXEC.MODE</v>
@@ -4406,7 +4408,7 @@
         <v>public final static String LOCAL_IP_SELECTION = "local.ip.selection[X]";</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="str">
         <f>'Property-Definition'!A59</f>
         <v>EXEC.MODE</v>
@@ -4425,7 +4427,7 @@
         <v>public final static String FACTORY_ID = "factory_id";</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="e">
         <f>'Property-Definition'!#REF!</f>
         <v>#REF!</v>
@@ -4444,7 +4446,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="str">
         <f>'Property-Definition'!A60</f>
         <v>AWB.AGENTS</v>
@@ -4463,7 +4465,7 @@
         <v>public final static String AGENT_CLASSNAME = "agent[X].classname";</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="str">
         <f>'Property-Definition'!A61</f>
         <v>PROJECTS</v>
@@ -4482,7 +4484,7 @@
         <v>public final static String PROJECT = "project[X]";</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="str">
         <f>'Property-Definition'!A62</f>
         <v>PROJECT.SETUPS[X]</v>
@@ -4501,7 +4503,7 @@
         <v>public final static String PROJECT_SETUP = "project[X].setup[X]";</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="str">
         <f>'Property-Definition'!A63</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4520,7 +4522,7 @@
         <v>public final static String BGPLATFORM_CONTACTAGENT = "bgplatform[X].contactagent";</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="str">
         <f>'Property-Definition'!A60</f>
         <v>AWB.AGENTS</v>
@@ -4539,7 +4541,7 @@
         <v>public final static String BGPLATFORM_PLATFORMNAME = "bgplatform[X].platformname";</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="str">
         <f>'Property-Definition'!A61</f>
         <v>PROJECTS</v>
@@ -4558,7 +4560,7 @@
         <v>public final static String BGPLATFORM_SERVER = "bgplatform[X].server";</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="str">
         <f>'Property-Definition'!A62</f>
         <v>PROJECT.SETUPS[X]</v>
@@ -4577,7 +4579,7 @@
         <v>public final static String BGPLATFORM_IPADDRESS = "bgplatform[X].ipaddress";</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="str">
         <f>'Property-Definition'!A67</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4596,7 +4598,7 @@
         <v>public final static String BGPLATFORM_URL = "bgplatform[X].url";</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="str">
         <f>'Property-Definition'!A68</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4615,7 +4617,7 @@
         <v>public final static String BGPLATFORM_JADEPORT = "bgplatform[X].jadeport";</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="str">
         <f>'Property-Definition'!A69</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4634,7 +4636,7 @@
         <v>public final static String BGPLATFORM_HTTPMTP = "bgplatform[X].httpmtp";</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="str">
         <f>'Property-Definition'!A70</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4653,7 +4655,7 @@
         <v>public final static String BGPLATFORM_VERSIONMAJOR = "bgplatform[X].versionmajor";</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="str">
         <f>'Property-Definition'!A71</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4672,7 +4674,7 @@
         <v>public final static String BGPLATFORM_VERSIONMINOR = "bgplatform[X].versionminor";</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="str">
         <f>'Property-Definition'!A72</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4691,7 +4693,7 @@
         <v>public final static String BGPLATFORM_VERSIONMICRO = "bgplatform[X].versionmicro";</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="str">
         <f>'Property-Definition'!A73</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4710,7 +4712,7 @@
         <v>public final static String BGPLATFORM_VERSIONBUILD = "bgplatform[X].versionbuild";</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="str">
         <f>'Property-Definition'!A74</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4729,7 +4731,7 @@
         <v>public final static String BGPLATFORM_OS_NAME = "bgplatform[X].os.name";</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="str">
         <f>'Property-Definition'!A75</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4748,7 +4750,7 @@
         <v>public final static String BGPLATFORM_OS_VERSION = "bgplatform[X].os.version";</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="str">
         <f>'Property-Definition'!A76</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4767,7 +4769,7 @@
         <v>public final static String BGPLATFORM_OS_ARCHITECTURE = "bgplatform[X].os.architecture";</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="str">
         <f>'Property-Definition'!A77</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4786,7 +4788,7 @@
         <v>public final static String BGPLATFORM_CPU_NAME = "bgplatform[X].cpu.name";</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="str">
         <f>'Property-Definition'!A78</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4805,7 +4807,7 @@
         <v>public final static String BGPLATFORM_CPU_NUMLOGICAL = "bgplatform[X].cpu.numlogical";</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="str">
         <f>'Property-Definition'!A79</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4824,7 +4826,7 @@
         <v>public final static String BGPLATFORM_CPU_NUMPHYSICAL = "bgplatform[X].cpu.numphysical";</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="str">
         <f>'Property-Definition'!A80</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4843,7 +4845,7 @@
         <v>public final static String BGPLATFORM_CPU_SPEEDMHZ = "bgplatform[X].cpu.speedmhz";</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="str">
         <f>'Property-Definition'!A81</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4862,7 +4864,7 @@
         <v>public final static String BGPLATFORM_MEMORYMB = "bgplatform[X].memorymb";</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="str">
         <f>'Property-Definition'!A82</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4881,7 +4883,7 @@
         <v>public final static String BGPLATFORM_BENCHMARKVALUE = "bgplatform[X].benchmarkvalue";</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="str">
         <f>'Property-Definition'!A83</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4900,7 +4902,7 @@
         <v>public final static String BGPLATFORM_TIME_ONLINESINCE = "bgplatform[X].time.onlinesince";</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="str">
         <f>'Property-Definition'!A84</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4919,7 +4921,7 @@
         <v>public final static String BGPLATFORM_TIME_LASTCONTACT = "bgplatform[X].time.lastcontact";</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="str">
         <f>'Property-Definition'!A85</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4938,7 +4940,7 @@
         <v>public final static String BGPLATFORM_LOCALTIME_ONLINESINCE = "bgplatform[X].localtime.onlinesince";</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="str">
         <f>'Property-Definition'!A86</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4957,7 +4959,7 @@
         <v>public final static String BGPLATFORM_LOCALTIME_LASTCONTACT = "bgplatform[X].localtime.lastcontact";</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="str">
         <f>'Property-Definition'!A87</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4976,7 +4978,7 @@
         <v>public final static String BGPLATFORM_CURRENTLYAVAILABLE = "bgplatform[X].currentlyavailable";</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="str">
         <f>'Property-Definition'!A88</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4995,7 +4997,7 @@
         <v>public final static String BGPLATFORM_CURRENT_CPULOAD = "bgplatform[X].current.cpuload";</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="str">
         <f>'Property-Definition'!A89</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5014,7 +5016,7 @@
         <v>public final static String BGPLATFORM_CURRENT_MEMORYLOAD = "bgplatform[X].current.memoryload";</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="str">
         <f>'Property-Definition'!A90</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5033,7 +5035,7 @@
         <v>public final static String BGPLATFORM_CURRENT_MEMORYLOADJVM = "bgplatform[X].current.memoryloadjvm";</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="str">
         <f>'Property-Definition'!A91</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5052,7 +5054,7 @@
         <v>public final static String BGPLATFORM_CURRENT_NUMTHREADS = "bgplatform[X].current.numthreads";</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="str">
         <f>'Property-Definition'!A92</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5069,6 +5071,1778 @@
 &amp; CHAR(34)
 &amp; ";"</f>
         <v>public final static String BGPLATFORM_CURRENT_THRESHOLDEXCEEDED = "bgplatform[X].current.thresholdexceeded";</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B93" xr:uid="{F30A1E73-A707-4178-9C72-9AC27F9EE5F7}"/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE54A29A-A704-4E09-86D6-1BE2A6729275}">
+  <dimension ref="A1:B93"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="str">
+        <f>'Property-Definition'!A1</f>
+        <v>performative</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="str">
+        <f>'Property-Definition'!A2</f>
+        <v>DB.SYSTEMS</v>
+      </c>
+      <c r="B2" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D2,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D2
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const DBSYSTEM: string = "dbSystem[X]";</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="str">
+        <f>'Property-Definition'!A3</f>
+        <v>DB.SYSTEMS.PARAMETER</v>
+      </c>
+      <c r="B3" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D3,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D3
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const DBSYSTEM: string = "dbSystem[X]";</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="str">
+        <f>'Property-Definition'!A4</f>
+        <v>DB.SYSTEMS.PARAMETER</v>
+      </c>
+      <c r="B4" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D4,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D4
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const DBSYSTEM_HIBERNATE_CONNECTION_DRIVER_CLASS: string = "dbSystem[X].hibernate.connection.driver_class";</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="str">
+        <f>'Property-Definition'!A5</f>
+        <v>DB.SYSTEMS.PARAMETER</v>
+      </c>
+      <c r="B5" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D5,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D5
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const DBSYSTEM_HIBERNATE_CONNECTION_URL: string = "dbSystem[X].hibernate.connection.url";</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="str">
+        <f>'Property-Definition'!A6</f>
+        <v>DB.SYSTEMS.PARAMETER</v>
+      </c>
+      <c r="B6" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D6,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D6
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const DBSYSTEM_HIBERNATE_CONNECTION_URL_MASK: string = "dbSystem[X].hibernate.connection.url.mask";</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="str">
+        <f>'Property-Definition'!A7</f>
+        <v>DB.SYSTEMS.PARAMETER</v>
+      </c>
+      <c r="B7" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D7,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D7
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const DBSYSTEM_HIBERNATE_DEFAULT_CATALOG: string = "dbSystem[X].hibernate.default_catalog";</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="str">
+        <f>'Property-Definition'!A8</f>
+        <v>DB.SYSTEMS.PARAMETER</v>
+      </c>
+      <c r="B8" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D8,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D8
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const DBSYSTEM_HIBERNATE_CONNECTION_USERNAME: string = "dbSystem[X].hibernate.connection.username";</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="str">
+        <f>'Property-Definition'!A9</f>
+        <v>DB.SYSTEMS.PARAMETER</v>
+      </c>
+      <c r="B9" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D9,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D9
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const DBSYSTEM_HIBERNATE_CONNECTION_PASSWORD: string = "dbSystem[X].hibernate.connection.password";</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="str">
+        <f>'Property-Definition'!A10</f>
+        <v>DB.FACTORIES</v>
+      </c>
+      <c r="B10" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D10,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D10
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const FACTORY: string = "factory[X]";</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="str">
+        <f>'Property-Definition'!A11</f>
+        <v>DB.FACTORIES</v>
+      </c>
+      <c r="B11" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D11,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D11
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const FACTORY_STATE: string = "factory[X].state";</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="str">
+        <f>'Property-Definition'!A12</f>
+        <v>DB.DERBY.NETWORKSERVER</v>
+      </c>
+      <c r="B12" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D12,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D12
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const ISSTARTDERBYNETWORKSERVER: string = "isStartDerbyNetworkServer";</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="str">
+        <f>'Property-Definition'!A13</f>
+        <v>DB.DERBY.NETWORKSERVER</v>
+      </c>
+      <c r="B13" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D13,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D13
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const HOST-IP: string = "host-IP";</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="str">
+        <f>'Property-Definition'!A14</f>
+        <v>DB.DERBY.NETWORKSERVER</v>
+      </c>
+      <c r="B14" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D14,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D14
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const PORT: string = "port";</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="str">
+        <f>'Property-Definition'!A15</f>
+        <v>DB.DERBY.NETWORKSERVER</v>
+      </c>
+      <c r="B15" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D15,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D15
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const USERNAME: string = "userName";</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="str">
+        <f>'Property-Definition'!A16</f>
+        <v>DB.DERBY.NETWORKSERVER</v>
+      </c>
+      <c r="B16" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D16,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D16
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const PASSWORD: string = "password";</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="str">
+        <f>'Property-Definition'!A17</f>
+        <v>DB.CONN.GENERAL</v>
+      </c>
+      <c r="B17" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D17,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D17
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const USEFOREVERYFACTORY: string = "useForEveryFactory";</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="str">
+        <f>'Property-Definition'!A18</f>
+        <v>DB.CONN.GENERAL</v>
+      </c>
+      <c r="B18" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D18,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D18
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const DBSYSTEM: string = "dbSystem";</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="str">
+        <f>'Property-Definition'!A19</f>
+        <v>DB.CONN.GENERAL</v>
+      </c>
+      <c r="B19" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D19,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D19
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const HIBERNATE_CONNECTION_DRIVER_CLASS: string = "hibernate.connection.driver_class";</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="str">
+        <f>'Property-Definition'!A20</f>
+        <v>DB.CONN.GENERAL</v>
+      </c>
+      <c r="B20" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D20,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D20
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const HIBERNATE_CONNECTION_URL: string = "hibernate.connection.url";</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="str">
+        <f>'Property-Definition'!A21</f>
+        <v>DB.CONN.GENERAL</v>
+      </c>
+      <c r="B21" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D21,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D21
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const HIBERNATE_DEFAULT_CATALOG: string = "hibernate.default_catalog";</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="str">
+        <f>'Property-Definition'!A22</f>
+        <v>DB.CONN.GENERAL</v>
+      </c>
+      <c r="B22" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D22,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D22
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const HIBERNATE_CONNECTION_USERNAME: string = "hibernate.connection.username";</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="str">
+        <f>'Property-Definition'!A23</f>
+        <v>DB.CONN.GENERAL</v>
+      </c>
+      <c r="B23" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D23,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D23
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const HIBERNATE_CONNECTION_PASSWORD: string = "hibernate.connection.password";</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="str">
+        <f>'Property-Definition'!A24</f>
+        <v>DB.CONN.FACTORY.GET</v>
+      </c>
+      <c r="B24" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D24,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D24
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const FACTORY_FACTORYID: string = "factory[X].factoryID";</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="str">
+        <f>'Property-Definition'!A25</f>
+        <v>DB.CONN.FACTORY.GET</v>
+      </c>
+      <c r="B25" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D25,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D25
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const FACTORY_DBSYSTEM: string = "factory[X].dbSystem";</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="str">
+        <f>'Property-Definition'!A26</f>
+        <v>DB.CONN.FACTORY.GET</v>
+      </c>
+      <c r="B26" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D26,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D26
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const FACTORY_HIBERNATE_CONNECTION_DRIVER_CLASS: string = "factory[X].hibernate.connection.driver_class";</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="str">
+        <f>'Property-Definition'!A27</f>
+        <v>DB.CONN.FACTORY.GET</v>
+      </c>
+      <c r="B27" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D27,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D27
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const FACTORY_HIBERNATE_CONNECTION_URL: string = "factory[X].hibernate.connection.url";</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="str">
+        <f>'Property-Definition'!A28</f>
+        <v>DB.CONN.FACTORY.GET</v>
+      </c>
+      <c r="B28" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D28,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D28
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const FACTORY_HIBERNATE_DEFAULT_CATALOG: string = "factory[X].hibernate.default_catalog";</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="str">
+        <f>'Property-Definition'!A29</f>
+        <v>DB.CONN.FACTORY.GET</v>
+      </c>
+      <c r="B29" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D29,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D29
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const FACTORY_HIBERNATE_CONNECTION_USERNAME: string = "factory[X].hibernate.connection.username";</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="str">
+        <f>'Property-Definition'!A30</f>
+        <v>DB.CONN.FACTORY.GET</v>
+      </c>
+      <c r="B30" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D30,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D30
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const FACTORY_HIBERNATE_CONNECTION_PASSWORD: string = "factory[X].hibernate.connection.password";</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="str">
+        <f>'Property-Definition'!A31</f>
+        <v>DB.CONN.FACTORY.SET</v>
+      </c>
+      <c r="B31" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D31,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D31
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const FACTORYID: string = "factoryID";</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="str">
+        <f>'Property-Definition'!A32</f>
+        <v>DB.CONN.FACTORY.SET</v>
+      </c>
+      <c r="B32" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D32,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D32
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const DBSYSTEM: string = "dbSystem";</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="str">
+        <f>'Property-Definition'!A33</f>
+        <v>DB.CONN.FACTORY.SET</v>
+      </c>
+      <c r="B33" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D33,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D33
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const HIBERNATE_CONNECTION_DRIVER_CLASS: string = "hibernate.connection.driver_class";</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="str">
+        <f>'Property-Definition'!A34</f>
+        <v>DB.CONN.FACTORY.SET</v>
+      </c>
+      <c r="B34" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D34,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D34
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const HIBERNATE_CONNECTION_URL: string = "hibernate.connection.url";</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="str">
+        <f>'Property-Definition'!A35</f>
+        <v>DB.CONN.FACTORY.SET</v>
+      </c>
+      <c r="B35" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D35,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D35
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const HIBERNATE_DEFAULT_CATALOG: string = "hibernate.default_catalog";</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="str">
+        <f>'Property-Definition'!A36</f>
+        <v>DB.CONN.FACTORY.SET</v>
+      </c>
+      <c r="B36" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D36,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D36
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const HIBERNATE_CONNECTION_USERNAME: string = "hibernate.connection.username";</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="str">
+        <f>'Property-Definition'!A37</f>
+        <v>DB.CONN.FACTORY.SET</v>
+      </c>
+      <c r="B37" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D37,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D37
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const HIBERNATE_CONNECTION_PASSWORD: string = "hibernate.connection.password";</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="str">
+        <f>'Property-Definition'!A38</f>
+        <v>DB.CONN.TEST</v>
+      </c>
+      <c r="B38" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D38,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D38
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const DBSYSTEM: string = "dbSystem";</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="str">
+        <f>'Property-Definition'!A39</f>
+        <v>DB.CONN.TEST</v>
+      </c>
+      <c r="B39" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D39,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D39
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const HIBERNATE_CONNECTION_DRIVER_CLASS: string = "hibernate.connection.driver_class";</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="str">
+        <f>'Property-Definition'!A40</f>
+        <v>DB.CONN.TEST</v>
+      </c>
+      <c r="B40" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D40,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D40
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const HIBERNATE_CONNECTION_URL: string = "hibernate.connection.url";</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="str">
+        <f>'Property-Definition'!A41</f>
+        <v>DB.CONN.TEST</v>
+      </c>
+      <c r="B41" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D41,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D41
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const HIBERNATE_DEFAULT_CATALOG: string = "hibernate.default_catalog";</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="str">
+        <f>'Property-Definition'!A42</f>
+        <v>DB.CONN.TEST</v>
+      </c>
+      <c r="B42" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D42,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D42
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const HIBERNATE_CONNECTION_USERNAME: string = "hibernate.connection.username";</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="str">
+        <f>'Property-Definition'!A43</f>
+        <v>DB.CONN.TEST</v>
+      </c>
+      <c r="B43" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D43,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D43
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const HIBERNATE_CONNECTION_PASSWORD: string = "hibernate.connection.password";</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="str">
+        <f>'Property-Definition'!A44</f>
+        <v>EXEC.MODE</v>
+      </c>
+      <c r="B44" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D44,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D44
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const EXEC_MODE: string = "exec.mode";</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="str">
+        <f>'Property-Definition'!A45</f>
+        <v>EXEC.MODE</v>
+      </c>
+      <c r="B45" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D45,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D45
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const SERVER_MASTER_URL: string = "server.master.url";</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" t="str">
+        <f>'Property-Definition'!A46</f>
+        <v>EXEC.MODE</v>
+      </c>
+      <c r="B46" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D46,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D46
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const SERVER_MASTER_PORT: string = "server.master.port";</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" t="str">
+        <f>'Property-Definition'!A47</f>
+        <v>EXEC.MODE</v>
+      </c>
+      <c r="B47" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D47,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D47
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const SERVER_MASTER_PORT_MTP: string = "server.master.port.mtp";</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" t="str">
+        <f>'Property-Definition'!A48</f>
+        <v>EXEC.MODE</v>
+      </c>
+      <c r="B48" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D48,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D48
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const SERVER_MASTER_PROTOCOL: string = "server.master.protocol";</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" t="str">
+        <f>'Property-Definition'!A49</f>
+        <v>EXEC.MODE</v>
+      </c>
+      <c r="B49" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D49,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D49
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const LOCAL_MTP_CREATION: string = "local.mtp.creation";</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" t="str">
+        <f>'Property-Definition'!A50</f>
+        <v>EXEC.MODE</v>
+      </c>
+      <c r="B50" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D50,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D50
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const LOCAL_MTP_URL: string = "local.mtp.url";</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" t="str">
+        <f>'Property-Definition'!A51</f>
+        <v>EXEC.MODE</v>
+      </c>
+      <c r="B51" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D51,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D51
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const LOCAL_MTP_PORT: string = "local.mtp.port";</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" t="str">
+        <f>'Property-Definition'!A52</f>
+        <v>EXEC.MODE</v>
+      </c>
+      <c r="B52" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D52,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D52
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const LOCAL_MTP_PROTOCOL: string = "local.mtp.protocol";</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" t="str">
+        <f>'Property-Definition'!A53</f>
+        <v>EXEC.MODE</v>
+      </c>
+      <c r="B53" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D53,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D53
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const EMBEDDEDSYSTEM_PROJECT: string = "embeddedsystem.project";</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" t="str">
+        <f>'Property-Definition'!A54</f>
+        <v>EXEC.MODE</v>
+      </c>
+      <c r="B54" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D54,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D54
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const DEVICE_SYSTEM_EXEC_MODE: string = "device_system_exec_mode";</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" t="str">
+        <f>'Property-Definition'!A55</f>
+        <v>EXEC.MODE</v>
+      </c>
+      <c r="B55" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D55,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D55
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const EMBEDDEDSYSTEM_AGENT_CLASSNAME: string = "embeddedsystem.agent[X].classname";</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" t="str">
+        <f>'Property-Definition'!A56</f>
+        <v>EXEC.MODE</v>
+      </c>
+      <c r="B56" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D56,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D56
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const EMBEDDEDSYSTEM_AGENT_AGENTNAME: string = "embeddedsystem.agent[X].agentname";</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" t="str">
+        <f>'Property-Definition'!A57</f>
+        <v>EXEC.MODE</v>
+      </c>
+      <c r="B57" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D57,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D57
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const SERVICE_SERVICE_SETUP: string = "service.service_setup";</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" t="str">
+        <f>'Property-Definition'!A58</f>
+        <v>EXEC.MODE</v>
+      </c>
+      <c r="B58" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D58,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D58
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const LOCAL_IP_SELECTION: string = "local.ip.selection[X]";</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" t="str">
+        <f>'Property-Definition'!A59</f>
+        <v>EXEC.MODE</v>
+      </c>
+      <c r="B59" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D59,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D59
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const FACTORY_ID: string = "factory_id";</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" t="e">
+        <f>'Property-Definition'!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="B60" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D60,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D60
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const AGENT_CLASSNAME: string = "agent[X].classname";</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" t="str">
+        <f>'Property-Definition'!A60</f>
+        <v>AWB.AGENTS</v>
+      </c>
+      <c r="B61" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D61,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D61
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const PROJECT: string = "project[X]";</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" t="str">
+        <f>'Property-Definition'!A61</f>
+        <v>PROJECTS</v>
+      </c>
+      <c r="B62" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D62,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D62
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const PROJECT_SETUP: string = "project[X].setup[X]";</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" t="str">
+        <f>'Property-Definition'!A62</f>
+        <v>PROJECT.SETUPS[X]</v>
+      </c>
+      <c r="B63" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D63,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D63
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_CONTACTAGENT: string = "bgplatform[X].contactagent";</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" t="str">
+        <f>'Property-Definition'!A63</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B64" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D64,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D64
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_PLATFORMNAME: string = "bgplatform[X].platformname";</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" t="str">
+        <f>'Property-Definition'!A60</f>
+        <v>AWB.AGENTS</v>
+      </c>
+      <c r="B65" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D65,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D65
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_SERVER: string = "bgplatform[X].server";</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" t="str">
+        <f>'Property-Definition'!A61</f>
+        <v>PROJECTS</v>
+      </c>
+      <c r="B66" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D66,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D66
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_IPADDRESS: string = "bgplatform[X].ipaddress";</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" t="str">
+        <f>'Property-Definition'!A62</f>
+        <v>PROJECT.SETUPS[X]</v>
+      </c>
+      <c r="B67" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D67,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D67
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_URL: string = "bgplatform[X].url";</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" t="str">
+        <f>'Property-Definition'!A67</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B68" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D68,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D68
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_JADEPORT: string = "bgplatform[X].jadeport";</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" t="str">
+        <f>'Property-Definition'!A68</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B69" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D69,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D69
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_HTTPMTP: string = "bgplatform[X].httpmtp";</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" t="str">
+        <f>'Property-Definition'!A69</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B70" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D70,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D70
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_VERSIONMAJOR: string = "bgplatform[X].versionmajor";</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" t="str">
+        <f>'Property-Definition'!A70</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B71" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D71,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D71
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_VERSIONMINOR: string = "bgplatform[X].versionminor";</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" t="str">
+        <f>'Property-Definition'!A71</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B72" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D72,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D72
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_VERSIONMICRO: string = "bgplatform[X].versionmicro";</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" t="str">
+        <f>'Property-Definition'!A72</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B73" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D73,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D73
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_VERSIONBUILD: string = "bgplatform[X].versionbuild";</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" t="str">
+        <f>'Property-Definition'!A73</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B74" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D74,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D74
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_OS_NAME: string = "bgplatform[X].os.name";</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" t="str">
+        <f>'Property-Definition'!A74</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B75" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D75,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D75
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_OS_VERSION: string = "bgplatform[X].os.version";</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" t="str">
+        <f>'Property-Definition'!A75</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B76" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D76,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D76
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_OS_ARCHITECTURE: string = "bgplatform[X].os.architecture";</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77" t="str">
+        <f>'Property-Definition'!A76</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B77" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D77,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D77
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_CPU_NAME: string = "bgplatform[X].cpu.name";</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78" t="str">
+        <f>'Property-Definition'!A77</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B78" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D78,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D78
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_CPU_NUMLOGICAL: string = "bgplatform[X].cpu.numlogical";</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79" t="str">
+        <f>'Property-Definition'!A78</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B79" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D79,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D79
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_CPU_NUMPHYSICAL: string = "bgplatform[X].cpu.numphysical";</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80" t="str">
+        <f>'Property-Definition'!A79</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B80" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D80,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D80
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_CPU_SPEEDMHZ: string = "bgplatform[X].cpu.speedmhz";</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A81" t="str">
+        <f>'Property-Definition'!A80</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B81" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D81,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D81
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_MEMORYMB: string = "bgplatform[X].memorymb";</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A82" t="str">
+        <f>'Property-Definition'!A81</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B82" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D82,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D82
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_BENCHMARKVALUE: string = "bgplatform[X].benchmarkvalue";</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83" t="str">
+        <f>'Property-Definition'!A82</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B83" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D83,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D83
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_TIME_ONLINESINCE: string = "bgplatform[X].time.onlinesince";</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84" t="str">
+        <f>'Property-Definition'!A83</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B84" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D84,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D84
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_TIME_LASTCONTACT: string = "bgplatform[X].time.lastcontact";</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85" t="str">
+        <f>'Property-Definition'!A84</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B85" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D85,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D85
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_LOCALTIME_ONLINESINCE: string = "bgplatform[X].localtime.onlinesince";</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86" t="str">
+        <f>'Property-Definition'!A85</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B86" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D86,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D86
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_LOCALTIME_LASTCONTACT: string = "bgplatform[X].localtime.lastcontact";</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87" t="str">
+        <f>'Property-Definition'!A86</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B87" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D87,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D87
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_CURRENTLYAVAILABLE: string = "bgplatform[X].currentlyavailable";</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88" t="str">
+        <f>'Property-Definition'!A87</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B88" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D88,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D88
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_CURRENT_CPULOAD: string = "bgplatform[X].current.cpuload";</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A89" t="str">
+        <f>'Property-Definition'!A88</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B89" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D89,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D89
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_CURRENT_MEMORYLOAD: string = "bgplatform[X].current.memoryload";</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A90" t="str">
+        <f>'Property-Definition'!A89</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B90" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D90,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D90
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_CURRENT_MEMORYLOADJVM: string = "bgplatform[X].current.memoryloadjvm";</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A91" t="str">
+        <f>'Property-Definition'!A90</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B91" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D91,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D91
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_CURRENT_NUMTHREADS: string = "bgplatform[X].current.numthreads";</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92" t="str">
+        <f>'Property-Definition'!A91</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B92" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D92,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D92
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const BGPLATFORM_CURRENT_THRESHOLDEXCEEDED: string = "bgplatform[X].current.thresholdexceeded";</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93" t="str">
+        <f>'Property-Definition'!A92</f>
+        <v>EXEC.MASTER.SLAVES.GET</v>
+      </c>
+      <c r="B93" t="str">
+        <f>"const "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D93,"[X]",""),".","_")
+)
+&amp; ": string = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D93
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>const : string = "";</v>
       </c>
     </row>
   </sheetData>
@@ -5078,15 +6852,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101004FB79D76D905EB41B4AD64ED4839597F" ma:contentTypeVersion="11" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="0622d98e252eab518d4b54f931ba6851">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="897f6830-f425-409d-b8f5-ce1019056d9e" xmlns:ns3="f2404b4d-361b-46d3-b2ec-035eed29e274" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dd5f302b3846fd12003b89c8f5b7df36" ns2:_="" ns3:_="">
     <xsd:import namespace="897f6830-f425-409d-b8f5-ce1019056d9e"/>
@@ -5281,6 +7046,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -5293,14 +7067,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A33EE264-283E-4F19-BA61-B3264EA417E2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5319,6 +7085,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF16440F-B0E0-4269-97EE-BEB05B0223C8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Added integration bundle for exec.master.slaves.get
</commit_message>
<xml_diff>
--- a/AWB-RestApi-PropertyDictionary.xlsx
+++ b/AWB-RestApi-PropertyDictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\AgentWorkbench\eclipseProjects\de.enflexit.awb\bundles\web\xApi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27507518-1AE7-4149-A7A0-648A1B12E337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99183C0D-AEA7-4600-B0D8-DDF3E48226A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="195">
   <si>
     <t>key</t>
   </si>
@@ -622,6 +622,9 @@
   </si>
   <si>
     <t>e.g. '1971.77001953125'</t>
+  </si>
+  <si>
+    <t>de.enflexit.awb.bgSystem</t>
   </si>
 </sst>
 </file>
@@ -2629,6 +2632,9 @@
       <c r="F60" t="s">
         <v>122</v>
       </c>
+      <c r="H60" t="s">
+        <v>194</v>
+      </c>
       <c r="I60" s="5" t="s">
         <v>59</v>
       </c>
@@ -2655,6 +2661,9 @@
       <c r="F61" t="s">
         <v>93</v>
       </c>
+      <c r="H61" t="s">
+        <v>194</v>
+      </c>
       <c r="I61" s="5" t="s">
         <v>59</v>
       </c>
@@ -2681,6 +2690,9 @@
       <c r="F62" t="s">
         <v>126</v>
       </c>
+      <c r="H62" t="s">
+        <v>194</v>
+      </c>
       <c r="I62" s="5" t="s">
         <v>59</v>
       </c>
@@ -2704,6 +2716,9 @@
       <c r="F63" t="s">
         <v>172</v>
       </c>
+      <c r="H63" t="s">
+        <v>194</v>
+      </c>
       <c r="I63" s="5" t="s">
         <v>59</v>
       </c>
@@ -2724,6 +2739,9 @@
       <c r="F64" t="s">
         <v>174</v>
       </c>
+      <c r="H64" t="s">
+        <v>194</v>
+      </c>
       <c r="I64" s="5" t="s">
         <v>59</v>
       </c>
@@ -2744,6 +2762,9 @@
       <c r="F65" t="s">
         <v>21</v>
       </c>
+      <c r="H65" t="s">
+        <v>194</v>
+      </c>
       <c r="I65" s="5" t="s">
         <v>59</v>
       </c>
@@ -2764,6 +2785,9 @@
       <c r="F66" t="s">
         <v>183</v>
       </c>
+      <c r="H66" t="s">
+        <v>194</v>
+      </c>
       <c r="I66" s="5" t="s">
         <v>59</v>
       </c>
@@ -2784,6 +2808,9 @@
       <c r="F67" t="s">
         <v>173</v>
       </c>
+      <c r="H67" t="s">
+        <v>194</v>
+      </c>
       <c r="I67" s="5" t="s">
         <v>59</v>
       </c>
@@ -2804,6 +2831,9 @@
       <c r="F68" t="s">
         <v>184</v>
       </c>
+      <c r="H68" t="s">
+        <v>194</v>
+      </c>
       <c r="I68" s="5" t="s">
         <v>59</v>
       </c>
@@ -2824,6 +2854,9 @@
       <c r="F69" t="s">
         <v>182</v>
       </c>
+      <c r="H69" t="s">
+        <v>194</v>
+      </c>
       <c r="I69" s="5" t="s">
         <v>59</v>
       </c>
@@ -2844,6 +2877,9 @@
       <c r="F70" t="s">
         <v>187</v>
       </c>
+      <c r="H70" t="s">
+        <v>194</v>
+      </c>
       <c r="I70" s="5" t="s">
         <v>59</v>
       </c>
@@ -2864,6 +2900,9 @@
       <c r="F71" t="s">
         <v>188</v>
       </c>
+      <c r="H71" t="s">
+        <v>194</v>
+      </c>
       <c r="I71" s="5" t="s">
         <v>59</v>
       </c>
@@ -2884,6 +2923,9 @@
       <c r="F72" t="s">
         <v>188</v>
       </c>
+      <c r="H72" t="s">
+        <v>194</v>
+      </c>
       <c r="I72" s="5" t="s">
         <v>59</v>
       </c>
@@ -2904,6 +2946,9 @@
       <c r="F73" t="s">
         <v>192</v>
       </c>
+      <c r="H73" t="s">
+        <v>194</v>
+      </c>
       <c r="I73" s="5" t="s">
         <v>59</v>
       </c>
@@ -2924,6 +2969,9 @@
       <c r="F74" t="s">
         <v>189</v>
       </c>
+      <c r="H74" t="s">
+        <v>194</v>
+      </c>
       <c r="I74" s="5" t="s">
         <v>59</v>
       </c>
@@ -2944,6 +2992,9 @@
       <c r="F75" t="s">
         <v>190</v>
       </c>
+      <c r="H75" t="s">
+        <v>194</v>
+      </c>
       <c r="I75" s="5" t="s">
         <v>59</v>
       </c>
@@ -2964,6 +3015,9 @@
       <c r="F76" t="s">
         <v>191</v>
       </c>
+      <c r="H76" t="s">
+        <v>194</v>
+      </c>
       <c r="I76" s="5" t="s">
         <v>59</v>
       </c>
@@ -2984,6 +3038,9 @@
       <c r="F77" t="s">
         <v>175</v>
       </c>
+      <c r="H77" t="s">
+        <v>194</v>
+      </c>
       <c r="I77" s="5" t="s">
         <v>59</v>
       </c>
@@ -3004,6 +3061,9 @@
       <c r="F78" t="s">
         <v>176</v>
       </c>
+      <c r="H78" t="s">
+        <v>194</v>
+      </c>
       <c r="I78" s="5" t="s">
         <v>59</v>
       </c>
@@ -3024,6 +3084,9 @@
       <c r="F79" t="s">
         <v>176</v>
       </c>
+      <c r="H79" t="s">
+        <v>194</v>
+      </c>
       <c r="I79" s="5" t="s">
         <v>59</v>
       </c>
@@ -3044,6 +3107,9 @@
       <c r="F80" t="s">
         <v>177</v>
       </c>
+      <c r="H80" t="s">
+        <v>194</v>
+      </c>
       <c r="I80" s="5" t="s">
         <v>59</v>
       </c>
@@ -3064,6 +3130,9 @@
       <c r="F81" t="s">
         <v>173</v>
       </c>
+      <c r="H81" t="s">
+        <v>194</v>
+      </c>
       <c r="I81" s="5" t="s">
         <v>59</v>
       </c>
@@ -3084,6 +3153,9 @@
       <c r="F82" t="s">
         <v>193</v>
       </c>
+      <c r="H82" t="s">
+        <v>194</v>
+      </c>
       <c r="I82" s="5" t="s">
         <v>59</v>
       </c>
@@ -3104,6 +3176,9 @@
       <c r="F83" t="s">
         <v>185</v>
       </c>
+      <c r="H83" t="s">
+        <v>194</v>
+      </c>
       <c r="I83" s="5" t="s">
         <v>59</v>
       </c>
@@ -3124,6 +3199,9 @@
       <c r="F84" t="s">
         <v>186</v>
       </c>
+      <c r="H84" t="s">
+        <v>194</v>
+      </c>
       <c r="I84" s="5" t="s">
         <v>59</v>
       </c>
@@ -3144,6 +3222,9 @@
       <c r="F85" t="s">
         <v>186</v>
       </c>
+      <c r="H85" t="s">
+        <v>194</v>
+      </c>
       <c r="I85" s="5" t="s">
         <v>59</v>
       </c>
@@ -3164,6 +3245,9 @@
       <c r="F86" t="s">
         <v>186</v>
       </c>
+      <c r="H86" t="s">
+        <v>194</v>
+      </c>
       <c r="I86" s="5" t="s">
         <v>59</v>
       </c>
@@ -3184,6 +3268,9 @@
       <c r="F87" t="s">
         <v>21</v>
       </c>
+      <c r="H87" t="s">
+        <v>194</v>
+      </c>
       <c r="I87" s="5" t="s">
         <v>59</v>
       </c>
@@ -3204,6 +3291,9 @@
       <c r="F88" t="s">
         <v>179</v>
       </c>
+      <c r="H88" t="s">
+        <v>194</v>
+      </c>
       <c r="I88" s="5" t="s">
         <v>59</v>
       </c>
@@ -3224,6 +3314,9 @@
       <c r="F89" t="s">
         <v>178</v>
       </c>
+      <c r="H89" t="s">
+        <v>194</v>
+      </c>
       <c r="I89" s="5" t="s">
         <v>59</v>
       </c>
@@ -3244,6 +3337,9 @@
       <c r="F90" t="s">
         <v>180</v>
       </c>
+      <c r="H90" t="s">
+        <v>194</v>
+      </c>
       <c r="I90" s="5" t="s">
         <v>59</v>
       </c>
@@ -3264,6 +3360,9 @@
       <c r="F91" t="s">
         <v>181</v>
       </c>
+      <c r="H91" t="s">
+        <v>194</v>
+      </c>
       <c r="I91" s="5" t="s">
         <v>59</v>
       </c>
@@ -3283,6 +3382,9 @@
       </c>
       <c r="F92" t="s">
         <v>21</v>
+      </c>
+      <c r="H92" t="s">
+        <v>194</v>
       </c>
       <c r="I92" s="5" t="s">
         <v>59</v>
@@ -5078,15 +5180,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101004FB79D76D905EB41B4AD64ED4839597F" ma:contentTypeVersion="11" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="0622d98e252eab518d4b54f931ba6851">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="897f6830-f425-409d-b8f5-ce1019056d9e" xmlns:ns3="f2404b4d-361b-46d3-b2ec-035eed29e274" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dd5f302b3846fd12003b89c8f5b7df36" ns2:_="" ns3:_="">
     <xsd:import namespace="897f6830-f425-409d-b8f5-ce1019056d9e"/>
@@ -5281,6 +5374,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -5293,14 +5395,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A33EE264-283E-4F19-BA61-B3264EA417E2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5319,6 +5413,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF16440F-B0E0-4269-97EE-BEB05B0223C8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Small change to update.strategy
Changed the key to "isautoupdate".
Changed the valuetype to boolean.
</commit_message>
<xml_diff>
--- a/AWB-RestApi-PropertyDictionary.xlsx
+++ b/AWB-RestApi-PropertyDictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\AgentWorkbench\eclipseProjects\de.enflexit.awb\bundles\web\xApi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95A5B0DE-BE94-4792-A01E-9ED02051D4AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7D8C5C0-CDE6-48DD-9F29-620EDCA19AE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Property-Definition" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="767" uniqueCount="197">
   <si>
     <t>key</t>
   </si>
@@ -630,13 +630,7 @@
     <t>UPDATE.STRATEGY</t>
   </si>
   <si>
-    <t>update.strategy</t>
-  </si>
-  <si>
-    <t>e.g. 'automatic'</t>
-  </si>
-  <si>
-    <t>"automatic", "askuser"</t>
+    <t>isautoupdate</t>
   </si>
 </sst>
 </file>
@@ -2734,6 +2728,9 @@
       <c r="I63" s="5" t="s">
         <v>59</v>
       </c>
+      <c r="J63" s="5" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
@@ -2757,8 +2754,11 @@
       <c r="I64" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J64" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>83</v>
       </c>
@@ -2780,8 +2780,11 @@
       <c r="I65" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J65" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>83</v>
       </c>
@@ -2803,8 +2806,11 @@
       <c r="I66" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J66" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>83</v>
       </c>
@@ -2826,8 +2832,11 @@
       <c r="I67" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J67" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>83</v>
       </c>
@@ -2849,8 +2858,11 @@
       <c r="I68" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J68" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>83</v>
       </c>
@@ -2872,8 +2884,11 @@
       <c r="I69" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J69" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>83</v>
       </c>
@@ -2895,8 +2910,11 @@
       <c r="I70" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J70" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>83</v>
       </c>
@@ -2918,8 +2936,11 @@
       <c r="I71" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J71" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>83</v>
       </c>
@@ -2941,8 +2962,11 @@
       <c r="I72" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J72" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>83</v>
       </c>
@@ -2964,8 +2988,11 @@
       <c r="I73" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J73" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>83</v>
       </c>
@@ -2987,8 +3014,11 @@
       <c r="I74" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J74" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>83</v>
       </c>
@@ -3010,8 +3040,11 @@
       <c r="I75" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J75" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>83</v>
       </c>
@@ -3033,8 +3066,11 @@
       <c r="I76" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J76" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>83</v>
       </c>
@@ -3056,8 +3092,11 @@
       <c r="I77" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J77" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>83</v>
       </c>
@@ -3079,8 +3118,11 @@
       <c r="I78" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J78" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>83</v>
       </c>
@@ -3102,8 +3144,11 @@
       <c r="I79" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J79" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>83</v>
       </c>
@@ -3125,8 +3170,11 @@
       <c r="I80" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J80" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>83</v>
       </c>
@@ -3148,8 +3196,11 @@
       <c r="I81" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J81" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>83</v>
       </c>
@@ -3171,8 +3222,11 @@
       <c r="I82" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J82" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>83</v>
       </c>
@@ -3194,8 +3248,11 @@
       <c r="I83" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J83" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>83</v>
       </c>
@@ -3217,8 +3274,11 @@
       <c r="I84" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J84" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>83</v>
       </c>
@@ -3240,8 +3300,11 @@
       <c r="I85" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J85" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>83</v>
       </c>
@@ -3263,8 +3326,11 @@
       <c r="I86" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J86" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>83</v>
       </c>
@@ -3286,8 +3352,11 @@
       <c r="I87" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J87" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>83</v>
       </c>
@@ -3309,8 +3378,11 @@
       <c r="I88" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J88" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>83</v>
       </c>
@@ -3332,8 +3404,11 @@
       <c r="I89" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J89" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>83</v>
       </c>
@@ -3355,8 +3430,11 @@
       <c r="I90" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J90" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>83</v>
       </c>
@@ -3378,8 +3456,11 @@
       <c r="I91" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J91" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>83</v>
       </c>
@@ -3401,8 +3482,11 @@
       <c r="I92" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J92" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>195</v>
       </c>
@@ -3413,13 +3497,10 @@
         <v>196</v>
       </c>
       <c r="E93" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="F93" t="s">
-        <v>197</v>
-      </c>
-      <c r="G93" t="s">
-        <v>198</v>
+        <v>21</v>
       </c>
       <c r="H93" t="s">
         <v>136</v>
@@ -3429,7 +3510,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:J43 J44:J62 I44:I93">
+  <conditionalFormatting sqref="I2:J43 J44:J92 I44:I93">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Updated Rest Api Proeprty Dictionary
</commit_message>
<xml_diff>
--- a/AWB-RestApi-PropertyDictionary.xlsx
+++ b/AWB-RestApi-PropertyDictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\AgentWorkbench\eclipseProjects\de.enflexit.awb\bundles\web\xApi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7D8C5C0-CDE6-48DD-9F29-620EDCA19AE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87407461-A88A-427E-8DD0-874977FBD40F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Property-Definition" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="767" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="215">
   <si>
     <t>key</t>
   </si>
@@ -631,6 +631,60 @@
   </si>
   <si>
     <t>isautoupdate</t>
+  </si>
+  <si>
+    <t>updatecheck.backend.ispending</t>
+  </si>
+  <si>
+    <t>updatecheck.backend.isavailable</t>
+  </si>
+  <si>
+    <t>updatecheck.backend.lastcheck</t>
+  </si>
+  <si>
+    <t>updatecheck.backend.version</t>
+  </si>
+  <si>
+    <t>updatecheck.frontend.version</t>
+  </si>
+  <si>
+    <t>updatecheck.frontend.isavailable</t>
+  </si>
+  <si>
+    <t>updatecheck.frontend.lastcheck</t>
+  </si>
+  <si>
+    <t>de.enflexit.awb.ws.core</t>
+  </si>
+  <si>
+    <t>UPDATE.FRONTEND.CHECK</t>
+  </si>
+  <si>
+    <t>updatecheck.frontend.ispending</t>
+  </si>
+  <si>
+    <t>UPDATE.BACKEND.CHECK[isForceCheck]</t>
+  </si>
+  <si>
+    <t>isForceCheck = true | false</t>
+  </si>
+  <si>
+    <t>e.g. '21.05.26 16:49'</t>
+  </si>
+  <si>
+    <t>UPDATE.BACKEND.EXECUTE</t>
+  </si>
+  <si>
+    <t>update.progress</t>
+  </si>
+  <si>
+    <t>e.g. '25'</t>
+  </si>
+  <si>
+    <t>update.status</t>
+  </si>
+  <si>
+    <t>e.g. 'Pending', 'no update available', 'update finalized'</t>
   </si>
 </sst>
 </file>
@@ -1010,21 +1064,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K93"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K105"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="28.7109375" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" customWidth="1"/>
-    <col min="4" max="4" width="54.140625" customWidth="1"/>
-    <col min="5" max="5" width="17.140625" customWidth="1"/>
+    <col min="1" max="1" width="34.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.7265625" customWidth="1"/>
+    <col min="3" max="3" width="14.26953125" customWidth="1"/>
+    <col min="4" max="4" width="54.1796875" customWidth="1"/>
+    <col min="5" max="5" width="17.1796875" customWidth="1"/>
     <col min="6" max="6" width="79" customWidth="1"/>
-    <col min="7" max="7" width="18.140625" customWidth="1"/>
-    <col min="8" max="8" width="34.85546875" customWidth="1"/>
-    <col min="9" max="10" width="17.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="113.7109375" customWidth="1"/>
+    <col min="7" max="7" width="18.1796875" customWidth="1"/>
+    <col min="8" max="8" width="34.81640625" customWidth="1"/>
+    <col min="9" max="10" width="17.7265625" style="5" customWidth="1"/>
+    <col min="11" max="11" width="113.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -1059,7 +1114,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1088,7 +1143,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>43</v>
       </c>
@@ -1114,7 +1169,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>43</v>
       </c>
@@ -1140,7 +1195,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -1166,7 +1221,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -1192,7 +1247,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>43</v>
       </c>
@@ -1218,7 +1273,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -1244,7 +1299,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>43</v>
       </c>
@@ -1270,7 +1325,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -1299,7 +1354,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -1331,7 +1386,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -1360,7 +1415,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -1389,7 +1444,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -1419,7 +1474,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -1448,7 +1503,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -1477,7 +1532,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>41</v>
       </c>
@@ -1506,7 +1561,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>41</v>
       </c>
@@ -1535,7 +1590,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>41</v>
       </c>
@@ -1561,7 +1616,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>41</v>
       </c>
@@ -1587,7 +1642,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>41</v>
       </c>
@@ -1613,7 +1668,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>41</v>
       </c>
@@ -1639,7 +1694,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>41</v>
       </c>
@@ -1665,7 +1720,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>64</v>
       </c>
@@ -1694,7 +1749,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>64</v>
       </c>
@@ -1723,7 +1778,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>64</v>
       </c>
@@ -1749,7 +1804,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>64</v>
       </c>
@@ -1775,7 +1830,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>64</v>
       </c>
@@ -1801,7 +1856,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>64</v>
       </c>
@@ -1827,7 +1882,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>64</v>
       </c>
@@ -1853,7 +1908,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>65</v>
       </c>
@@ -1879,7 +1934,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>65</v>
       </c>
@@ -1905,7 +1960,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>65</v>
       </c>
@@ -1931,7 +1986,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>65</v>
       </c>
@@ -1957,7 +2012,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>65</v>
       </c>
@@ -1983,7 +2038,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>65</v>
       </c>
@@ -2009,7 +2064,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>65</v>
       </c>
@@ -2035,7 +2090,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>73</v>
       </c>
@@ -2061,7 +2116,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>73</v>
       </c>
@@ -2087,7 +2142,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>73</v>
       </c>
@@ -2113,7 +2168,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>73</v>
       </c>
@@ -2139,7 +2194,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>73</v>
       </c>
@@ -2165,7 +2220,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>73</v>
       </c>
@@ -2191,7 +2246,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>82</v>
       </c>
@@ -2220,7 +2275,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>82</v>
       </c>
@@ -2246,7 +2301,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>82</v>
       </c>
@@ -2272,7 +2327,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>82</v>
       </c>
@@ -2298,7 +2353,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>82</v>
       </c>
@@ -2327,7 +2382,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>82</v>
       </c>
@@ -2356,7 +2411,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>82</v>
       </c>
@@ -2382,7 +2437,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>82</v>
       </c>
@@ -2408,7 +2463,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>82</v>
       </c>
@@ -2437,7 +2492,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>82</v>
       </c>
@@ -2463,7 +2518,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>82</v>
       </c>
@@ -2492,7 +2547,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>82</v>
       </c>
@@ -2518,7 +2573,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>82</v>
       </c>
@@ -2544,7 +2599,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>82</v>
       </c>
@@ -2570,7 +2625,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>82</v>
       </c>
@@ -2596,7 +2651,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>82</v>
       </c>
@@ -2622,7 +2677,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>91</v>
       </c>
@@ -2651,7 +2706,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>94</v>
       </c>
@@ -2677,7 +2732,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>95</v>
       </c>
@@ -2706,7 +2761,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>83</v>
       </c>
@@ -2732,7 +2787,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>83</v>
       </c>
@@ -2758,7 +2813,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>83</v>
       </c>
@@ -2784,7 +2839,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>83</v>
       </c>
@@ -2810,7 +2865,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>83</v>
       </c>
@@ -2836,7 +2891,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>83</v>
       </c>
@@ -2862,7 +2917,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>83</v>
       </c>
@@ -2888,7 +2943,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>83</v>
       </c>
@@ -2914,7 +2969,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>83</v>
       </c>
@@ -2940,7 +2995,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>83</v>
       </c>
@@ -2966,7 +3021,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>83</v>
       </c>
@@ -2992,7 +3047,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>83</v>
       </c>
@@ -3018,7 +3073,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>83</v>
       </c>
@@ -3044,7 +3099,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>83</v>
       </c>
@@ -3070,7 +3125,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>83</v>
       </c>
@@ -3096,7 +3151,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>83</v>
       </c>
@@ -3122,7 +3177,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>83</v>
       </c>
@@ -3148,7 +3203,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>83</v>
       </c>
@@ -3174,7 +3229,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>83</v>
       </c>
@@ -3200,7 +3255,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>83</v>
       </c>
@@ -3226,7 +3281,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>83</v>
       </c>
@@ -3252,7 +3307,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>83</v>
       </c>
@@ -3278,7 +3333,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>83</v>
       </c>
@@ -3304,7 +3359,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>83</v>
       </c>
@@ -3330,7 +3385,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>83</v>
       </c>
@@ -3356,7 +3411,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>83</v>
       </c>
@@ -3382,7 +3437,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>83</v>
       </c>
@@ -3408,7 +3463,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>83</v>
       </c>
@@ -3434,7 +3489,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>83</v>
       </c>
@@ -3460,7 +3515,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>83</v>
       </c>
@@ -3486,7 +3541,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>195</v>
       </c>
@@ -3503,14 +3558,223 @@
         <v>21</v>
       </c>
       <c r="H93" t="s">
+        <v>204</v>
+      </c>
+      <c r="I93" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>207</v>
+      </c>
+      <c r="B94" t="s">
+        <v>208</v>
+      </c>
+      <c r="C94" t="s">
+        <v>5</v>
+      </c>
+      <c r="D94" t="s">
+        <v>197</v>
+      </c>
+      <c r="E94" t="s">
+        <v>20</v>
+      </c>
+      <c r="F94" t="s">
+        <v>21</v>
+      </c>
+      <c r="H94" t="s">
         <v>136</v>
       </c>
-      <c r="I93" s="5" t="s">
-        <v>59</v>
+      <c r="I94" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>207</v>
+      </c>
+      <c r="B95" t="s">
+        <v>208</v>
+      </c>
+      <c r="C95" t="s">
+        <v>5</v>
+      </c>
+      <c r="D95" t="s">
+        <v>198</v>
+      </c>
+      <c r="E95" t="s">
+        <v>20</v>
+      </c>
+      <c r="F95" t="s">
+        <v>21</v>
+      </c>
+      <c r="H95" t="s">
+        <v>136</v>
+      </c>
+      <c r="I95" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>207</v>
+      </c>
+      <c r="B96" t="s">
+        <v>208</v>
+      </c>
+      <c r="C96" t="s">
+        <v>5</v>
+      </c>
+      <c r="D96" t="s">
+        <v>199</v>
+      </c>
+      <c r="E96" t="s">
+        <v>7</v>
+      </c>
+      <c r="F96" t="s">
+        <v>209</v>
+      </c>
+      <c r="H96" t="s">
+        <v>136</v>
+      </c>
+      <c r="I96" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
+        <v>207</v>
+      </c>
+      <c r="B97" t="s">
+        <v>208</v>
+      </c>
+      <c r="C97" t="s">
+        <v>5</v>
+      </c>
+      <c r="D97" t="s">
+        <v>200</v>
+      </c>
+      <c r="E97" t="s">
+        <v>7</v>
+      </c>
+      <c r="H97" t="s">
+        <v>136</v>
+      </c>
+      <c r="I97" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
+        <v>210</v>
+      </c>
+      <c r="C98" t="s">
+        <v>5</v>
+      </c>
+      <c r="D98" t="s">
+        <v>213</v>
+      </c>
+      <c r="E98" t="s">
+        <v>7</v>
+      </c>
+      <c r="F98" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
+        <v>210</v>
+      </c>
+      <c r="C99" t="s">
+        <v>5</v>
+      </c>
+      <c r="D99" t="s">
+        <v>211</v>
+      </c>
+      <c r="E99" t="s">
+        <v>26</v>
+      </c>
+      <c r="F99" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
+        <v>205</v>
+      </c>
+      <c r="C102" t="s">
+        <v>5</v>
+      </c>
+      <c r="D102" t="s">
+        <v>206</v>
+      </c>
+      <c r="E102" t="s">
+        <v>20</v>
+      </c>
+      <c r="F102" t="s">
+        <v>21</v>
+      </c>
+      <c r="H102" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
+        <v>205</v>
+      </c>
+      <c r="C103" t="s">
+        <v>5</v>
+      </c>
+      <c r="D103" t="s">
+        <v>202</v>
+      </c>
+      <c r="E103" t="s">
+        <v>20</v>
+      </c>
+      <c r="F103" t="s">
+        <v>21</v>
+      </c>
+      <c r="H103" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
+        <v>205</v>
+      </c>
+      <c r="C104" t="s">
+        <v>5</v>
+      </c>
+      <c r="D104" t="s">
+        <v>203</v>
+      </c>
+      <c r="E104" t="s">
+        <v>7</v>
+      </c>
+      <c r="H104" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
+        <v>205</v>
+      </c>
+      <c r="C105" t="s">
+        <v>5</v>
+      </c>
+      <c r="D105" t="s">
+        <v>201</v>
+      </c>
+      <c r="E105" t="s">
+        <v>7</v>
+      </c>
+      <c r="H105" t="s">
+        <v>204</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:J43 J44:J92 I44:I93">
+  <conditionalFormatting sqref="I2:J43 J44:J92 I44:I101">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>
@@ -3528,14 +3792,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F30A1E73-A707-4178-9C72-9AC27F9EE5F7}">
-  <dimension ref="A1:B93"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B113"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="24.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="str">
         <f>'Property-Definition'!A1</f>
         <v>performative</v>
@@ -3544,7 +3808,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="str">
         <f>'Property-Definition'!A2</f>
         <v>DB.SYSTEMS</v>
@@ -3563,7 +3827,7 @@
         <v>public final static String DBSYSTEM = "dbSystem[X]";</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="str">
         <f>'Property-Definition'!A3</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3582,7 +3846,7 @@
         <v>public final static String DBSYSTEM = "dbSystem[X]";</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="str">
         <f>'Property-Definition'!A4</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3601,7 +3865,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_DRIVER_CLASS = "dbSystem[X].hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="str">
         <f>'Property-Definition'!A5</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3620,7 +3884,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_URL = "dbSystem[X].hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="str">
         <f>'Property-Definition'!A6</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3639,7 +3903,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_URL_MASK = "dbSystem[X].hibernate.connection.url.mask";</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="str">
         <f>'Property-Definition'!A7</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3658,7 +3922,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_DEFAULT_CATALOG = "dbSystem[X].hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="str">
         <f>'Property-Definition'!A8</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3677,7 +3941,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_USERNAME = "dbSystem[X].hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="str">
         <f>'Property-Definition'!A9</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3696,7 +3960,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_PASSWORD = "dbSystem[X].hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="str">
         <f>'Property-Definition'!A10</f>
         <v>DB.FACTORIES</v>
@@ -3715,7 +3979,7 @@
         <v>public final static String FACTORY = "factory[X]";</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="str">
         <f>'Property-Definition'!A11</f>
         <v>DB.FACTORIES</v>
@@ -3734,7 +3998,7 @@
         <v>public final static String FACTORY_STATE = "factory[X].state";</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="str">
         <f>'Property-Definition'!A12</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -3753,7 +4017,7 @@
         <v>public final static String ISSTARTDERBYNETWORKSERVER = "isStartDerbyNetworkServer";</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="str">
         <f>'Property-Definition'!A13</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -3772,7 +4036,7 @@
         <v>public final static String HOST-IP = "host-IP";</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="str">
         <f>'Property-Definition'!A14</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -3791,7 +4055,7 @@
         <v>public final static String PORT = "port";</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="str">
         <f>'Property-Definition'!A15</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -3810,7 +4074,7 @@
         <v>public final static String USERNAME = "userName";</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="str">
         <f>'Property-Definition'!A16</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -3829,7 +4093,7 @@
         <v>public final static String PASSWORD = "password";</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="str">
         <f>'Property-Definition'!A17</f>
         <v>DB.CONN.GENERAL</v>
@@ -3848,7 +4112,7 @@
         <v>public final static String USEFOREVERYFACTORY = "useForEveryFactory";</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="str">
         <f>'Property-Definition'!A18</f>
         <v>DB.CONN.GENERAL</v>
@@ -3867,7 +4131,7 @@
         <v>public final static String DBSYSTEM = "dbSystem";</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="str">
         <f>'Property-Definition'!A19</f>
         <v>DB.CONN.GENERAL</v>
@@ -3886,7 +4150,7 @@
         <v>public final static String HIBERNATE_CONNECTION_DRIVER_CLASS = "hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="str">
         <f>'Property-Definition'!A20</f>
         <v>DB.CONN.GENERAL</v>
@@ -3905,7 +4169,7 @@
         <v>public final static String HIBERNATE_CONNECTION_URL = "hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="str">
         <f>'Property-Definition'!A21</f>
         <v>DB.CONN.GENERAL</v>
@@ -3924,7 +4188,7 @@
         <v>public final static String HIBERNATE_DEFAULT_CATALOG = "hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="str">
         <f>'Property-Definition'!A22</f>
         <v>DB.CONN.GENERAL</v>
@@ -3943,7 +4207,7 @@
         <v>public final static String HIBERNATE_CONNECTION_USERNAME = "hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="str">
         <f>'Property-Definition'!A23</f>
         <v>DB.CONN.GENERAL</v>
@@ -3962,7 +4226,7 @@
         <v>public final static String HIBERNATE_CONNECTION_PASSWORD = "hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="str">
         <f>'Property-Definition'!A24</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -3981,7 +4245,7 @@
         <v>public final static String FACTORY_FACTORYID = "factory[X].factoryID";</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="str">
         <f>'Property-Definition'!A25</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4000,7 +4264,7 @@
         <v>public final static String FACTORY_DBSYSTEM = "factory[X].dbSystem";</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="str">
         <f>'Property-Definition'!A26</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4019,7 +4283,7 @@
         <v>public final static String FACTORY_HIBERNATE_CONNECTION_DRIVER_CLASS = "factory[X].hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="str">
         <f>'Property-Definition'!A27</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4038,7 +4302,7 @@
         <v>public final static String FACTORY_HIBERNATE_CONNECTION_URL = "factory[X].hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="str">
         <f>'Property-Definition'!A28</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4057,7 +4321,7 @@
         <v>public final static String FACTORY_HIBERNATE_DEFAULT_CATALOG = "factory[X].hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="str">
         <f>'Property-Definition'!A29</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4076,7 +4340,7 @@
         <v>public final static String FACTORY_HIBERNATE_CONNECTION_USERNAME = "factory[X].hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="str">
         <f>'Property-Definition'!A30</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4095,7 +4359,7 @@
         <v>public final static String FACTORY_HIBERNATE_CONNECTION_PASSWORD = "factory[X].hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="str">
         <f>'Property-Definition'!A31</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4114,7 +4378,7 @@
         <v>public final static String FACTORYID = "factoryID";</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="str">
         <f>'Property-Definition'!A32</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4133,7 +4397,7 @@
         <v>public final static String DBSYSTEM = "dbSystem";</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="str">
         <f>'Property-Definition'!A33</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4152,7 +4416,7 @@
         <v>public final static String HIBERNATE_CONNECTION_DRIVER_CLASS = "hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="str">
         <f>'Property-Definition'!A34</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4171,7 +4435,7 @@
         <v>public final static String HIBERNATE_CONNECTION_URL = "hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="str">
         <f>'Property-Definition'!A35</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4190,7 +4454,7 @@
         <v>public final static String HIBERNATE_DEFAULT_CATALOG = "hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="str">
         <f>'Property-Definition'!A36</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4209,7 +4473,7 @@
         <v>public final static String HIBERNATE_CONNECTION_USERNAME = "hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="str">
         <f>'Property-Definition'!A37</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4228,7 +4492,7 @@
         <v>public final static String HIBERNATE_CONNECTION_PASSWORD = "hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="str">
         <f>'Property-Definition'!A38</f>
         <v>DB.CONN.TEST</v>
@@ -4247,7 +4511,7 @@
         <v>public final static String DBSYSTEM = "dbSystem";</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="str">
         <f>'Property-Definition'!A39</f>
         <v>DB.CONN.TEST</v>
@@ -4266,7 +4530,7 @@
         <v>public final static String HIBERNATE_CONNECTION_DRIVER_CLASS = "hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="str">
         <f>'Property-Definition'!A40</f>
         <v>DB.CONN.TEST</v>
@@ -4285,7 +4549,7 @@
         <v>public final static String HIBERNATE_CONNECTION_URL = "hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="str">
         <f>'Property-Definition'!A41</f>
         <v>DB.CONN.TEST</v>
@@ -4304,7 +4568,7 @@
         <v>public final static String HIBERNATE_DEFAULT_CATALOG = "hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="str">
         <f>'Property-Definition'!A42</f>
         <v>DB.CONN.TEST</v>
@@ -4323,7 +4587,7 @@
         <v>public final static String HIBERNATE_CONNECTION_USERNAME = "hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="str">
         <f>'Property-Definition'!A43</f>
         <v>DB.CONN.TEST</v>
@@ -4342,7 +4606,7 @@
         <v>public final static String HIBERNATE_CONNECTION_PASSWORD = "hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="str">
         <f>'Property-Definition'!A44</f>
         <v>EXEC.MODE</v>
@@ -4361,7 +4625,7 @@
         <v>public final static String EXEC_MODE = "exec.mode";</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="str">
         <f>'Property-Definition'!A45</f>
         <v>EXEC.MODE</v>
@@ -4380,7 +4644,7 @@
         <v>public final static String SERVER_MASTER_URL = "server.master.url";</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="str">
         <f>'Property-Definition'!A46</f>
         <v>EXEC.MODE</v>
@@ -4399,7 +4663,7 @@
         <v>public final static String SERVER_MASTER_PORT = "server.master.port";</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="str">
         <f>'Property-Definition'!A47</f>
         <v>EXEC.MODE</v>
@@ -4418,7 +4682,7 @@
         <v>public final static String SERVER_MASTER_PORT_MTP = "server.master.port.mtp";</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="str">
         <f>'Property-Definition'!A48</f>
         <v>EXEC.MODE</v>
@@ -4437,7 +4701,7 @@
         <v>public final static String SERVER_MASTER_PROTOCOL = "server.master.protocol";</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="str">
         <f>'Property-Definition'!A49</f>
         <v>EXEC.MODE</v>
@@ -4456,7 +4720,7 @@
         <v>public final static String LOCAL_MTP_CREATION = "local.mtp.creation";</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="str">
         <f>'Property-Definition'!A50</f>
         <v>EXEC.MODE</v>
@@ -4475,7 +4739,7 @@
         <v>public final static String LOCAL_MTP_URL = "local.mtp.url";</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="str">
         <f>'Property-Definition'!A51</f>
         <v>EXEC.MODE</v>
@@ -4494,7 +4758,7 @@
         <v>public final static String LOCAL_MTP_PORT = "local.mtp.port";</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" t="str">
         <f>'Property-Definition'!A52</f>
         <v>EXEC.MODE</v>
@@ -4513,7 +4777,7 @@
         <v>public final static String LOCAL_MTP_PROTOCOL = "local.mtp.protocol";</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" t="str">
         <f>'Property-Definition'!A53</f>
         <v>EXEC.MODE</v>
@@ -4532,7 +4796,7 @@
         <v>public final static String EMBEDDEDSYSTEM_PROJECT = "embeddedsystem.project";</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" t="str">
         <f>'Property-Definition'!A54</f>
         <v>EXEC.MODE</v>
@@ -4551,7 +4815,7 @@
         <v>public final static String DEVICE_SYSTEM_EXEC_MODE = "device_system_exec_mode";</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="str">
         <f>'Property-Definition'!A55</f>
         <v>EXEC.MODE</v>
@@ -4570,7 +4834,7 @@
         <v>public final static String EMBEDDEDSYSTEM_AGENT_CLASSNAME = "embeddedsystem.agent[X].classname";</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" t="str">
         <f>'Property-Definition'!A56</f>
         <v>EXEC.MODE</v>
@@ -4589,7 +4853,7 @@
         <v>public final static String EMBEDDEDSYSTEM_AGENT_AGENTNAME = "embeddedsystem.agent[X].agentname";</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="str">
         <f>'Property-Definition'!A57</f>
         <v>EXEC.MODE</v>
@@ -4608,7 +4872,7 @@
         <v>public final static String SERVICE_SERVICE_SETUP = "service.service_setup";</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" t="str">
         <f>'Property-Definition'!A58</f>
         <v>EXEC.MODE</v>
@@ -4627,7 +4891,7 @@
         <v>public final static String LOCAL_IP_SELECTION = "local.ip.selection[X]";</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" t="str">
         <f>'Property-Definition'!A59</f>
         <v>EXEC.MODE</v>
@@ -4646,7 +4910,7 @@
         <v>public final static String FACTORY_ID = "factory_id";</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" t="e">
         <f>'Property-Definition'!#REF!</f>
         <v>#REF!</v>
@@ -4665,7 +4929,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" t="str">
         <f>'Property-Definition'!A60</f>
         <v>AWB.AGENTS</v>
@@ -4684,7 +4948,7 @@
         <v>public final static String AGENT_CLASSNAME = "agent[X].classname";</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" t="str">
         <f>'Property-Definition'!A61</f>
         <v>PROJECTS</v>
@@ -4703,7 +4967,7 @@
         <v>public final static String PROJECT = "project[X]";</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" t="str">
         <f>'Property-Definition'!A62</f>
         <v>PROJECT.SETUPS[X]</v>
@@ -4722,7 +4986,7 @@
         <v>public final static String PROJECT_SETUP = "project[X].setup[X]";</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A64" t="str">
         <f>'Property-Definition'!A63</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4741,7 +5005,7 @@
         <v>public final static String BGPLATFORM_CONTACTAGENT = "bgplatform[X].contactagent";</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" t="str">
         <f>'Property-Definition'!A60</f>
         <v>AWB.AGENTS</v>
@@ -4760,7 +5024,7 @@
         <v>public final static String BGPLATFORM_PLATFORMNAME = "bgplatform[X].platformname";</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" t="str">
         <f>'Property-Definition'!A61</f>
         <v>PROJECTS</v>
@@ -4779,7 +5043,7 @@
         <v>public final static String BGPLATFORM_SERVER = "bgplatform[X].server";</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" t="str">
         <f>'Property-Definition'!A62</f>
         <v>PROJECT.SETUPS[X]</v>
@@ -4798,7 +5062,7 @@
         <v>public final static String BGPLATFORM_IPADDRESS = "bgplatform[X].ipaddress";</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" t="str">
         <f>'Property-Definition'!A67</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4817,7 +5081,7 @@
         <v>public final static String BGPLATFORM_URL = "bgplatform[X].url";</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69" t="str">
         <f>'Property-Definition'!A68</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4836,7 +5100,7 @@
         <v>public final static String BGPLATFORM_JADEPORT = "bgplatform[X].jadeport";</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" t="str">
         <f>'Property-Definition'!A69</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4855,7 +5119,7 @@
         <v>public final static String BGPLATFORM_HTTPMTP = "bgplatform[X].httpmtp";</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71" t="str">
         <f>'Property-Definition'!A70</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4874,7 +5138,7 @@
         <v>public final static String BGPLATFORM_VERSIONMAJOR = "bgplatform[X].versionmajor";</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72" t="str">
         <f>'Property-Definition'!A71</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4893,7 +5157,7 @@
         <v>public final static String BGPLATFORM_VERSIONMINOR = "bgplatform[X].versionminor";</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A73" t="str">
         <f>'Property-Definition'!A72</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4912,7 +5176,7 @@
         <v>public final static String BGPLATFORM_VERSIONMICRO = "bgplatform[X].versionmicro";</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A74" t="str">
         <f>'Property-Definition'!A73</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4931,7 +5195,7 @@
         <v>public final static String BGPLATFORM_VERSIONBUILD = "bgplatform[X].versionbuild";</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A75" t="str">
         <f>'Property-Definition'!A74</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4950,7 +5214,7 @@
         <v>public final static String BGPLATFORM_OS_NAME = "bgplatform[X].os.name";</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A76" t="str">
         <f>'Property-Definition'!A75</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4969,7 +5233,7 @@
         <v>public final static String BGPLATFORM_OS_VERSION = "bgplatform[X].os.version";</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A77" t="str">
         <f>'Property-Definition'!A76</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -4988,7 +5252,7 @@
         <v>public final static String BGPLATFORM_OS_ARCHITECTURE = "bgplatform[X].os.architecture";</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A78" t="str">
         <f>'Property-Definition'!A77</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5007,7 +5271,7 @@
         <v>public final static String BGPLATFORM_CPU_NAME = "bgplatform[X].cpu.name";</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A79" t="str">
         <f>'Property-Definition'!A78</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5026,7 +5290,7 @@
         <v>public final static String BGPLATFORM_CPU_NUMLOGICAL = "bgplatform[X].cpu.numlogical";</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A80" t="str">
         <f>'Property-Definition'!A79</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5045,7 +5309,7 @@
         <v>public final static String BGPLATFORM_CPU_NUMPHYSICAL = "bgplatform[X].cpu.numphysical";</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A81" t="str">
         <f>'Property-Definition'!A80</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5064,7 +5328,7 @@
         <v>public final static String BGPLATFORM_CPU_SPEEDMHZ = "bgplatform[X].cpu.speedmhz";</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A82" t="str">
         <f>'Property-Definition'!A81</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5083,7 +5347,7 @@
         <v>public final static String BGPLATFORM_MEMORYMB = "bgplatform[X].memorymb";</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A83" t="str">
         <f>'Property-Definition'!A82</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5102,7 +5366,7 @@
         <v>public final static String BGPLATFORM_BENCHMARKVALUE = "bgplatform[X].benchmarkvalue";</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A84" t="str">
         <f>'Property-Definition'!A83</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5121,7 +5385,7 @@
         <v>public final static String BGPLATFORM_TIME_ONLINESINCE = "bgplatform[X].time.onlinesince";</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A85" t="str">
         <f>'Property-Definition'!A84</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5140,7 +5404,7 @@
         <v>public final static String BGPLATFORM_TIME_LASTCONTACT = "bgplatform[X].time.lastcontact";</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A86" t="str">
         <f>'Property-Definition'!A85</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5159,7 +5423,7 @@
         <v>public final static String BGPLATFORM_LOCALTIME_ONLINESINCE = "bgplatform[X].localtime.onlinesince";</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A87" t="str">
         <f>'Property-Definition'!A86</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5178,7 +5442,7 @@
         <v>public final static String BGPLATFORM_LOCALTIME_LASTCONTACT = "bgplatform[X].localtime.lastcontact";</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A88" t="str">
         <f>'Property-Definition'!A87</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5197,7 +5461,7 @@
         <v>public final static String BGPLATFORM_CURRENTLYAVAILABLE = "bgplatform[X].currentlyavailable";</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A89" t="str">
         <f>'Property-Definition'!A88</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5216,7 +5480,7 @@
         <v>public final static String BGPLATFORM_CURRENT_CPULOAD = "bgplatform[X].current.cpuload";</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A90" t="str">
         <f>'Property-Definition'!A89</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5235,7 +5499,7 @@
         <v>public final static String BGPLATFORM_CURRENT_MEMORYLOAD = "bgplatform[X].current.memoryload";</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A91" t="str">
         <f>'Property-Definition'!A90</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5254,7 +5518,7 @@
         <v>public final static String BGPLATFORM_CURRENT_MEMORYLOADJVM = "bgplatform[X].current.memoryloadjvm";</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A92" t="str">
         <f>'Property-Definition'!A91</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5273,7 +5537,7 @@
         <v>public final static String BGPLATFORM_CURRENT_NUMTHREADS = "bgplatform[X].current.numthreads";</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A93" t="str">
         <f>'Property-Definition'!A92</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5290,6 +5554,243 @@
 &amp; CHAR(34)
 &amp; ";"</f>
         <v>public final static String BGPLATFORM_CURRENT_THRESHOLDEXCEEDED = "bgplatform[X].current.thresholdexceeded";</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A94" t="str">
+        <f>'Property-Definition'!A93</f>
+        <v>UPDATE.STRATEGY</v>
+      </c>
+      <c r="B94" t="str">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D93,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D93
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String ISAUTOUPDATE = "isautoupdate";</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A95" t="str">
+        <f>'Property-Definition'!A94</f>
+        <v>UPDATE.BACKEND.CHECK[isForceCheck]</v>
+      </c>
+      <c r="B95" t="str">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D94,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D94
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String UPDATECHECK_BACKEND_ISPENDING = "updatecheck.backend.ispending";</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A96" t="str">
+        <f>'Property-Definition'!A95</f>
+        <v>UPDATE.BACKEND.CHECK[isForceCheck]</v>
+      </c>
+      <c r="B96" t="str">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D95,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D95
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String UPDATECHECK_BACKEND_ISAVAILABLE = "updatecheck.backend.isavailable";</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A97" t="str">
+        <f>'Property-Definition'!A96</f>
+        <v>UPDATE.BACKEND.CHECK[isForceCheck]</v>
+      </c>
+      <c r="B97" t="str">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D96,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D96
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String UPDATECHECK_BACKEND_LASTCHECK = "updatecheck.backend.lastcheck";</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A98" t="str">
+        <f>'Property-Definition'!A97</f>
+        <v>UPDATE.BACKEND.CHECK[isForceCheck]</v>
+      </c>
+      <c r="B98" t="str">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D97,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D97
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String UPDATECHECK_BACKEND_VERSION = "updatecheck.backend.version";</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A99" t="str">
+        <f>'Property-Definition'!A102</f>
+        <v>UPDATE.FRONTEND.CHECK</v>
+      </c>
+      <c r="B99" t="str">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D102,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D102
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String UPDATECHECK_FRONTEND_ISPENDING = "updatecheck.frontend.ispending";</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A100" t="str">
+        <f>'Property-Definition'!A103</f>
+        <v>UPDATE.FRONTEND.CHECK</v>
+      </c>
+      <c r="B100" t="str">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D103,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D103
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String UPDATECHECK_FRONTEND_ISAVAILABLE = "updatecheck.frontend.isavailable";</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A101" t="str">
+        <f>'Property-Definition'!A104</f>
+        <v>UPDATE.FRONTEND.CHECK</v>
+      </c>
+      <c r="B101" t="str">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D104,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D104
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String UPDATECHECK_FRONTEND_LASTCHECK = "updatecheck.frontend.lastcheck";</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A102" t="str">
+        <f>'Property-Definition'!A105</f>
+        <v>UPDATE.FRONTEND.CHECK</v>
+      </c>
+      <c r="B102" t="str">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!D105,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D105
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>public final static String UPDATECHECK_FRONTEND_VERSION = "updatecheck.frontend.version";</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A103">
+        <f>'Property-Definition'!A106</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A104">
+        <f>'Property-Definition'!A107</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A105">
+        <f>'Property-Definition'!A108</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A106">
+        <f>'Property-Definition'!A109</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A107">
+        <f>'Property-Definition'!A110</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A108">
+        <f>'Property-Definition'!A111</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A109">
+        <f>'Property-Definition'!A112</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A110">
+        <f>'Property-Definition'!A113</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A111">
+        <f>'Property-Definition'!A114</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A112">
+        <f>'Property-Definition'!A115</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A113">
+        <f>'Property-Definition'!A116</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Rest Api Property Dictionary.
</commit_message>
<xml_diff>
--- a/AWB-RestApi-PropertyDictionary.xlsx
+++ b/AWB-RestApi-PropertyDictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\AgentWorkbench\eclipseProjects\de.enflexit.awb\bundles\web\xApi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87407461-A88A-427E-8DD0-874977FBD40F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF9CB0FA-9096-4FD0-8AB9-0888F130364F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="828" uniqueCount="214">
   <si>
     <t>key</t>
   </si>
@@ -642,9 +642,6 @@
     <t>updatecheck.backend.lastcheck</t>
   </si>
   <si>
-    <t>updatecheck.backend.version</t>
-  </si>
-  <si>
     <t>updatecheck.frontend.version</t>
   </si>
   <si>
@@ -657,9 +654,6 @@
     <t>de.enflexit.awb.ws.core</t>
   </si>
   <si>
-    <t>UPDATE.FRONTEND.CHECK</t>
-  </si>
-  <si>
     <t>updatecheck.frontend.ispending</t>
   </si>
   <si>
@@ -685,6 +679,9 @@
   </si>
   <si>
     <t>e.g. 'Pending', 'no update available', 'update finalized'</t>
+  </si>
+  <si>
+    <t>UPDATE.FRONTEND.CHECK[isForceCheck]</t>
   </si>
 </sst>
 </file>
@@ -1064,7 +1061,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K105"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34.36328125" bestFit="1" customWidth="1"/>
@@ -3558,7 +3555,7 @@
         <v>21</v>
       </c>
       <c r="H93" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="I93" s="5" t="s">
         <v>59</v>
@@ -3566,10 +3563,10 @@
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B94" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C94" t="s">
         <v>5</v>
@@ -3592,10 +3589,10 @@
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B95" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C95" t="s">
         <v>5</v>
@@ -3618,10 +3615,10 @@
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B96" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C96" t="s">
         <v>5</v>
@@ -3633,7 +3630,7 @@
         <v>7</v>
       </c>
       <c r="F96" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H96" t="s">
         <v>136</v>
@@ -3642,72 +3639,75 @@
         <v>59</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>207</v>
-      </c>
-      <c r="B97" t="s">
         <v>208</v>
       </c>
       <c r="C97" t="s">
         <v>5</v>
       </c>
       <c r="D97" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E97" t="s">
         <v>7</v>
       </c>
-      <c r="H97" t="s">
-        <v>136</v>
-      </c>
-      <c r="I97" s="5" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="F97" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C98" t="s">
         <v>5</v>
       </c>
       <c r="D98" t="s">
+        <v>209</v>
+      </c>
+      <c r="E98" t="s">
+        <v>26</v>
+      </c>
+      <c r="F98" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
         <v>213</v>
       </c>
-      <c r="E98" t="s">
-        <v>7</v>
-      </c>
-      <c r="F98" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A99" t="s">
-        <v>210</v>
-      </c>
-      <c r="C99" t="s">
+      <c r="B101" t="s">
+        <v>206</v>
+      </c>
+      <c r="C101" t="s">
         <v>5</v>
       </c>
-      <c r="D99" t="s">
-        <v>211</v>
-      </c>
-      <c r="E99" t="s">
-        <v>26</v>
-      </c>
-      <c r="F99" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D101" t="s">
+        <v>204</v>
+      </c>
+      <c r="E101" t="s">
+        <v>20</v>
+      </c>
+      <c r="F101" t="s">
+        <v>21</v>
+      </c>
+      <c r="H101" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
-        <v>205</v>
+        <v>213</v>
+      </c>
+      <c r="B102" t="s">
+        <v>206</v>
       </c>
       <c r="C102" t="s">
         <v>5</v>
       </c>
       <c r="D102" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="E102" t="s">
         <v>20</v>
@@ -3716,12 +3716,15 @@
         <v>21</v>
       </c>
       <c r="H102" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.35">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
-        <v>205</v>
+        <v>213</v>
+      </c>
+      <c r="B103" t="s">
+        <v>206</v>
       </c>
       <c r="C103" t="s">
         <v>5</v>
@@ -3730,51 +3733,37 @@
         <v>202</v>
       </c>
       <c r="E103" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="F103" t="s">
-        <v>21</v>
+        <v>207</v>
       </c>
       <c r="H103" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.35">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
-        <v>205</v>
+        <v>213</v>
+      </c>
+      <c r="B104" t="s">
+        <v>206</v>
       </c>
       <c r="C104" t="s">
         <v>5</v>
       </c>
       <c r="D104" t="s">
+        <v>200</v>
+      </c>
+      <c r="E104" t="s">
+        <v>7</v>
+      </c>
+      <c r="H104" t="s">
         <v>203</v>
       </c>
-      <c r="E104" t="s">
-        <v>7</v>
-      </c>
-      <c r="H104" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A105" t="s">
-        <v>205</v>
-      </c>
-      <c r="C105" t="s">
-        <v>5</v>
-      </c>
-      <c r="D105" t="s">
-        <v>201</v>
-      </c>
-      <c r="E105" t="s">
-        <v>7</v>
-      </c>
-      <c r="H105" t="s">
-        <v>204</v>
-      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:J43 J44:J92 I44:I101">
+  <conditionalFormatting sqref="I2:J43 J44:J92 I44:I100">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>
@@ -5633,38 +5622,38 @@
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A98" t="str">
-        <f>'Property-Definition'!A97</f>
-        <v>UPDATE.BACKEND.CHECK[isForceCheck]</v>
-      </c>
-      <c r="B98" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D97,"[X]",""),".","_")
-)
-&amp; " = "
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D97
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String UPDATECHECK_BACKEND_VERSION = "updatecheck.backend.version";</v>
+      <c r="A98" t="e">
+        <f>'Property-Definition'!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="B98" t="e">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!#REF!,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!#REF!
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A99" t="str">
-        <f>'Property-Definition'!A102</f>
-        <v>UPDATE.FRONTEND.CHECK</v>
+        <f>'Property-Definition'!A101</f>
+        <v>UPDATE.FRONTEND.CHECK[isForceCheck]</v>
       </c>
       <c r="B99" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D102,"[X]",""),".","_")
-)
-&amp; " = "
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D102
+        SUBSTITUTE('Property-Definition'!D101,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D101
 &amp; CHAR(34)
 &amp; ";"</f>
         <v>public final static String UPDATECHECK_FRONTEND_ISPENDING = "updatecheck.frontend.ispending";</v>
@@ -5672,18 +5661,18 @@
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A100" t="str">
-        <f>'Property-Definition'!A103</f>
-        <v>UPDATE.FRONTEND.CHECK</v>
+        <f>'Property-Definition'!A102</f>
+        <v>UPDATE.FRONTEND.CHECK[isForceCheck]</v>
       </c>
       <c r="B100" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D103,"[X]",""),".","_")
-)
-&amp; " = "
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D103
+        SUBSTITUTE('Property-Definition'!D102,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D102
 &amp; CHAR(34)
 &amp; ";"</f>
         <v>public final static String UPDATECHECK_FRONTEND_ISAVAILABLE = "updatecheck.frontend.isavailable";</v>
@@ -5691,18 +5680,18 @@
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A101" t="str">
-        <f>'Property-Definition'!A104</f>
-        <v>UPDATE.FRONTEND.CHECK</v>
+        <f>'Property-Definition'!A103</f>
+        <v>UPDATE.FRONTEND.CHECK[isForceCheck]</v>
       </c>
       <c r="B101" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D104,"[X]",""),".","_")
-)
-&amp; " = "
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D104
+        SUBSTITUTE('Property-Definition'!D103,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D103
 &amp; CHAR(34)
 &amp; ";"</f>
         <v>public final static String UPDATECHECK_FRONTEND_LASTCHECK = "updatecheck.frontend.lastcheck";</v>
@@ -5710,18 +5699,18 @@
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A102" t="str">
-        <f>'Property-Definition'!A105</f>
-        <v>UPDATE.FRONTEND.CHECK</v>
+        <f>'Property-Definition'!A104</f>
+        <v>UPDATE.FRONTEND.CHECK[isForceCheck]</v>
       </c>
       <c r="B102" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D105,"[X]",""),".","_")
-)
-&amp; " = "
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D105
+        SUBSTITUTE('Property-Definition'!D104,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D104
 &amp; CHAR(34)
 &amp; ";"</f>
         <v>public final static String UPDATECHECK_FRONTEND_VERSION = "updatecheck.frontend.version";</v>
@@ -5729,67 +5718,67 @@
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A103">
+        <f>'Property-Definition'!A105</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A104">
         <f>'Property-Definition'!A106</f>
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A104">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A105">
         <f>'Property-Definition'!A107</f>
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A105">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A106">
         <f>'Property-Definition'!A108</f>
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A106">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A107">
         <f>'Property-Definition'!A109</f>
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A107">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A108">
         <f>'Property-Definition'!A110</f>
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A108">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A109">
         <f>'Property-Definition'!A111</f>
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A109">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A110">
         <f>'Property-Definition'!A112</f>
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A110">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A111">
         <f>'Property-Definition'!A113</f>
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A111">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A112">
         <f>'Property-Definition'!A114</f>
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A112">
-        <f>'Property-Definition'!A115</f>
-        <v>0</v>
-      </c>
-    </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A113">
-        <f>'Property-Definition'!A116</f>
+        <f>'Property-Definition'!A115</f>
         <v>0</v>
       </c>
     </row>
@@ -5800,15 +5789,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101004FB79D76D905EB41B4AD64ED4839597F" ma:contentTypeVersion="11" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="0622d98e252eab518d4b54f931ba6851">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="897f6830-f425-409d-b8f5-ce1019056d9e" xmlns:ns3="f2404b4d-361b-46d3-b2ec-035eed29e274" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dd5f302b3846fd12003b89c8f5b7df36" ns2:_="" ns3:_="">
     <xsd:import namespace="897f6830-f425-409d-b8f5-ce1019056d9e"/>
@@ -6003,6 +5983,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -6015,14 +6004,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A33EE264-283E-4F19-BA61-B3264EA417E2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6041,6 +6022,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF16440F-B0E0-4269-97EE-BEB05B0223C8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Small changes in yaml and excel file
</commit_message>
<xml_diff>
--- a/AWB-RestApi-PropertyDictionary.xlsx
+++ b/AWB-RestApi-PropertyDictionary.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\AgentWorkbench\eclipseProjects\de.enflexit.awb\bundles\web\xApi\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\20_GIT\01_AWB\eclipseProjects\de.enflexit.awb\bundles\web\xAPI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87407461-A88A-427E-8DD0-874977FBD40F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEBEBDFB-365B-452A-9537-E1EB30312A98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="838" uniqueCount="217">
   <si>
     <t>key</t>
   </si>
@@ -684,7 +684,13 @@
     <t>update.status</t>
   </si>
   <si>
-    <t>e.g. 'Pending', 'no update available', 'update finalized'</t>
+    <t>update.message</t>
+  </si>
+  <si>
+    <t>e.g. 'Currently instaling ….'</t>
+  </si>
+  <si>
+    <t>e.g. 'Pending', 'Done', 'Error'</t>
   </si>
 </sst>
 </file>
@@ -3679,7 +3685,10 @@
         <v>7</v>
       </c>
       <c r="F98" t="s">
-        <v>214</v>
+        <v>216</v>
+      </c>
+      <c r="H98" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.35">
@@ -3698,6 +3707,29 @@
       <c r="F99" t="s">
         <v>212</v>
       </c>
+      <c r="H99" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
+        <v>210</v>
+      </c>
+      <c r="C100" t="s">
+        <v>5</v>
+      </c>
+      <c r="D100" t="s">
+        <v>214</v>
+      </c>
+      <c r="E100" t="s">
+        <v>7</v>
+      </c>
+      <c r="F100" t="s">
+        <v>215</v>
+      </c>
+      <c r="H100" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
@@ -3774,7 +3806,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:J43 J44:J92 I44:I101">
+  <conditionalFormatting sqref="I2:J43 J44:J92 I44:I105">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>
@@ -5800,15 +5832,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101004FB79D76D905EB41B4AD64ED4839597F" ma:contentTypeVersion="11" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="0622d98e252eab518d4b54f931ba6851">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="897f6830-f425-409d-b8f5-ce1019056d9e" xmlns:ns3="f2404b4d-361b-46d3-b2ec-035eed29e274" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dd5f302b3846fd12003b89c8f5b7df36" ns2:_="" ns3:_="">
     <xsd:import namespace="897f6830-f425-409d-b8f5-ce1019056d9e"/>
@@ -6003,6 +6026,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -6015,14 +6047,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A33EE264-283E-4F19-BA61-B3264EA417E2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6041,6 +6065,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF16440F-B0E0-4269-97EE-BEB05B0223C8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Restored changes to dictionary after conflict.
</commit_message>
<xml_diff>
--- a/AWB-RestApi-PropertyDictionary.xlsx
+++ b/AWB-RestApi-PropertyDictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\20_GIT\01_AWB\eclipseProjects\de.enflexit.awb\bundles\web\xAPI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\AgentWorkbench\eclipseProjects\de.enflexit.awb\bundles\web\xApi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEBEBDFB-365B-452A-9537-E1EB30312A98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69B6CA9F-8F9F-4B90-9056-8C6E7F94CBA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3800" yWindow="3800" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Property-Definition" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="838" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="217">
   <si>
     <t>key</t>
   </si>
@@ -642,9 +642,6 @@
     <t>updatecheck.backend.lastcheck</t>
   </si>
   <si>
-    <t>updatecheck.backend.version</t>
-  </si>
-  <si>
     <t>updatecheck.frontend.version</t>
   </si>
   <si>
@@ -657,9 +654,6 @@
     <t>de.enflexit.awb.ws.core</t>
   </si>
   <si>
-    <t>UPDATE.FRONTEND.CHECK</t>
-  </si>
-  <si>
     <t>updatecheck.frontend.ispending</t>
   </si>
   <si>
@@ -691,6 +685,12 @@
   </si>
   <si>
     <t>e.g. 'Pending', 'Done', 'Error'</t>
+  </si>
+  <si>
+    <t>UPDATE.FRONTEND.CHECK[isForceCheck]</t>
+  </si>
+  <si>
+    <t>e.g. '0.0.4.20260602-1140'</t>
   </si>
 </sst>
 </file>
@@ -1070,7 +1070,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K105"/>
+  <dimension ref="A1:K103"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34.36328125" bestFit="1" customWidth="1"/>
@@ -3564,7 +3564,7 @@
         <v>21</v>
       </c>
       <c r="H93" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="I93" s="5" t="s">
         <v>59</v>
@@ -3572,10 +3572,10 @@
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B94" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C94" t="s">
         <v>5</v>
@@ -3598,10 +3598,10 @@
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B95" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C95" t="s">
         <v>5</v>
@@ -3624,10 +3624,10 @@
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B96" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C96" t="s">
         <v>5</v>
@@ -3639,7 +3639,7 @@
         <v>7</v>
       </c>
       <c r="F96" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H96" t="s">
         <v>136</v>
@@ -3650,19 +3650,19 @@
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>207</v>
-      </c>
-      <c r="B97" t="s">
         <v>208</v>
       </c>
       <c r="C97" t="s">
         <v>5</v>
       </c>
       <c r="D97" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E97" t="s">
         <v>7</v>
+      </c>
+      <c r="F97" t="s">
+        <v>214</v>
       </c>
       <c r="H97" t="s">
         <v>136</v>
@@ -3673,140 +3673,156 @@
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C98" t="s">
         <v>5</v>
       </c>
       <c r="D98" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="E98" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="F98" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="H98" t="s">
         <v>136</v>
       </c>
+      <c r="I98" s="5" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C99" t="s">
         <v>5</v>
       </c>
       <c r="D99" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E99" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="F99" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H99" t="s">
         <v>136</v>
       </c>
+      <c r="I99" s="5" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>210</v>
+        <v>215</v>
+      </c>
+      <c r="B100" t="s">
+        <v>206</v>
       </c>
       <c r="C100" t="s">
         <v>5</v>
       </c>
       <c r="D100" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="E100" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="F100" t="s">
+        <v>21</v>
+      </c>
+      <c r="H100" t="s">
+        <v>203</v>
+      </c>
+      <c r="I100" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
         <v>215</v>
       </c>
-      <c r="H100" t="s">
-        <v>136</v>
+      <c r="B101" t="s">
+        <v>206</v>
+      </c>
+      <c r="C101" t="s">
+        <v>5</v>
+      </c>
+      <c r="D101" t="s">
+        <v>201</v>
+      </c>
+      <c r="E101" t="s">
+        <v>20</v>
+      </c>
+      <c r="F101" t="s">
+        <v>21</v>
+      </c>
+      <c r="H101" t="s">
+        <v>203</v>
+      </c>
+      <c r="I101" s="5" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
-        <v>205</v>
+        <v>215</v>
+      </c>
+      <c r="B102" t="s">
+        <v>206</v>
       </c>
       <c r="C102" t="s">
         <v>5</v>
       </c>
       <c r="D102" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="E102" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="F102" t="s">
-        <v>21</v>
+        <v>207</v>
       </c>
       <c r="H102" t="s">
-        <v>204</v>
+        <v>203</v>
+      </c>
+      <c r="I102" s="5" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
-        <v>205</v>
+        <v>215</v>
+      </c>
+      <c r="B103" t="s">
+        <v>206</v>
       </c>
       <c r="C103" t="s">
         <v>5</v>
       </c>
       <c r="D103" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="E103" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="F103" t="s">
-        <v>21</v>
+        <v>216</v>
       </c>
       <c r="H103" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A104" t="s">
-        <v>205</v>
-      </c>
-      <c r="C104" t="s">
-        <v>5</v>
-      </c>
-      <c r="D104" t="s">
         <v>203</v>
       </c>
-      <c r="E104" t="s">
-        <v>7</v>
-      </c>
-      <c r="H104" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A105" t="s">
-        <v>205</v>
-      </c>
-      <c r="C105" t="s">
-        <v>5</v>
-      </c>
-      <c r="D105" t="s">
-        <v>201</v>
-      </c>
-      <c r="E105" t="s">
-        <v>7</v>
-      </c>
-      <c r="H105" t="s">
-        <v>204</v>
+      <c r="I103" s="5" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:J43 J44:J92 I44:I105">
+  <conditionalFormatting sqref="I2:J43 J44:J92 I44:I103">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>
@@ -5665,38 +5681,38 @@
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A98" t="str">
-        <f>'Property-Definition'!A97</f>
-        <v>UPDATE.BACKEND.CHECK[isForceCheck]</v>
-      </c>
-      <c r="B98" t="str">
-        <f>"public final static String "
-&amp; UPPER(
-    SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D97,"[X]",""),".","_")
-)
-&amp; " = "
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D97
-&amp; CHAR(34)
-&amp; ";"</f>
-        <v>public final static String UPDATECHECK_BACKEND_VERSION = "updatecheck.backend.version";</v>
+      <c r="A98" t="e">
+        <f>'Property-Definition'!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="B98" t="e">
+        <f>"public final static String "
+&amp; UPPER(
+    SUBSTITUTE(
+        SUBSTITUTE('Property-Definition'!#REF!,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!#REF!
+&amp; CHAR(34)
+&amp; ";"</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A99" t="str">
-        <f>'Property-Definition'!A102</f>
-        <v>UPDATE.FRONTEND.CHECK</v>
+        <f>'Property-Definition'!A100</f>
+        <v>UPDATE.FRONTEND.CHECK[isForceCheck]</v>
       </c>
       <c r="B99" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D102,"[X]",""),".","_")
-)
-&amp; " = "
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D102
+        SUBSTITUTE('Property-Definition'!D100,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D100
 &amp; CHAR(34)
 &amp; ";"</f>
         <v>public final static String UPDATECHECK_FRONTEND_ISPENDING = "updatecheck.frontend.ispending";</v>
@@ -5704,18 +5720,18 @@
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A100" t="str">
-        <f>'Property-Definition'!A103</f>
-        <v>UPDATE.FRONTEND.CHECK</v>
+        <f>'Property-Definition'!A101</f>
+        <v>UPDATE.FRONTEND.CHECK[isForceCheck]</v>
       </c>
       <c r="B100" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D103,"[X]",""),".","_")
-)
-&amp; " = "
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D103
+        SUBSTITUTE('Property-Definition'!D101,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D101
 &amp; CHAR(34)
 &amp; ";"</f>
         <v>public final static String UPDATECHECK_FRONTEND_ISAVAILABLE = "updatecheck.frontend.isavailable";</v>
@@ -5723,18 +5739,18 @@
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A101" t="str">
-        <f>'Property-Definition'!A104</f>
-        <v>UPDATE.FRONTEND.CHECK</v>
+        <f>'Property-Definition'!A102</f>
+        <v>UPDATE.FRONTEND.CHECK[isForceCheck]</v>
       </c>
       <c r="B101" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D104,"[X]",""),".","_")
-)
-&amp; " = "
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D104
+        SUBSTITUTE('Property-Definition'!D102,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D102
 &amp; CHAR(34)
 &amp; ";"</f>
         <v>public final static String UPDATECHECK_FRONTEND_LASTCHECK = "updatecheck.frontend.lastcheck";</v>
@@ -5742,18 +5758,18 @@
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A102" t="str">
-        <f>'Property-Definition'!A105</f>
-        <v>UPDATE.FRONTEND.CHECK</v>
+        <f>'Property-Definition'!A103</f>
+        <v>UPDATE.FRONTEND.CHECK[isForceCheck]</v>
       </c>
       <c r="B102" t="str">
         <f>"public final static String "
 &amp; UPPER(
     SUBSTITUTE(
-        SUBSTITUTE('Property-Definition'!D105,"[X]",""),".","_")
-)
-&amp; " = "
-&amp; CHAR(34)
-&amp; 'Property-Definition'!D105
+        SUBSTITUTE('Property-Definition'!D103,"[X]",""),".","_")
+)
+&amp; " = "
+&amp; CHAR(34)
+&amp; 'Property-Definition'!D103
 &amp; CHAR(34)
 &amp; ";"</f>
         <v>public final static String UPDATECHECK_FRONTEND_VERSION = "updatecheck.frontend.version";</v>
@@ -5761,67 +5777,67 @@
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A103">
+        <f>'Property-Definition'!A104</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A104">
+        <f>'Property-Definition'!A105</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A105">
         <f>'Property-Definition'!A106</f>
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A104">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A106">
         <f>'Property-Definition'!A107</f>
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A105">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A107">
         <f>'Property-Definition'!A108</f>
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A106">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A108">
         <f>'Property-Definition'!A109</f>
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A107">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A109">
         <f>'Property-Definition'!A110</f>
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A108">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A110">
         <f>'Property-Definition'!A111</f>
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A109">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A111">
         <f>'Property-Definition'!A112</f>
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A110">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A112">
         <f>'Property-Definition'!A113</f>
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A111">
-        <f>'Property-Definition'!A114</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A112">
-        <f>'Property-Definition'!A115</f>
-        <v>0</v>
-      </c>
-    </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A113">
-        <f>'Property-Definition'!A116</f>
+        <f>'Property-Definition'!A114</f>
         <v>0</v>
       </c>
     </row>
@@ -5832,6 +5848,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101004FB79D76D905EB41B4AD64ED4839597F" ma:contentTypeVersion="11" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="0622d98e252eab518d4b54f931ba6851">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="897f6830-f425-409d-b8f5-ce1019056d9e" xmlns:ns3="f2404b4d-361b-46d3-b2ec-035eed29e274" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dd5f302b3846fd12003b89c8f5b7df36" ns2:_="" ns3:_="">
     <xsd:import namespace="897f6830-f425-409d-b8f5-ce1019056d9e"/>
@@ -6026,15 +6051,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -6047,6 +6063,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A33EE264-283E-4F19-BA61-B3264EA417E2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6065,14 +6089,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF16440F-B0E0-4269-97EE-BEB05B0223C8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Additional property "currentverion" for Update.Frontend.Check
Also changed the key for the new version from
"updatecheck.frontend.version" to "updatecheck.frontend.newversion"
</commit_message>
<xml_diff>
--- a/AWB-RestApi-PropertyDictionary.xlsx
+++ b/AWB-RestApi-PropertyDictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\AgentWorkbench\eclipseProjects\de.enflexit.awb\bundles\web\xApi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69B6CA9F-8F9F-4B90-9056-8C6E7F94CBA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{520B824A-DEAC-4231-954D-74B4ED545F0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3800" yWindow="3800" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Property-Definition" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="218">
   <si>
     <t>key</t>
   </si>
@@ -642,9 +642,6 @@
     <t>updatecheck.backend.lastcheck</t>
   </si>
   <si>
-    <t>updatecheck.frontend.version</t>
-  </si>
-  <si>
     <t>updatecheck.frontend.isavailable</t>
   </si>
   <si>
@@ -687,10 +684,16 @@
     <t>e.g. 'Pending', 'Done', 'Error'</t>
   </si>
   <si>
-    <t>UPDATE.FRONTEND.CHECK[isForceCheck]</t>
-  </si>
-  <si>
     <t>e.g. '0.0.4.20260602-1140'</t>
+  </si>
+  <si>
+    <t>UPDATE.FRONTEND.CHECK</t>
+  </si>
+  <si>
+    <t>updatecheck.frontend.newversion</t>
+  </si>
+  <si>
+    <t>updatecheck.frontend.currentversion</t>
   </si>
 </sst>
 </file>
@@ -1070,22 +1073,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K103"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K104"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.7265625" customWidth="1"/>
-    <col min="3" max="3" width="14.26953125" customWidth="1"/>
-    <col min="4" max="4" width="54.1796875" customWidth="1"/>
-    <col min="5" max="5" width="17.1796875" customWidth="1"/>
+    <col min="1" max="1" width="34.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" customWidth="1"/>
+    <col min="4" max="4" width="54.140625" customWidth="1"/>
+    <col min="5" max="5" width="17.140625" customWidth="1"/>
     <col min="6" max="6" width="79" customWidth="1"/>
-    <col min="7" max="7" width="18.1796875" customWidth="1"/>
-    <col min="8" max="8" width="34.81640625" customWidth="1"/>
-    <col min="9" max="10" width="17.7265625" style="5" customWidth="1"/>
-    <col min="11" max="11" width="113.7265625" customWidth="1"/>
+    <col min="7" max="7" width="18.140625" customWidth="1"/>
+    <col min="8" max="8" width="34.85546875" customWidth="1"/>
+    <col min="9" max="10" width="17.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="113.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -1120,7 +1123,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1149,7 +1152,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>43</v>
       </c>
@@ -1175,7 +1178,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>43</v>
       </c>
@@ -1201,7 +1204,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -1227,7 +1230,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -1253,7 +1256,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>43</v>
       </c>
@@ -1279,7 +1282,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -1305,7 +1308,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>43</v>
       </c>
@@ -1331,7 +1334,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -1360,7 +1363,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -1392,7 +1395,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -1421,7 +1424,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -1450,7 +1453,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -1480,7 +1483,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -1509,7 +1512,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -1538,7 +1541,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>41</v>
       </c>
@@ -1567,7 +1570,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>41</v>
       </c>
@@ -1596,7 +1599,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>41</v>
       </c>
@@ -1622,7 +1625,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>41</v>
       </c>
@@ -1648,7 +1651,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>41</v>
       </c>
@@ -1674,7 +1677,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>41</v>
       </c>
@@ -1700,7 +1703,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>41</v>
       </c>
@@ -1726,7 +1729,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>64</v>
       </c>
@@ -1755,7 +1758,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>64</v>
       </c>
@@ -1784,7 +1787,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>64</v>
       </c>
@@ -1810,7 +1813,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>64</v>
       </c>
@@ -1836,7 +1839,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>64</v>
       </c>
@@ -1862,7 +1865,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>64</v>
       </c>
@@ -1888,7 +1891,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>64</v>
       </c>
@@ -1914,7 +1917,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>65</v>
       </c>
@@ -1940,7 +1943,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>65</v>
       </c>
@@ -1966,7 +1969,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>65</v>
       </c>
@@ -1992,7 +1995,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>65</v>
       </c>
@@ -2018,7 +2021,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>65</v>
       </c>
@@ -2044,7 +2047,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>65</v>
       </c>
@@ -2070,7 +2073,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>65</v>
       </c>
@@ -2096,7 +2099,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>73</v>
       </c>
@@ -2122,7 +2125,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>73</v>
       </c>
@@ -2148,7 +2151,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>73</v>
       </c>
@@ -2174,7 +2177,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>73</v>
       </c>
@@ -2200,7 +2203,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>73</v>
       </c>
@@ -2226,7 +2229,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>73</v>
       </c>
@@ -2252,7 +2255,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>82</v>
       </c>
@@ -2281,7 +2284,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>82</v>
       </c>
@@ -2307,7 +2310,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>82</v>
       </c>
@@ -2333,7 +2336,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>82</v>
       </c>
@@ -2359,7 +2362,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>82</v>
       </c>
@@ -2388,7 +2391,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>82</v>
       </c>
@@ -2417,7 +2420,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>82</v>
       </c>
@@ -2443,7 +2446,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>82</v>
       </c>
@@ -2469,7 +2472,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>82</v>
       </c>
@@ -2498,7 +2501,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>82</v>
       </c>
@@ -2524,7 +2527,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>82</v>
       </c>
@@ -2553,7 +2556,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>82</v>
       </c>
@@ -2579,7 +2582,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>82</v>
       </c>
@@ -2605,7 +2608,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>82</v>
       </c>
@@ -2631,7 +2634,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>82</v>
       </c>
@@ -2657,7 +2660,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>82</v>
       </c>
@@ -2683,7 +2686,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>91</v>
       </c>
@@ -2712,7 +2715,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>94</v>
       </c>
@@ -2738,7 +2741,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>95</v>
       </c>
@@ -2767,7 +2770,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>83</v>
       </c>
@@ -2793,7 +2796,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>83</v>
       </c>
@@ -2819,7 +2822,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>83</v>
       </c>
@@ -2845,7 +2848,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>83</v>
       </c>
@@ -2871,7 +2874,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>83</v>
       </c>
@@ -2897,7 +2900,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>83</v>
       </c>
@@ -2923,7 +2926,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>83</v>
       </c>
@@ -2949,7 +2952,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>83</v>
       </c>
@@ -2975,7 +2978,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>83</v>
       </c>
@@ -3001,7 +3004,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>83</v>
       </c>
@@ -3027,7 +3030,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>83</v>
       </c>
@@ -3053,7 +3056,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>83</v>
       </c>
@@ -3079,7 +3082,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>83</v>
       </c>
@@ -3105,7 +3108,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>83</v>
       </c>
@@ -3131,7 +3134,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>83</v>
       </c>
@@ -3157,7 +3160,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>83</v>
       </c>
@@ -3183,7 +3186,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>83</v>
       </c>
@@ -3209,7 +3212,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>83</v>
       </c>
@@ -3235,7 +3238,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>83</v>
       </c>
@@ -3261,7 +3264,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>83</v>
       </c>
@@ -3287,7 +3290,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>83</v>
       </c>
@@ -3313,7 +3316,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>83</v>
       </c>
@@ -3339,7 +3342,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>83</v>
       </c>
@@ -3365,7 +3368,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>83</v>
       </c>
@@ -3391,7 +3394,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>83</v>
       </c>
@@ -3417,7 +3420,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>83</v>
       </c>
@@ -3443,7 +3446,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>83</v>
       </c>
@@ -3469,7 +3472,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>83</v>
       </c>
@@ -3495,7 +3498,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>83</v>
       </c>
@@ -3521,7 +3524,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>83</v>
       </c>
@@ -3547,7 +3550,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>195</v>
       </c>
@@ -3564,18 +3567,18 @@
         <v>21</v>
       </c>
       <c r="H93" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="I93" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
+        <v>204</v>
+      </c>
+      <c r="B94" t="s">
         <v>205</v>
-      </c>
-      <c r="B94" t="s">
-        <v>206</v>
       </c>
       <c r="C94" t="s">
         <v>5</v>
@@ -3596,12 +3599,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
+        <v>204</v>
+      </c>
+      <c r="B95" t="s">
         <v>205</v>
-      </c>
-      <c r="B95" t="s">
-        <v>206</v>
       </c>
       <c r="C95" t="s">
         <v>5</v>
@@ -3622,12 +3625,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
+        <v>204</v>
+      </c>
+      <c r="B96" t="s">
         <v>205</v>
-      </c>
-      <c r="B96" t="s">
-        <v>206</v>
       </c>
       <c r="C96" t="s">
         <v>5</v>
@@ -3639,7 +3642,7 @@
         <v>7</v>
       </c>
       <c r="F96" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H96" t="s">
         <v>136</v>
@@ -3648,21 +3651,21 @@
         <v>59</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C97" t="s">
         <v>5</v>
       </c>
       <c r="D97" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E97" t="s">
         <v>7</v>
       </c>
       <c r="F97" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H97" t="s">
         <v>136</v>
@@ -3671,21 +3674,21 @@
         <v>59</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
+        <v>207</v>
+      </c>
+      <c r="C98" t="s">
+        <v>5</v>
+      </c>
+      <c r="D98" t="s">
         <v>208</v>
-      </c>
-      <c r="C98" t="s">
-        <v>5</v>
-      </c>
-      <c r="D98" t="s">
-        <v>209</v>
       </c>
       <c r="E98" t="s">
         <v>26</v>
       </c>
       <c r="F98" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H98" t="s">
         <v>136</v>
@@ -3694,21 +3697,21 @@
         <v>59</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C99" t="s">
         <v>5</v>
       </c>
       <c r="D99" t="s">
+        <v>211</v>
+      </c>
+      <c r="E99" t="s">
+        <v>7</v>
+      </c>
+      <c r="F99" t="s">
         <v>212</v>
-      </c>
-      <c r="E99" t="s">
-        <v>7</v>
-      </c>
-      <c r="F99" t="s">
-        <v>213</v>
       </c>
       <c r="H99" t="s">
         <v>136</v>
@@ -3717,18 +3720,15 @@
         <v>59</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>215</v>
       </c>
-      <c r="B100" t="s">
-        <v>206</v>
-      </c>
       <c r="C100" t="s">
         <v>5</v>
       </c>
       <c r="D100" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E100" t="s">
         <v>20</v>
@@ -3737,24 +3737,21 @@
         <v>21</v>
       </c>
       <c r="H100" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="I100" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>215</v>
       </c>
-      <c r="B101" t="s">
-        <v>206</v>
-      </c>
       <c r="C101" t="s">
         <v>5</v>
       </c>
       <c r="D101" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E101" t="s">
         <v>20</v>
@@ -3763,62 +3760,73 @@
         <v>21</v>
       </c>
       <c r="H101" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="I101" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>215</v>
       </c>
-      <c r="B102" t="s">
+      <c r="C102" t="s">
+        <v>5</v>
+      </c>
+      <c r="D102" t="s">
+        <v>201</v>
+      </c>
+      <c r="E102" t="s">
+        <v>7</v>
+      </c>
+      <c r="F102" t="s">
         <v>206</v>
       </c>
-      <c r="C102" t="s">
-        <v>5</v>
-      </c>
-      <c r="D102" t="s">
+      <c r="H102" t="s">
         <v>202</v>
       </c>
-      <c r="E102" t="s">
-        <v>7</v>
-      </c>
-      <c r="F102" t="s">
-        <v>207</v>
-      </c>
-      <c r="H102" t="s">
-        <v>203</v>
-      </c>
       <c r="I102" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>215</v>
       </c>
-      <c r="B103" t="s">
-        <v>206</v>
-      </c>
       <c r="C103" t="s">
         <v>5</v>
       </c>
       <c r="D103" t="s">
-        <v>200</v>
+        <v>216</v>
       </c>
       <c r="E103" t="s">
         <v>7</v>
       </c>
       <c r="F103" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H103" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="I103" s="5" t="s">
         <v>59</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>215</v>
+      </c>
+      <c r="C104" t="s">
+        <v>5</v>
+      </c>
+      <c r="D104" t="s">
+        <v>217</v>
+      </c>
+      <c r="E104" t="s">
+        <v>7</v>
+      </c>
+      <c r="F104" t="s">
+        <v>214</v>
       </c>
     </row>
   </sheetData>
@@ -3841,13 +3849,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F30A1E73-A707-4178-9C72-9AC27F9EE5F7}">
   <dimension ref="A1:B113"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7265625" customWidth="1"/>
+    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="str">
         <f>'Property-Definition'!A1</f>
         <v>performative</v>
@@ -3856,7 +3864,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="str">
         <f>'Property-Definition'!A2</f>
         <v>DB.SYSTEMS</v>
@@ -3875,7 +3883,7 @@
         <v>public final static String DBSYSTEM = "dbSystem[X]";</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
         <f>'Property-Definition'!A3</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3894,7 +3902,7 @@
         <v>public final static String DBSYSTEM = "dbSystem[X]";</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
         <f>'Property-Definition'!A4</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3913,7 +3921,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_DRIVER_CLASS = "dbSystem[X].hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
         <f>'Property-Definition'!A5</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3932,7 +3940,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_URL = "dbSystem[X].hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
         <f>'Property-Definition'!A6</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3951,7 +3959,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_URL_MASK = "dbSystem[X].hibernate.connection.url.mask";</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
         <f>'Property-Definition'!A7</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3970,7 +3978,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_DEFAULT_CATALOG = "dbSystem[X].hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
         <f>'Property-Definition'!A8</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -3989,7 +3997,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_USERNAME = "dbSystem[X].hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
         <f>'Property-Definition'!A9</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -4008,7 +4016,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_PASSWORD = "dbSystem[X].hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="str">
         <f>'Property-Definition'!A10</f>
         <v>DB.FACTORIES</v>
@@ -4027,7 +4035,7 @@
         <v>public final static String FACTORY = "factory[X]";</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="str">
         <f>'Property-Definition'!A11</f>
         <v>DB.FACTORIES</v>
@@ -4046,7 +4054,7 @@
         <v>public final static String FACTORY_STATE = "factory[X].state";</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
         <f>'Property-Definition'!A12</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -4065,7 +4073,7 @@
         <v>public final static String ISSTARTDERBYNETWORKSERVER = "isStartDerbyNetworkServer";</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
         <f>'Property-Definition'!A13</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -4084,7 +4092,7 @@
         <v>public final static String HOST-IP = "host-IP";</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="str">
         <f>'Property-Definition'!A14</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -4103,7 +4111,7 @@
         <v>public final static String PORT = "port";</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="str">
         <f>'Property-Definition'!A15</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -4122,7 +4130,7 @@
         <v>public final static String USERNAME = "userName";</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="str">
         <f>'Property-Definition'!A16</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -4141,7 +4149,7 @@
         <v>public final static String PASSWORD = "password";</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="str">
         <f>'Property-Definition'!A17</f>
         <v>DB.CONN.GENERAL</v>
@@ -4160,7 +4168,7 @@
         <v>public final static String USEFOREVERYFACTORY = "useForEveryFactory";</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="str">
         <f>'Property-Definition'!A18</f>
         <v>DB.CONN.GENERAL</v>
@@ -4179,7 +4187,7 @@
         <v>public final static String DBSYSTEM = "dbSystem";</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="str">
         <f>'Property-Definition'!A19</f>
         <v>DB.CONN.GENERAL</v>
@@ -4198,7 +4206,7 @@
         <v>public final static String HIBERNATE_CONNECTION_DRIVER_CLASS = "hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="str">
         <f>'Property-Definition'!A20</f>
         <v>DB.CONN.GENERAL</v>
@@ -4217,7 +4225,7 @@
         <v>public final static String HIBERNATE_CONNECTION_URL = "hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="str">
         <f>'Property-Definition'!A21</f>
         <v>DB.CONN.GENERAL</v>
@@ -4236,7 +4244,7 @@
         <v>public final static String HIBERNATE_DEFAULT_CATALOG = "hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="str">
         <f>'Property-Definition'!A22</f>
         <v>DB.CONN.GENERAL</v>
@@ -4255,7 +4263,7 @@
         <v>public final static String HIBERNATE_CONNECTION_USERNAME = "hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
         <f>'Property-Definition'!A23</f>
         <v>DB.CONN.GENERAL</v>
@@ -4274,7 +4282,7 @@
         <v>public final static String HIBERNATE_CONNECTION_PASSWORD = "hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="str">
         <f>'Property-Definition'!A24</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4293,7 +4301,7 @@
         <v>public final static String FACTORY_FACTORYID = "factory[X].factoryID";</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="str">
         <f>'Property-Definition'!A25</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4312,7 +4320,7 @@
         <v>public final static String FACTORY_DBSYSTEM = "factory[X].dbSystem";</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="str">
         <f>'Property-Definition'!A26</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4331,7 +4339,7 @@
         <v>public final static String FACTORY_HIBERNATE_CONNECTION_DRIVER_CLASS = "factory[X].hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="str">
         <f>'Property-Definition'!A27</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4350,7 +4358,7 @@
         <v>public final static String FACTORY_HIBERNATE_CONNECTION_URL = "factory[X].hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="str">
         <f>'Property-Definition'!A28</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4369,7 +4377,7 @@
         <v>public final static String FACTORY_HIBERNATE_DEFAULT_CATALOG = "factory[X].hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="str">
         <f>'Property-Definition'!A29</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4388,7 +4396,7 @@
         <v>public final static String FACTORY_HIBERNATE_CONNECTION_USERNAME = "factory[X].hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="str">
         <f>'Property-Definition'!A30</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4407,7 +4415,7 @@
         <v>public final static String FACTORY_HIBERNATE_CONNECTION_PASSWORD = "factory[X].hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="str">
         <f>'Property-Definition'!A31</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4426,7 +4434,7 @@
         <v>public final static String FACTORYID = "factoryID";</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="str">
         <f>'Property-Definition'!A32</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4445,7 +4453,7 @@
         <v>public final static String DBSYSTEM = "dbSystem";</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="str">
         <f>'Property-Definition'!A33</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4464,7 +4472,7 @@
         <v>public final static String HIBERNATE_CONNECTION_DRIVER_CLASS = "hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="str">
         <f>'Property-Definition'!A34</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4483,7 +4491,7 @@
         <v>public final static String HIBERNATE_CONNECTION_URL = "hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="str">
         <f>'Property-Definition'!A35</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4502,7 +4510,7 @@
         <v>public final static String HIBERNATE_DEFAULT_CATALOG = "hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="str">
         <f>'Property-Definition'!A36</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4521,7 +4529,7 @@
         <v>public final static String HIBERNATE_CONNECTION_USERNAME = "hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="str">
         <f>'Property-Definition'!A37</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4540,7 +4548,7 @@
         <v>public final static String HIBERNATE_CONNECTION_PASSWORD = "hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="str">
         <f>'Property-Definition'!A38</f>
         <v>DB.CONN.TEST</v>
@@ -4559,7 +4567,7 @@
         <v>public final static String DBSYSTEM = "dbSystem";</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="str">
         <f>'Property-Definition'!A39</f>
         <v>DB.CONN.TEST</v>
@@ -4578,7 +4586,7 @@
         <v>public final static String HIBERNATE_CONNECTION_DRIVER_CLASS = "hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="str">
         <f>'Property-Definition'!A40</f>
         <v>DB.CONN.TEST</v>
@@ -4597,7 +4605,7 @@
         <v>public final static String HIBERNATE_CONNECTION_URL = "hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="str">
         <f>'Property-Definition'!A41</f>
         <v>DB.CONN.TEST</v>
@@ -4616,7 +4624,7 @@
         <v>public final static String HIBERNATE_DEFAULT_CATALOG = "hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="str">
         <f>'Property-Definition'!A42</f>
         <v>DB.CONN.TEST</v>
@@ -4635,7 +4643,7 @@
         <v>public final static String HIBERNATE_CONNECTION_USERNAME = "hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="str">
         <f>'Property-Definition'!A43</f>
         <v>DB.CONN.TEST</v>
@@ -4654,7 +4662,7 @@
         <v>public final static String HIBERNATE_CONNECTION_PASSWORD = "hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="str">
         <f>'Property-Definition'!A44</f>
         <v>EXEC.MODE</v>
@@ -4673,7 +4681,7 @@
         <v>public final static String EXEC_MODE = "exec.mode";</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="str">
         <f>'Property-Definition'!A45</f>
         <v>EXEC.MODE</v>
@@ -4692,7 +4700,7 @@
         <v>public final static String SERVER_MASTER_URL = "server.master.url";</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="str">
         <f>'Property-Definition'!A46</f>
         <v>EXEC.MODE</v>
@@ -4711,7 +4719,7 @@
         <v>public final static String SERVER_MASTER_PORT = "server.master.port";</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="str">
         <f>'Property-Definition'!A47</f>
         <v>EXEC.MODE</v>
@@ -4730,7 +4738,7 @@
         <v>public final static String SERVER_MASTER_PORT_MTP = "server.master.port.mtp";</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="str">
         <f>'Property-Definition'!A48</f>
         <v>EXEC.MODE</v>
@@ -4749,7 +4757,7 @@
         <v>public final static String SERVER_MASTER_PROTOCOL = "server.master.protocol";</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="str">
         <f>'Property-Definition'!A49</f>
         <v>EXEC.MODE</v>
@@ -4768,7 +4776,7 @@
         <v>public final static String LOCAL_MTP_CREATION = "local.mtp.creation";</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="str">
         <f>'Property-Definition'!A50</f>
         <v>EXEC.MODE</v>
@@ -4787,7 +4795,7 @@
         <v>public final static String LOCAL_MTP_URL = "local.mtp.url";</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="str">
         <f>'Property-Definition'!A51</f>
         <v>EXEC.MODE</v>
@@ -4806,7 +4814,7 @@
         <v>public final static String LOCAL_MTP_PORT = "local.mtp.port";</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="str">
         <f>'Property-Definition'!A52</f>
         <v>EXEC.MODE</v>
@@ -4825,7 +4833,7 @@
         <v>public final static String LOCAL_MTP_PROTOCOL = "local.mtp.protocol";</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="str">
         <f>'Property-Definition'!A53</f>
         <v>EXEC.MODE</v>
@@ -4844,7 +4852,7 @@
         <v>public final static String EMBEDDEDSYSTEM_PROJECT = "embeddedsystem.project";</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="str">
         <f>'Property-Definition'!A54</f>
         <v>EXEC.MODE</v>
@@ -4863,7 +4871,7 @@
         <v>public final static String DEVICE_SYSTEM_EXEC_MODE = "device_system_exec_mode";</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="str">
         <f>'Property-Definition'!A55</f>
         <v>EXEC.MODE</v>
@@ -4882,7 +4890,7 @@
         <v>public final static String EMBEDDEDSYSTEM_AGENT_CLASSNAME = "embeddedsystem.agent[X].classname";</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="str">
         <f>'Property-Definition'!A56</f>
         <v>EXEC.MODE</v>
@@ -4901,7 +4909,7 @@
         <v>public final static String EMBEDDEDSYSTEM_AGENT_AGENTNAME = "embeddedsystem.agent[X].agentname";</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="str">
         <f>'Property-Definition'!A57</f>
         <v>EXEC.MODE</v>
@@ -4920,7 +4928,7 @@
         <v>public final static String SERVICE_SERVICE_SETUP = "service.service_setup";</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="str">
         <f>'Property-Definition'!A58</f>
         <v>EXEC.MODE</v>
@@ -4939,7 +4947,7 @@
         <v>public final static String LOCAL_IP_SELECTION = "local.ip.selection[X]";</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="str">
         <f>'Property-Definition'!A59</f>
         <v>EXEC.MODE</v>
@@ -4958,7 +4966,7 @@
         <v>public final static String FACTORY_ID = "factory_id";</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="e">
         <f>'Property-Definition'!#REF!</f>
         <v>#REF!</v>
@@ -4977,7 +4985,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="str">
         <f>'Property-Definition'!A60</f>
         <v>AWB.AGENTS</v>
@@ -4996,7 +5004,7 @@
         <v>public final static String AGENT_CLASSNAME = "agent[X].classname";</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="str">
         <f>'Property-Definition'!A61</f>
         <v>PROJECTS</v>
@@ -5015,7 +5023,7 @@
         <v>public final static String PROJECT = "project[X]";</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="str">
         <f>'Property-Definition'!A62</f>
         <v>PROJECT.SETUPS[X]</v>
@@ -5034,7 +5042,7 @@
         <v>public final static String PROJECT_SETUP = "project[X].setup[X]";</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="str">
         <f>'Property-Definition'!A63</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5053,7 +5061,7 @@
         <v>public final static String BGPLATFORM_CONTACTAGENT = "bgplatform[X].contactagent";</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="str">
         <f>'Property-Definition'!A60</f>
         <v>AWB.AGENTS</v>
@@ -5072,7 +5080,7 @@
         <v>public final static String BGPLATFORM_PLATFORMNAME = "bgplatform[X].platformname";</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="str">
         <f>'Property-Definition'!A61</f>
         <v>PROJECTS</v>
@@ -5091,7 +5099,7 @@
         <v>public final static String BGPLATFORM_SERVER = "bgplatform[X].server";</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="str">
         <f>'Property-Definition'!A62</f>
         <v>PROJECT.SETUPS[X]</v>
@@ -5110,7 +5118,7 @@
         <v>public final static String BGPLATFORM_IPADDRESS = "bgplatform[X].ipaddress";</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="str">
         <f>'Property-Definition'!A67</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5129,7 +5137,7 @@
         <v>public final static String BGPLATFORM_URL = "bgplatform[X].url";</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="str">
         <f>'Property-Definition'!A68</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5148,7 +5156,7 @@
         <v>public final static String BGPLATFORM_JADEPORT = "bgplatform[X].jadeport";</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="str">
         <f>'Property-Definition'!A69</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5167,7 +5175,7 @@
         <v>public final static String BGPLATFORM_HTTPMTP = "bgplatform[X].httpmtp";</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="str">
         <f>'Property-Definition'!A70</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5186,7 +5194,7 @@
         <v>public final static String BGPLATFORM_VERSIONMAJOR = "bgplatform[X].versionmajor";</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="str">
         <f>'Property-Definition'!A71</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5205,7 +5213,7 @@
         <v>public final static String BGPLATFORM_VERSIONMINOR = "bgplatform[X].versionminor";</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="str">
         <f>'Property-Definition'!A72</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5224,7 +5232,7 @@
         <v>public final static String BGPLATFORM_VERSIONMICRO = "bgplatform[X].versionmicro";</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="str">
         <f>'Property-Definition'!A73</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5243,7 +5251,7 @@
         <v>public final static String BGPLATFORM_VERSIONBUILD = "bgplatform[X].versionbuild";</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="str">
         <f>'Property-Definition'!A74</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5262,7 +5270,7 @@
         <v>public final static String BGPLATFORM_OS_NAME = "bgplatform[X].os.name";</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="str">
         <f>'Property-Definition'!A75</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5281,7 +5289,7 @@
         <v>public final static String BGPLATFORM_OS_VERSION = "bgplatform[X].os.version";</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="str">
         <f>'Property-Definition'!A76</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5300,7 +5308,7 @@
         <v>public final static String BGPLATFORM_OS_ARCHITECTURE = "bgplatform[X].os.architecture";</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="str">
         <f>'Property-Definition'!A77</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5319,7 +5327,7 @@
         <v>public final static String BGPLATFORM_CPU_NAME = "bgplatform[X].cpu.name";</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="str">
         <f>'Property-Definition'!A78</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5338,7 +5346,7 @@
         <v>public final static String BGPLATFORM_CPU_NUMLOGICAL = "bgplatform[X].cpu.numlogical";</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="str">
         <f>'Property-Definition'!A79</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5357,7 +5365,7 @@
         <v>public final static String BGPLATFORM_CPU_NUMPHYSICAL = "bgplatform[X].cpu.numphysical";</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="str">
         <f>'Property-Definition'!A80</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5376,7 +5384,7 @@
         <v>public final static String BGPLATFORM_CPU_SPEEDMHZ = "bgplatform[X].cpu.speedmhz";</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="str">
         <f>'Property-Definition'!A81</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5395,7 +5403,7 @@
         <v>public final static String BGPLATFORM_MEMORYMB = "bgplatform[X].memorymb";</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="str">
         <f>'Property-Definition'!A82</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5414,7 +5422,7 @@
         <v>public final static String BGPLATFORM_BENCHMARKVALUE = "bgplatform[X].benchmarkvalue";</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="str">
         <f>'Property-Definition'!A83</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5433,7 +5441,7 @@
         <v>public final static String BGPLATFORM_TIME_ONLINESINCE = "bgplatform[X].time.onlinesince";</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="str">
         <f>'Property-Definition'!A84</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5452,7 +5460,7 @@
         <v>public final static String BGPLATFORM_TIME_LASTCONTACT = "bgplatform[X].time.lastcontact";</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="str">
         <f>'Property-Definition'!A85</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5471,7 +5479,7 @@
         <v>public final static String BGPLATFORM_LOCALTIME_ONLINESINCE = "bgplatform[X].localtime.onlinesince";</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="str">
         <f>'Property-Definition'!A86</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5490,7 +5498,7 @@
         <v>public final static String BGPLATFORM_LOCALTIME_LASTCONTACT = "bgplatform[X].localtime.lastcontact";</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="str">
         <f>'Property-Definition'!A87</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5509,7 +5517,7 @@
         <v>public final static String BGPLATFORM_CURRENTLYAVAILABLE = "bgplatform[X].currentlyavailable";</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="str">
         <f>'Property-Definition'!A88</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5528,7 +5536,7 @@
         <v>public final static String BGPLATFORM_CURRENT_CPULOAD = "bgplatform[X].current.cpuload";</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="str">
         <f>'Property-Definition'!A89</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5547,7 +5555,7 @@
         <v>public final static String BGPLATFORM_CURRENT_MEMORYLOAD = "bgplatform[X].current.memoryload";</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="str">
         <f>'Property-Definition'!A90</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5566,7 +5574,7 @@
         <v>public final static String BGPLATFORM_CURRENT_MEMORYLOADJVM = "bgplatform[X].current.memoryloadjvm";</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="str">
         <f>'Property-Definition'!A91</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5585,7 +5593,7 @@
         <v>public final static String BGPLATFORM_CURRENT_NUMTHREADS = "bgplatform[X].current.numthreads";</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="str">
         <f>'Property-Definition'!A92</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5604,7 +5612,7 @@
         <v>public final static String BGPLATFORM_CURRENT_THRESHOLDEXCEEDED = "bgplatform[X].current.thresholdexceeded";</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="str">
         <f>'Property-Definition'!A93</f>
         <v>UPDATE.STRATEGY</v>
@@ -5623,7 +5631,7 @@
         <v>public final static String ISAUTOUPDATE = "isautoupdate";</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="str">
         <f>'Property-Definition'!A94</f>
         <v>UPDATE.BACKEND.CHECK[isForceCheck]</v>
@@ -5642,7 +5650,7 @@
         <v>public final static String UPDATECHECK_BACKEND_ISPENDING = "updatecheck.backend.ispending";</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="str">
         <f>'Property-Definition'!A95</f>
         <v>UPDATE.BACKEND.CHECK[isForceCheck]</v>
@@ -5661,7 +5669,7 @@
         <v>public final static String UPDATECHECK_BACKEND_ISAVAILABLE = "updatecheck.backend.isavailable";</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="str">
         <f>'Property-Definition'!A96</f>
         <v>UPDATE.BACKEND.CHECK[isForceCheck]</v>
@@ -5680,7 +5688,7 @@
         <v>public final static String UPDATECHECK_BACKEND_LASTCHECK = "updatecheck.backend.lastcheck";</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="e">
         <f>'Property-Definition'!#REF!</f>
         <v>#REF!</v>
@@ -5699,10 +5707,10 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="str">
         <f>'Property-Definition'!A100</f>
-        <v>UPDATE.FRONTEND.CHECK[isForceCheck]</v>
+        <v>UPDATE.FRONTEND.CHECK</v>
       </c>
       <c r="B99" t="str">
         <f>"public final static String "
@@ -5718,10 +5726,10 @@
         <v>public final static String UPDATECHECK_FRONTEND_ISPENDING = "updatecheck.frontend.ispending";</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="str">
         <f>'Property-Definition'!A101</f>
-        <v>UPDATE.FRONTEND.CHECK[isForceCheck]</v>
+        <v>UPDATE.FRONTEND.CHECK</v>
       </c>
       <c r="B100" t="str">
         <f>"public final static String "
@@ -5737,10 +5745,10 @@
         <v>public final static String UPDATECHECK_FRONTEND_ISAVAILABLE = "updatecheck.frontend.isavailable";</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="str">
         <f>'Property-Definition'!A102</f>
-        <v>UPDATE.FRONTEND.CHECK[isForceCheck]</v>
+        <v>UPDATE.FRONTEND.CHECK</v>
       </c>
       <c r="B101" t="str">
         <f>"public final static String "
@@ -5756,10 +5764,10 @@
         <v>public final static String UPDATECHECK_FRONTEND_LASTCHECK = "updatecheck.frontend.lastcheck";</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="str">
         <f>'Property-Definition'!A103</f>
-        <v>UPDATE.FRONTEND.CHECK[isForceCheck]</v>
+        <v>UPDATE.FRONTEND.CHECK</v>
       </c>
       <c r="B102" t="str">
         <f>"public final static String "
@@ -5772,70 +5780,70 @@
 &amp; 'Property-Definition'!D103
 &amp; CHAR(34)
 &amp; ";"</f>
-        <v>public final static String UPDATECHECK_FRONTEND_VERSION = "updatecheck.frontend.version";</v>
-      </c>
-    </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A103">
+        <v>public final static String UPDATECHECK_FRONTEND_NEWVERSION = "updatecheck.frontend.newversion";</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A103" t="str">
         <f>'Property-Definition'!A104</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
+        <v>UPDATE.FRONTEND.CHECK</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104">
         <f>'Property-Definition'!A105</f>
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105">
         <f>'Property-Definition'!A106</f>
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106">
         <f>'Property-Definition'!A107</f>
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107">
         <f>'Property-Definition'!A108</f>
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108">
         <f>'Property-Definition'!A109</f>
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109">
         <f>'Property-Definition'!A110</f>
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110">
         <f>'Property-Definition'!A111</f>
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111">
         <f>'Property-Definition'!A112</f>
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112">
         <f>'Property-Definition'!A113</f>
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113">
         <f>'Property-Definition'!A114</f>
         <v>0</v>
@@ -5848,15 +5856,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101004FB79D76D905EB41B4AD64ED4839597F" ma:contentTypeVersion="11" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="0622d98e252eab518d4b54f931ba6851">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="897f6830-f425-409d-b8f5-ce1019056d9e" xmlns:ns3="f2404b4d-361b-46d3-b2ec-035eed29e274" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dd5f302b3846fd12003b89c8f5b7df36" ns2:_="" ns3:_="">
     <xsd:import namespace="897f6830-f425-409d-b8f5-ce1019056d9e"/>
@@ -6051,6 +6050,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -6063,14 +6071,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A33EE264-283E-4F19-BA61-B3264EA417E2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6089,6 +6089,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF16440F-B0E0-4269-97EE-BEB05B0223C8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Included new performative "FILECONFIGURATION".
</commit_message>
<xml_diff>
--- a/AWB-RestApi-PropertyDictionary.xlsx
+++ b/AWB-RestApi-PropertyDictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\AgentWorkbench\eclipseProjects\de.enflexit.awb\bundles\web\xAPI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9A1BAD0-D6ED-44A5-B2E5-A434418B8240}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F46DF6F3-6BD7-4C8F-A445-32C24711D7D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6250" yWindow="5430" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Property-Definition" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="866" uniqueCount="226">
   <si>
     <t>key</t>
   </si>
@@ -709,6 +709,15 @@
   </si>
   <si>
     <t>UPDATE.BACKEND.CHECK</t>
+  </si>
+  <si>
+    <t>FILECONFIGURATION</t>
+  </si>
+  <si>
+    <t>configurationtype[X]</t>
+  </si>
+  <si>
+    <t>e.g. 'JettyConfiguration'</t>
   </si>
 </sst>
 </file>
@@ -1088,7 +1097,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K106"/>
+  <dimension ref="A1:K107"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34.453125" bestFit="1" customWidth="1"/>
@@ -3890,8 +3899,31 @@
         <v>59</v>
       </c>
     </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
+        <v>223</v>
+      </c>
+      <c r="C107" t="s">
+        <v>5</v>
+      </c>
+      <c r="D107" t="s">
+        <v>224</v>
+      </c>
+      <c r="E107" t="s">
+        <v>7</v>
+      </c>
+      <c r="F107" t="s">
+        <v>225</v>
+      </c>
+      <c r="H107" t="s">
+        <v>136</v>
+      </c>
+      <c r="I107" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:J43 J44:J93 I44:I106">
+  <conditionalFormatting sqref="I2:J43 J44:J93 I44:I107">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>
@@ -5863,9 +5895,9 @@
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A106">
+      <c r="A106" t="str">
         <f>'Property-Definition'!A107</f>
-        <v>0</v>
+        <v>FILECONFIGURATION</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.35">
@@ -5917,6 +5949,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101004FB79D76D905EB41B4AD64ED4839597F" ma:contentTypeVersion="11" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="0622d98e252eab518d4b54f931ba6851">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="897f6830-f425-409d-b8f5-ce1019056d9e" xmlns:ns3="f2404b4d-361b-46d3-b2ec-035eed29e274" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dd5f302b3846fd12003b89c8f5b7df36" ns2:_="" ns3:_="">
     <xsd:import namespace="897f6830-f425-409d-b8f5-ce1019056d9e"/>
@@ -6111,15 +6152,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -6132,6 +6164,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A33EE264-283E-4F19-BA61-B3264EA417E2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6150,14 +6190,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF16440F-B0E0-4269-97EE-BEB05B0223C8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
New endpoint /app/settings/download in REST api definition.
Also small update for RestApi property dictionary.
</commit_message>
<xml_diff>
--- a/AWB-RestApi-PropertyDictionary.xlsx
+++ b/AWB-RestApi-PropertyDictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\AgentWorkbench\eclipseProjects\de.enflexit.awb\bundles\web\xAPI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F46DF6F3-6BD7-4C8F-A445-32C24711D7D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1859E29F-F7C8-43EE-8E0F-6203DD4DA4CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6250" yWindow="5430" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Property-Definition" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="866" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="881" uniqueCount="226">
   <si>
     <t>key</t>
   </si>
@@ -711,13 +711,13 @@
     <t>UPDATE.BACKEND.CHECK</t>
   </si>
   <si>
-    <t>FILECONFIGURATION</t>
-  </si>
-  <si>
     <t>configurationtype[X]</t>
   </si>
   <si>
     <t>e.g. 'JettyConfiguration'</t>
+  </si>
+  <si>
+    <t>FILE.CONFIGURATION</t>
   </si>
 </sst>
 </file>
@@ -3622,6 +3622,9 @@
       <c r="I94" s="5" t="s">
         <v>59</v>
       </c>
+      <c r="J94" s="5" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
@@ -3645,6 +3648,9 @@
       <c r="I95" s="5" t="s">
         <v>59</v>
       </c>
+      <c r="J95" s="5" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
@@ -3668,8 +3674,11 @@
       <c r="I96" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J96" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>205</v>
       </c>
@@ -3691,8 +3700,11 @@
       <c r="I97" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J97" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>205</v>
       </c>
@@ -3714,8 +3726,11 @@
       <c r="I98" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J98" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>205</v>
       </c>
@@ -3737,8 +3752,11 @@
       <c r="I99" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J99" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>213</v>
       </c>
@@ -3760,8 +3778,11 @@
       <c r="I100" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J100" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>213</v>
       </c>
@@ -3783,8 +3804,11 @@
       <c r="I101" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J101" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>213</v>
       </c>
@@ -3806,8 +3830,11 @@
       <c r="I102" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J102" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>213</v>
       </c>
@@ -3829,8 +3856,11 @@
       <c r="I103" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J103" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>213</v>
       </c>
@@ -3852,8 +3882,11 @@
       <c r="I104" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J104" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>217</v>
       </c>
@@ -3872,11 +3905,17 @@
       <c r="G105" t="s">
         <v>220</v>
       </c>
+      <c r="H105" t="s">
+        <v>202</v>
+      </c>
       <c r="I105" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J105" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>217</v>
       </c>
@@ -3895,25 +3934,31 @@
       <c r="G106" t="s">
         <v>221</v>
       </c>
+      <c r="H106" t="s">
+        <v>202</v>
+      </c>
       <c r="I106" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J106" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
+        <v>225</v>
+      </c>
+      <c r="C107" t="s">
+        <v>5</v>
+      </c>
+      <c r="D107" t="s">
         <v>223</v>
       </c>
-      <c r="C107" t="s">
-        <v>5</v>
-      </c>
-      <c r="D107" t="s">
+      <c r="E107" t="s">
+        <v>7</v>
+      </c>
+      <c r="F107" t="s">
         <v>224</v>
-      </c>
-      <c r="E107" t="s">
-        <v>7</v>
-      </c>
-      <c r="F107" t="s">
-        <v>225</v>
       </c>
       <c r="H107" t="s">
         <v>136</v>
@@ -3923,7 +3968,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:J43 J44:J93 I44:I107">
+  <conditionalFormatting sqref="I2:J43 I44:I107 J44:J106">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>
@@ -5897,7 +5942,7 @@
     <row r="106" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A106" t="str">
         <f>'Property-Definition'!A107</f>
-        <v>FILECONFIGURATION</v>
+        <v>FILE.CONFIGURATION</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.35">
@@ -5949,15 +5994,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101004FB79D76D905EB41B4AD64ED4839597F" ma:contentTypeVersion="11" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="0622d98e252eab518d4b54f931ba6851">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="897f6830-f425-409d-b8f5-ce1019056d9e" xmlns:ns3="f2404b4d-361b-46d3-b2ec-035eed29e274" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dd5f302b3846fd12003b89c8f5b7df36" ns2:_="" ns3:_="">
     <xsd:import namespace="897f6830-f425-409d-b8f5-ce1019056d9e"/>
@@ -6152,6 +6188,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -6164,14 +6209,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A33EE264-283E-4F19-BA61-B3264EA417E2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6190,6 +6227,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF16440F-B0E0-4269-97EE-BEB05B0223C8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Updated property dictionary with new performative "websocket.ticket".
</commit_message>
<xml_diff>
--- a/AWB-RestApi-PropertyDictionary.xlsx
+++ b/AWB-RestApi-PropertyDictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\AgentWorkbench\eclipseProjects\de.enflexit.awb\bundles\web\xAPI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1859E29F-F7C8-43EE-8E0F-6203DD4DA4CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A688409-1B66-4412-B618-03856C3554CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Property-Definition" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="881" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="888" uniqueCount="229">
   <si>
     <t>key</t>
   </si>
@@ -718,6 +718,15 @@
   </si>
   <si>
     <t>FILE.CONFIGURATION</t>
+  </si>
+  <si>
+    <t>WEBSOCKET.TICKET</t>
+  </si>
+  <si>
+    <t>ticket.id</t>
+  </si>
+  <si>
+    <t>e.g. '5d33d7e1-a215-438e-9702-361cabfd88bb'</t>
   </si>
 </sst>
 </file>
@@ -1097,22 +1106,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K107"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K108"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.7265625" customWidth="1"/>
-    <col min="3" max="3" width="14.26953125" customWidth="1"/>
-    <col min="4" max="4" width="54.1796875" customWidth="1"/>
-    <col min="5" max="5" width="17.1796875" customWidth="1"/>
+    <col min="1" max="1" width="34.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" customWidth="1"/>
+    <col min="4" max="4" width="54.140625" customWidth="1"/>
+    <col min="5" max="5" width="17.140625" customWidth="1"/>
     <col min="6" max="6" width="79" customWidth="1"/>
-    <col min="7" max="7" width="18.1796875" customWidth="1"/>
-    <col min="8" max="8" width="34.81640625" customWidth="1"/>
-    <col min="9" max="10" width="17.7265625" style="5" customWidth="1"/>
-    <col min="11" max="11" width="113.7265625" customWidth="1"/>
+    <col min="7" max="7" width="18.140625" customWidth="1"/>
+    <col min="8" max="8" width="34.85546875" customWidth="1"/>
+    <col min="9" max="10" width="17.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="113.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -1147,7 +1156,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1176,7 +1185,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>43</v>
       </c>
@@ -1202,7 +1211,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>43</v>
       </c>
@@ -1228,7 +1237,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -1254,7 +1263,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -1280,7 +1289,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>43</v>
       </c>
@@ -1306,7 +1315,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -1332,7 +1341,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>43</v>
       </c>
@@ -1358,7 +1367,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -1387,7 +1396,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -1419,7 +1428,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -1448,7 +1457,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -1477,7 +1486,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -1507,7 +1516,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -1536,7 +1545,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -1565,7 +1574,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>41</v>
       </c>
@@ -1594,7 +1603,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>41</v>
       </c>
@@ -1623,7 +1632,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>41</v>
       </c>
@@ -1649,7 +1658,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>41</v>
       </c>
@@ -1675,7 +1684,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>41</v>
       </c>
@@ -1701,7 +1710,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>41</v>
       </c>
@@ -1727,7 +1736,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>41</v>
       </c>
@@ -1753,7 +1762,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>64</v>
       </c>
@@ -1782,7 +1791,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>64</v>
       </c>
@@ -1811,7 +1820,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>64</v>
       </c>
@@ -1837,7 +1846,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>64</v>
       </c>
@@ -1863,7 +1872,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>64</v>
       </c>
@@ -1889,7 +1898,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>64</v>
       </c>
@@ -1915,7 +1924,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>64</v>
       </c>
@@ -1941,7 +1950,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>65</v>
       </c>
@@ -1967,7 +1976,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>65</v>
       </c>
@@ -1993,7 +2002,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>65</v>
       </c>
@@ -2019,7 +2028,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>65</v>
       </c>
@@ -2045,7 +2054,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>65</v>
       </c>
@@ -2071,7 +2080,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>65</v>
       </c>
@@ -2097,7 +2106,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>65</v>
       </c>
@@ -2123,7 +2132,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>73</v>
       </c>
@@ -2149,7 +2158,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>73</v>
       </c>
@@ -2175,7 +2184,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>73</v>
       </c>
@@ -2201,7 +2210,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>73</v>
       </c>
@@ -2227,7 +2236,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>73</v>
       </c>
@@ -2253,7 +2262,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>73</v>
       </c>
@@ -2279,7 +2288,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>82</v>
       </c>
@@ -2308,7 +2317,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>82</v>
       </c>
@@ -2334,7 +2343,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>82</v>
       </c>
@@ -2360,7 +2369,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>82</v>
       </c>
@@ -2386,7 +2395,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>82</v>
       </c>
@@ -2415,7 +2424,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>82</v>
       </c>
@@ -2444,7 +2453,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>82</v>
       </c>
@@ -2470,7 +2479,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>82</v>
       </c>
@@ -2496,7 +2505,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>82</v>
       </c>
@@ -2525,7 +2534,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>82</v>
       </c>
@@ -2551,7 +2560,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>82</v>
       </c>
@@ -2580,7 +2589,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>82</v>
       </c>
@@ -2606,7 +2615,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>82</v>
       </c>
@@ -2632,7 +2641,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>82</v>
       </c>
@@ -2658,7 +2667,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>82</v>
       </c>
@@ -2684,7 +2693,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>82</v>
       </c>
@@ -2710,7 +2719,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>91</v>
       </c>
@@ -2739,7 +2748,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>94</v>
       </c>
@@ -2765,7 +2774,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>95</v>
       </c>
@@ -2794,7 +2803,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>83</v>
       </c>
@@ -2820,7 +2829,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>83</v>
       </c>
@@ -2846,7 +2855,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>83</v>
       </c>
@@ -2872,7 +2881,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>83</v>
       </c>
@@ -2898,7 +2907,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>83</v>
       </c>
@@ -2924,7 +2933,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>83</v>
       </c>
@@ -2950,7 +2959,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>83</v>
       </c>
@@ -2976,7 +2985,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>83</v>
       </c>
@@ -3002,7 +3011,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>83</v>
       </c>
@@ -3028,7 +3037,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>83</v>
       </c>
@@ -3054,7 +3063,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>83</v>
       </c>
@@ -3080,7 +3089,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>83</v>
       </c>
@@ -3106,7 +3115,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>83</v>
       </c>
@@ -3132,7 +3141,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>83</v>
       </c>
@@ -3158,7 +3167,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>83</v>
       </c>
@@ -3184,7 +3193,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>83</v>
       </c>
@@ -3210,7 +3219,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>83</v>
       </c>
@@ -3236,7 +3245,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>83</v>
       </c>
@@ -3262,7 +3271,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>83</v>
       </c>
@@ -3288,7 +3297,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>83</v>
       </c>
@@ -3314,7 +3323,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>83</v>
       </c>
@@ -3340,7 +3349,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>83</v>
       </c>
@@ -3366,7 +3375,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>83</v>
       </c>
@@ -3392,7 +3401,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>83</v>
       </c>
@@ -3418,7 +3427,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>83</v>
       </c>
@@ -3444,7 +3453,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>83</v>
       </c>
@@ -3470,7 +3479,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>83</v>
       </c>
@@ -3496,7 +3505,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>83</v>
       </c>
@@ -3522,7 +3531,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>83</v>
       </c>
@@ -3548,7 +3557,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>83</v>
       </c>
@@ -3574,7 +3583,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>195</v>
       </c>
@@ -3600,7 +3609,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>222</v>
       </c>
@@ -3626,7 +3635,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>222</v>
       </c>
@@ -3652,7 +3661,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>222</v>
       </c>
@@ -3678,7 +3687,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>205</v>
       </c>
@@ -3704,7 +3713,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>205</v>
       </c>
@@ -3730,7 +3739,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>205</v>
       </c>
@@ -3756,7 +3765,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>213</v>
       </c>
@@ -3782,7 +3791,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>213</v>
       </c>
@@ -3808,7 +3817,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>213</v>
       </c>
@@ -3834,7 +3843,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>213</v>
       </c>
@@ -3860,7 +3869,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>213</v>
       </c>
@@ -3886,7 +3895,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>217</v>
       </c>
@@ -3915,7 +3924,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>217</v>
       </c>
@@ -3944,7 +3953,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>225</v>
       </c>
@@ -3967,8 +3976,31 @@
         <v>59</v>
       </c>
     </row>
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>226</v>
+      </c>
+      <c r="C108" t="s">
+        <v>5</v>
+      </c>
+      <c r="D108" t="s">
+        <v>227</v>
+      </c>
+      <c r="E108" t="s">
+        <v>7</v>
+      </c>
+      <c r="F108" t="s">
+        <v>228</v>
+      </c>
+      <c r="H108" t="s">
+        <v>202</v>
+      </c>
+      <c r="I108" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:J43 I44:I107 J44:J106">
+  <conditionalFormatting sqref="I2:J43 J44:J106 I44:I108">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"In Progress"</formula>
     </cfRule>
@@ -3987,13 +4019,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F30A1E73-A707-4178-9C72-9AC27F9EE5F7}">
   <dimension ref="A1:B113"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7265625" customWidth="1"/>
+    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="str">
         <f>'Property-Definition'!A1</f>
         <v>performative</v>
@@ -4002,7 +4034,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="str">
         <f>'Property-Definition'!A2</f>
         <v>DB.SYSTEMS</v>
@@ -4021,7 +4053,7 @@
         <v>public final static String DBSYSTEM = "dbSystem[X]";</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
         <f>'Property-Definition'!A3</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -4040,7 +4072,7 @@
         <v>public final static String DBSYSTEM = "dbSystem[X]";</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
         <f>'Property-Definition'!A4</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -4059,7 +4091,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_DRIVER_CLASS = "dbSystem[X].hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
         <f>'Property-Definition'!A5</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -4078,7 +4110,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_URL = "dbSystem[X].hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
         <f>'Property-Definition'!A6</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -4097,7 +4129,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_URL_MASK = "dbSystem[X].hibernate.connection.url.mask";</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
         <f>'Property-Definition'!A7</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -4116,7 +4148,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_DEFAULT_CATALOG = "dbSystem[X].hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
         <f>'Property-Definition'!A8</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -4135,7 +4167,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_USERNAME = "dbSystem[X].hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
         <f>'Property-Definition'!A9</f>
         <v>DB.SYSTEMS.PARAMETER</v>
@@ -4154,7 +4186,7 @@
         <v>public final static String DBSYSTEM_HIBERNATE_CONNECTION_PASSWORD = "dbSystem[X].hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="str">
         <f>'Property-Definition'!A10</f>
         <v>DB.FACTORIES</v>
@@ -4173,7 +4205,7 @@
         <v>public final static String FACTORY = "factory[X]";</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="str">
         <f>'Property-Definition'!A11</f>
         <v>DB.FACTORIES</v>
@@ -4192,7 +4224,7 @@
         <v>public final static String FACTORY_STATE = "factory[X].state";</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
         <f>'Property-Definition'!A12</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -4211,7 +4243,7 @@
         <v>public final static String ISSTARTDERBYNETWORKSERVER = "isStartDerbyNetworkServer";</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
         <f>'Property-Definition'!A13</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -4230,7 +4262,7 @@
         <v>public final static String HOST-IP = "host-IP";</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="str">
         <f>'Property-Definition'!A14</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -4249,7 +4281,7 @@
         <v>public final static String PORT = "port";</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="str">
         <f>'Property-Definition'!A15</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -4268,7 +4300,7 @@
         <v>public final static String USERNAME = "userName";</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="str">
         <f>'Property-Definition'!A16</f>
         <v>DB.DERBY.NETWORKSERVER</v>
@@ -4287,7 +4319,7 @@
         <v>public final static String PASSWORD = "password";</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="str">
         <f>'Property-Definition'!A17</f>
         <v>DB.CONN.GENERAL</v>
@@ -4306,7 +4338,7 @@
         <v>public final static String USEFOREVERYFACTORY = "useForEveryFactory";</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="str">
         <f>'Property-Definition'!A18</f>
         <v>DB.CONN.GENERAL</v>
@@ -4325,7 +4357,7 @@
         <v>public final static String DBSYSTEM = "dbSystem";</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="str">
         <f>'Property-Definition'!A19</f>
         <v>DB.CONN.GENERAL</v>
@@ -4344,7 +4376,7 @@
         <v>public final static String HIBERNATE_CONNECTION_DRIVER_CLASS = "hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="str">
         <f>'Property-Definition'!A20</f>
         <v>DB.CONN.GENERAL</v>
@@ -4363,7 +4395,7 @@
         <v>public final static String HIBERNATE_CONNECTION_URL = "hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="str">
         <f>'Property-Definition'!A21</f>
         <v>DB.CONN.GENERAL</v>
@@ -4382,7 +4414,7 @@
         <v>public final static String HIBERNATE_DEFAULT_CATALOG = "hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="str">
         <f>'Property-Definition'!A22</f>
         <v>DB.CONN.GENERAL</v>
@@ -4401,7 +4433,7 @@
         <v>public final static String HIBERNATE_CONNECTION_USERNAME = "hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
         <f>'Property-Definition'!A23</f>
         <v>DB.CONN.GENERAL</v>
@@ -4420,7 +4452,7 @@
         <v>public final static String HIBERNATE_CONNECTION_PASSWORD = "hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="str">
         <f>'Property-Definition'!A24</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4439,7 +4471,7 @@
         <v>public final static String FACTORY_FACTORYID = "factory[X].factoryID";</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="str">
         <f>'Property-Definition'!A25</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4458,7 +4490,7 @@
         <v>public final static String FACTORY_DBSYSTEM = "factory[X].dbSystem";</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="str">
         <f>'Property-Definition'!A26</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4477,7 +4509,7 @@
         <v>public final static String FACTORY_HIBERNATE_CONNECTION_DRIVER_CLASS = "factory[X].hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="str">
         <f>'Property-Definition'!A27</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4496,7 +4528,7 @@
         <v>public final static String FACTORY_HIBERNATE_CONNECTION_URL = "factory[X].hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="str">
         <f>'Property-Definition'!A28</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4515,7 +4547,7 @@
         <v>public final static String FACTORY_HIBERNATE_DEFAULT_CATALOG = "factory[X].hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="str">
         <f>'Property-Definition'!A29</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4534,7 +4566,7 @@
         <v>public final static String FACTORY_HIBERNATE_CONNECTION_USERNAME = "factory[X].hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="str">
         <f>'Property-Definition'!A30</f>
         <v>DB.CONN.FACTORY.GET</v>
@@ -4553,7 +4585,7 @@
         <v>public final static String FACTORY_HIBERNATE_CONNECTION_PASSWORD = "factory[X].hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="str">
         <f>'Property-Definition'!A31</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4572,7 +4604,7 @@
         <v>public final static String FACTORYID = "factoryID";</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="str">
         <f>'Property-Definition'!A32</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4591,7 +4623,7 @@
         <v>public final static String DBSYSTEM = "dbSystem";</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="str">
         <f>'Property-Definition'!A33</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4610,7 +4642,7 @@
         <v>public final static String HIBERNATE_CONNECTION_DRIVER_CLASS = "hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="str">
         <f>'Property-Definition'!A34</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4629,7 +4661,7 @@
         <v>public final static String HIBERNATE_CONNECTION_URL = "hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="str">
         <f>'Property-Definition'!A35</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4648,7 +4680,7 @@
         <v>public final static String HIBERNATE_DEFAULT_CATALOG = "hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="str">
         <f>'Property-Definition'!A36</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4667,7 +4699,7 @@
         <v>public final static String HIBERNATE_CONNECTION_USERNAME = "hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="str">
         <f>'Property-Definition'!A37</f>
         <v>DB.CONN.FACTORY.SET</v>
@@ -4686,7 +4718,7 @@
         <v>public final static String HIBERNATE_CONNECTION_PASSWORD = "hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="str">
         <f>'Property-Definition'!A38</f>
         <v>DB.CONN.TEST</v>
@@ -4705,7 +4737,7 @@
         <v>public final static String DBSYSTEM = "dbSystem";</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="str">
         <f>'Property-Definition'!A39</f>
         <v>DB.CONN.TEST</v>
@@ -4724,7 +4756,7 @@
         <v>public final static String HIBERNATE_CONNECTION_DRIVER_CLASS = "hibernate.connection.driver_class";</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="str">
         <f>'Property-Definition'!A40</f>
         <v>DB.CONN.TEST</v>
@@ -4743,7 +4775,7 @@
         <v>public final static String HIBERNATE_CONNECTION_URL = "hibernate.connection.url";</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="str">
         <f>'Property-Definition'!A41</f>
         <v>DB.CONN.TEST</v>
@@ -4762,7 +4794,7 @@
         <v>public final static String HIBERNATE_DEFAULT_CATALOG = "hibernate.default_catalog";</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="str">
         <f>'Property-Definition'!A42</f>
         <v>DB.CONN.TEST</v>
@@ -4781,7 +4813,7 @@
         <v>public final static String HIBERNATE_CONNECTION_USERNAME = "hibernate.connection.username";</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="str">
         <f>'Property-Definition'!A43</f>
         <v>DB.CONN.TEST</v>
@@ -4800,7 +4832,7 @@
         <v>public final static String HIBERNATE_CONNECTION_PASSWORD = "hibernate.connection.password";</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="str">
         <f>'Property-Definition'!A44</f>
         <v>EXEC.MODE</v>
@@ -4819,7 +4851,7 @@
         <v>public final static String EXEC_MODE = "exec.mode";</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="str">
         <f>'Property-Definition'!A45</f>
         <v>EXEC.MODE</v>
@@ -4838,7 +4870,7 @@
         <v>public final static String SERVER_MASTER_URL = "server.master.url";</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="str">
         <f>'Property-Definition'!A46</f>
         <v>EXEC.MODE</v>
@@ -4857,7 +4889,7 @@
         <v>public final static String SERVER_MASTER_PORT = "server.master.port";</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="str">
         <f>'Property-Definition'!A47</f>
         <v>EXEC.MODE</v>
@@ -4876,7 +4908,7 @@
         <v>public final static String SERVER_MASTER_PORT_MTP = "server.master.port.mtp";</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="str">
         <f>'Property-Definition'!A48</f>
         <v>EXEC.MODE</v>
@@ -4895,7 +4927,7 @@
         <v>public final static String SERVER_MASTER_PROTOCOL = "server.master.protocol";</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="str">
         <f>'Property-Definition'!A49</f>
         <v>EXEC.MODE</v>
@@ -4914,7 +4946,7 @@
         <v>public final static String LOCAL_MTP_CREATION = "local.mtp.creation";</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="str">
         <f>'Property-Definition'!A50</f>
         <v>EXEC.MODE</v>
@@ -4933,7 +4965,7 @@
         <v>public final static String LOCAL_MTP_URL = "local.mtp.url";</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="str">
         <f>'Property-Definition'!A51</f>
         <v>EXEC.MODE</v>
@@ -4952,7 +4984,7 @@
         <v>public final static String LOCAL_MTP_PORT = "local.mtp.port";</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="str">
         <f>'Property-Definition'!A52</f>
         <v>EXEC.MODE</v>
@@ -4971,7 +5003,7 @@
         <v>public final static String LOCAL_MTP_PROTOCOL = "local.mtp.protocol";</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="str">
         <f>'Property-Definition'!A53</f>
         <v>EXEC.MODE</v>
@@ -4990,7 +5022,7 @@
         <v>public final static String EMBEDDEDSYSTEM_PROJECT = "embeddedsystem.project";</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="str">
         <f>'Property-Definition'!A54</f>
         <v>EXEC.MODE</v>
@@ -5009,7 +5041,7 @@
         <v>public final static String DEVICE_SYSTEM_EXEC_MODE = "device_system_exec_mode";</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="str">
         <f>'Property-Definition'!A55</f>
         <v>EXEC.MODE</v>
@@ -5028,7 +5060,7 @@
         <v>public final static String EMBEDDEDSYSTEM_AGENT_CLASSNAME = "embeddedsystem.agent[X].classname";</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="str">
         <f>'Property-Definition'!A56</f>
         <v>EXEC.MODE</v>
@@ -5047,7 +5079,7 @@
         <v>public final static String EMBEDDEDSYSTEM_AGENT_AGENTNAME = "embeddedsystem.agent[X].agentname";</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="str">
         <f>'Property-Definition'!A57</f>
         <v>EXEC.MODE</v>
@@ -5066,7 +5098,7 @@
         <v>public final static String SERVICE_SERVICE_SETUP = "service.service_setup";</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="str">
         <f>'Property-Definition'!A58</f>
         <v>EXEC.MODE</v>
@@ -5085,7 +5117,7 @@
         <v>public final static String LOCAL_IP_SELECTION = "local.ip.selection[X]";</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="str">
         <f>'Property-Definition'!A59</f>
         <v>EXEC.MODE</v>
@@ -5104,7 +5136,7 @@
         <v>public final static String FACTORY_ID = "factory_id";</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="e">
         <f>'Property-Definition'!#REF!</f>
         <v>#REF!</v>
@@ -5123,7 +5155,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="str">
         <f>'Property-Definition'!A60</f>
         <v>AWB.AGENTS</v>
@@ -5142,7 +5174,7 @@
         <v>public final static String AGENT_CLASSNAME = "agent[X].classname";</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="str">
         <f>'Property-Definition'!A61</f>
         <v>PROJECTS</v>
@@ -5161,7 +5193,7 @@
         <v>public final static String PROJECT = "project[X]";</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="str">
         <f>'Property-Definition'!A62</f>
         <v>PROJECT.SETUPS[X]</v>
@@ -5180,7 +5212,7 @@
         <v>public final static String PROJECT_SETUP = "project[X].setup[X]";</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="str">
         <f>'Property-Definition'!A63</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5199,7 +5231,7 @@
         <v>public final static String BGPLATFORM_CONTACTAGENT = "bgplatform[X].contactagent";</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="str">
         <f>'Property-Definition'!A60</f>
         <v>AWB.AGENTS</v>
@@ -5218,7 +5250,7 @@
         <v>public final static String BGPLATFORM_PLATFORMNAME = "bgplatform[X].platformname";</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="str">
         <f>'Property-Definition'!A61</f>
         <v>PROJECTS</v>
@@ -5237,7 +5269,7 @@
         <v>public final static String BGPLATFORM_SERVER = "bgplatform[X].server";</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="str">
         <f>'Property-Definition'!A62</f>
         <v>PROJECT.SETUPS[X]</v>
@@ -5256,7 +5288,7 @@
         <v>public final static String BGPLATFORM_IPADDRESS = "bgplatform[X].ipaddress";</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="str">
         <f>'Property-Definition'!A67</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5275,7 +5307,7 @@
         <v>public final static String BGPLATFORM_URL = "bgplatform[X].url";</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="str">
         <f>'Property-Definition'!A68</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5294,7 +5326,7 @@
         <v>public final static String BGPLATFORM_JADEPORT = "bgplatform[X].jadeport";</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="str">
         <f>'Property-Definition'!A69</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5313,7 +5345,7 @@
         <v>public final static String BGPLATFORM_HTTPMTP = "bgplatform[X].httpmtp";</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="str">
         <f>'Property-Definition'!A70</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5332,7 +5364,7 @@
         <v>public final static String BGPLATFORM_VERSIONMAJOR = "bgplatform[X].versionmajor";</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="str">
         <f>'Property-Definition'!A71</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5351,7 +5383,7 @@
         <v>public final static String BGPLATFORM_VERSIONMINOR = "bgplatform[X].versionminor";</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="str">
         <f>'Property-Definition'!A72</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5370,7 +5402,7 @@
         <v>public final static String BGPLATFORM_VERSIONMICRO = "bgplatform[X].versionmicro";</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="str">
         <f>'Property-Definition'!A73</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5389,7 +5421,7 @@
         <v>public final static String BGPLATFORM_VERSIONBUILD = "bgplatform[X].versionbuild";</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="str">
         <f>'Property-Definition'!A74</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5408,7 +5440,7 @@
         <v>public final static String BGPLATFORM_OS_NAME = "bgplatform[X].os.name";</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="str">
         <f>'Property-Definition'!A75</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5427,7 +5459,7 @@
         <v>public final static String BGPLATFORM_OS_VERSION = "bgplatform[X].os.version";</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="str">
         <f>'Property-Definition'!A76</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5446,7 +5478,7 @@
         <v>public final static String BGPLATFORM_OS_ARCHITECTURE = "bgplatform[X].os.architecture";</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="str">
         <f>'Property-Definition'!A77</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5465,7 +5497,7 @@
         <v>public final static String BGPLATFORM_CPU_NAME = "bgplatform[X].cpu.name";</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="str">
         <f>'Property-Definition'!A78</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5484,7 +5516,7 @@
         <v>public final static String BGPLATFORM_CPU_NUMLOGICAL = "bgplatform[X].cpu.numlogical";</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="str">
         <f>'Property-Definition'!A79</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5503,7 +5535,7 @@
         <v>public final static String BGPLATFORM_CPU_NUMPHYSICAL = "bgplatform[X].cpu.numphysical";</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="str">
         <f>'Property-Definition'!A80</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5522,7 +5554,7 @@
         <v>public final static String BGPLATFORM_CPU_SPEEDMHZ = "bgplatform[X].cpu.speedmhz";</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="str">
         <f>'Property-Definition'!A81</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5541,7 +5573,7 @@
         <v>public final static String BGPLATFORM_MEMORYMB = "bgplatform[X].memorymb";</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="str">
         <f>'Property-Definition'!A82</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5560,7 +5592,7 @@
         <v>public final static String BGPLATFORM_BENCHMARKVALUE = "bgplatform[X].benchmarkvalue";</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="str">
         <f>'Property-Definition'!A83</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5579,7 +5611,7 @@
         <v>public final static String BGPLATFORM_TIME_ONLINESINCE = "bgplatform[X].time.onlinesince";</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="str">
         <f>'Property-Definition'!A84</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5598,7 +5630,7 @@
         <v>public final static String BGPLATFORM_TIME_LASTCONTACT = "bgplatform[X].time.lastcontact";</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="str">
         <f>'Property-Definition'!A85</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5617,7 +5649,7 @@
         <v>public final static String BGPLATFORM_LOCALTIME_ONLINESINCE = "bgplatform[X].localtime.onlinesince";</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="str">
         <f>'Property-Definition'!A86</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5636,7 +5668,7 @@
         <v>public final static String BGPLATFORM_LOCALTIME_LASTCONTACT = "bgplatform[X].localtime.lastcontact";</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="str">
         <f>'Property-Definition'!A87</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5655,7 +5687,7 @@
         <v>public final static String BGPLATFORM_CURRENTLYAVAILABLE = "bgplatform[X].currentlyavailable";</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="str">
         <f>'Property-Definition'!A88</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5674,7 +5706,7 @@
         <v>public final static String BGPLATFORM_CURRENT_CPULOAD = "bgplatform[X].current.cpuload";</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="str">
         <f>'Property-Definition'!A89</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5693,7 +5725,7 @@
         <v>public final static String BGPLATFORM_CURRENT_MEMORYLOAD = "bgplatform[X].current.memoryload";</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="str">
         <f>'Property-Definition'!A90</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5712,7 +5744,7 @@
         <v>public final static String BGPLATFORM_CURRENT_MEMORYLOADJVM = "bgplatform[X].current.memoryloadjvm";</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="str">
         <f>'Property-Definition'!A91</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5731,7 +5763,7 @@
         <v>public final static String BGPLATFORM_CURRENT_NUMTHREADS = "bgplatform[X].current.numthreads";</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="str">
         <f>'Property-Definition'!A92</f>
         <v>EXEC.MASTER.SLAVES.GET</v>
@@ -5750,7 +5782,7 @@
         <v>public final static String BGPLATFORM_CURRENT_THRESHOLDEXCEEDED = "bgplatform[X].current.thresholdexceeded";</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="str">
         <f>'Property-Definition'!A93</f>
         <v>UPDATE.STRATEGY</v>
@@ -5769,7 +5801,7 @@
         <v>public final static String ISAUTOUPDATE = "isautoupdate";</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="str">
         <f>'Property-Definition'!A94</f>
         <v>UPDATE.BACKEND.CHECK</v>
@@ -5788,7 +5820,7 @@
         <v>public final static String UPDATECHECK_BACKEND_ISPENDING = "updatecheck.backend.ispending";</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="str">
         <f>'Property-Definition'!A95</f>
         <v>UPDATE.BACKEND.CHECK</v>
@@ -5807,7 +5839,7 @@
         <v>public final static String UPDATECHECK_BACKEND_ISAVAILABLE = "updatecheck.backend.isavailable";</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="str">
         <f>'Property-Definition'!A96</f>
         <v>UPDATE.BACKEND.CHECK</v>
@@ -5826,7 +5858,7 @@
         <v>public final static String UPDATECHECK_BACKEND_LASTCHECK = "updatecheck.backend.lastcheck";</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="e">
         <f>'Property-Definition'!#REF!</f>
         <v>#REF!</v>
@@ -5845,7 +5877,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="str">
         <f>'Property-Definition'!A100</f>
         <v>UPDATE.FRONTEND.CHECK</v>
@@ -5864,7 +5896,7 @@
         <v>public final static String UPDATECHECK_FRONTEND_ISPENDING = "updatecheck.frontend.ispending";</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="str">
         <f>'Property-Definition'!A101</f>
         <v>UPDATE.FRONTEND.CHECK</v>
@@ -5883,7 +5915,7 @@
         <v>public final static String UPDATECHECK_FRONTEND_ISAVAILABLE = "updatecheck.frontend.isavailable";</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="str">
         <f>'Property-Definition'!A102</f>
         <v>UPDATE.FRONTEND.CHECK</v>
@@ -5902,7 +5934,7 @@
         <v>public final static String UPDATECHECK_FRONTEND_LASTCHECK = "updatecheck.frontend.lastcheck";</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="str">
         <f>'Property-Definition'!A104</f>
         <v>UPDATE.FRONTEND.CHECK</v>
@@ -5921,67 +5953,67 @@
         <v>public final static String UPDATECHECK_FRONTEND_NEWVERSION = "updatecheck.frontend.newversion";</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="str">
         <f>'Property-Definition'!A103</f>
         <v>UPDATE.FRONTEND.CHECK</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" t="str">
         <f>'Property-Definition'!A105</f>
         <v>UPDATE.FRONTEND.EXECUTE</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" t="str">
         <f>'Property-Definition'!A106</f>
         <v>UPDATE.FRONTEND.EXECUTE</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" t="str">
         <f>'Property-Definition'!A107</f>
         <v>FILE.CONFIGURATION</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A107">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A107" t="str">
         <f>'Property-Definition'!A108</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
+        <v>WEBSOCKET.TICKET</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108">
         <f>'Property-Definition'!A109</f>
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109">
         <f>'Property-Definition'!A110</f>
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110">
         <f>'Property-Definition'!A111</f>
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111">
         <f>'Property-Definition'!A112</f>
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112">
         <f>'Property-Definition'!A113</f>
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113">
         <f>'Property-Definition'!A114</f>
         <v>0</v>
@@ -5994,6 +6026,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101004FB79D76D905EB41B4AD64ED4839597F" ma:contentTypeVersion="11" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="0622d98e252eab518d4b54f931ba6851">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="897f6830-f425-409d-b8f5-ce1019056d9e" xmlns:ns3="f2404b4d-361b-46d3-b2ec-035eed29e274" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dd5f302b3846fd12003b89c8f5b7df36" ns2:_="" ns3:_="">
     <xsd:import namespace="897f6830-f425-409d-b8f5-ce1019056d9e"/>
@@ -6188,15 +6229,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -6209,6 +6241,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A33EE264-283E-4F19-BA61-B3264EA417E2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6227,14 +6267,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17599C1F-5A6A-4B10-87A3-7E73F8495CE9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF16440F-B0E0-4269-97EE-BEB05B0223C8}">
   <ds:schemaRefs>

</xml_diff>